<commit_message>
feat: v1.26 — game/lottery.js를 server.js에 통합 (첫 모듈 통합)
신규 모듈을 실제 동작하도록 wire-up:
- require('./game/lottery') 추가
- 소켓 핸들러 3종 추가:
  * lottery_status — 룰렛 상태/가격/상품 풀 조회
  * lottery_free_spin — 매일 무료 1회 스핀
  * lottery_paid_spin — 유료 1회 / 10연속 스핀
- applyLotteryReward() 헬퍼: 골드/다이아/재료/상자 자동 지급
- 전설/영웅 보상 획득 시 전 서버 알림 송출
- ach_lucky 업적 자동 추적 (lucky_spin)
- savePlayer + player_update로 영속화

v1.20부터 추가한 6개 신규 모듈 중 첫 통합 사례.
나머지 모듈(season/event/boss_rush/fishing/auction)도 동일한 패턴으로
점진적 통합 가능.

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutoBattle_io_기획서.xlsx
+++ b/AutoBattle_io_기획서.xlsx
@@ -40,7 +40,7 @@
     <sheet name="월드 보스" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="연금술" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="패치 노트" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="v1.9 ~ v1.25" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="v1.9 ~ v1.26" sheetId="34" state="visible" r:id="rId34"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -13685,7 +13685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D56"/>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13726,7 +13726,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -13736,19 +13736,19 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>입찰식 경매 시스템 (game/auction.js 신규 모듈)</t>
+          <t>game/lottery.js → server.js 통합 (require + 소켓 핸들러 3종)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -13758,19 +13758,19 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>룰렛</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>3가지 기간(1h/6h/24h) + 등록2% + 낙찰5% + 스나이핑 방지</t>
+          <t>lottery_status / lottery_free_spin / lottery_paid_spin 이벤트 추가</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
@@ -13780,19 +13780,19 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>룰렛</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>경매장 시트 신규 추가</t>
+          <t>전설/영웅 보상 획득 시 전 서버 알림 + ach_lucky 업적 추적</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -13802,19 +13802,19 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>11종 어종 + 5등급 낚싯대 + 4종 미끼 (game/fishing.js 신규 모듈)</t>
+          <t>입찰식 경매 시스템 (game/auction.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -13824,19 +13824,19 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>신화 크라켄 (밤+낚시터+드래곤대 한정), 바다의 군주 칭호 연계</t>
+          <t>3가지 기간(1h/6h/24h) + 등록2% + 낙찰5% + 스나이핑 방지</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -13851,14 +13851,14 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>낚시 시트 신규 추가</t>
+          <t>경매장 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -13868,19 +13868,19 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>20웨이브 엔드리스 보스 러시 모드 (game/boss_rush.js 신규 모듈)</t>
+          <t>11종 어종 + 5등급 낚싯대 + 4종 미끼 (game/fishing.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -13890,19 +13890,19 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>매일 무료 3회 + 랭킹 1위 챔피언 칭호</t>
+          <t>신화 크라켄 (밤+낚시터+드래곤대 한정), 바다의 군주 칭호 연계</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -13917,14 +13917,14 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>보스 러시 시트 신규 추가</t>
+          <t>낚시 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -13934,19 +13934,19 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>행운의 룰렛</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>10종 보상 + 가중치 시스템 (game/lottery.js 신규 모듈)</t>
+          <t>20웨이브 엔드리스 보스 러시 모드 (game/boss_rush.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -13956,19 +13956,19 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>룰렛</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>매일 무료 1회 / 유료 50💎 / 10연속 450💎 (10% 할인)</t>
+          <t>매일 무료 3회 + 랭킹 1위 챔피언 칭호</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -13983,14 +13983,14 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>행운의 룰렛 시트 신규 추가</t>
+          <t>보스 러시 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
@@ -14000,19 +14000,19 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>행운의 룰렛</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>5종 시즌 축제 추가 (신년/봄꽃/한여름/할로윈/겨울)</t>
+          <t>10종 보상 + 가중치 시스템 (game/lottery.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
@@ -14022,19 +14022,19 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>모듈화</t>
+          <t>룰렛</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>game/event.js 신규 파일 (실제 달력 기반 자동 활성화)</t>
+          <t>매일 무료 1회 / 유료 50💎 / 10연속 450💎 (10% 할인)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -14049,14 +14049,14 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>축제 이벤트 시트 신규 추가</t>
+          <t>행운의 룰렛 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
@@ -14066,19 +14066,19 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>15티어 배틀 패스 시스템 추가 (game/season.js 신규 모듈)</t>
+          <t>5종 시즌 축제 추가 (신년/봄꽃/한여름/할로윈/겨울)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -14088,19 +14088,19 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>모듈화</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>30일 사이클, 무료+프리미엄(1500💎) 트랙</t>
+          <t>game/event.js 신규 파일 (실제 달력 기반 자동 활성화)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
@@ -14115,14 +14115,14 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스 시트 신규 추가</t>
+          <t>축제 이벤트 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -14132,19 +14132,19 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>마일스톤 5종 추가 (Lv.40/50, 첫 환생, 첫 월드 보스, 업적 50)</t>
+          <t>15티어 배틀 패스 시스템 추가 (game/season.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
@@ -14154,19 +14154,19 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아 시트 신규 추가</t>
+          <t>30일 사이클, 무료+프리미엄(1500💎) 트랙</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -14176,19 +14176,19 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>상점</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>프리미엄 5종 추가 (불사조/폭풍 스킨, 자동물약 24h, 보물상자, 재료 패키지)</t>
+          <t>시즌 패스 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
@@ -14198,19 +14198,19 @@
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>상점 시트 갱신</t>
+          <t>마일스톤 5종 추가 (Lv.40/50, 첫 환생, 첫 월드 보스, 업적 50)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -14220,19 +14220,19 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>혈맹</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>혈맹 Lv.6-10 + 신규 스킬 5종 (분노/신속/회복/운명/전설)</t>
+          <t>무료 다이아 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
@@ -14242,19 +14242,19 @@
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>혈맹</t>
+          <t>상점</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>최대 인원 50→100명 (Lv.10 기준)</t>
+          <t>프리미엄 5종 추가 (불사조/폭풍 스킨, 자동물약 24h, 보물상자, 재료 패키지)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -14269,14 +14269,14 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>길드(혈맹) 시트 신규 추가</t>
+          <t>상점 시트 갱신</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
@@ -14286,19 +14286,19 @@
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>혈맹</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>점쟁이/감정사/수집가 3종 추가 (운세/감정/희귀품 매입)</t>
+          <t>혈맹 Lv.6-10 + 신규 스킬 5종 (분노/신속/회복/운명/전설)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -14308,19 +14308,19 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>대사 시스템</t>
+          <t>혈맹</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>신규 NPC 상황별 대사 (밤/카르마/레벨/골드 연동)</t>
+          <t>최대 인원 50→100명 (Lv.10 기준)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
@@ -14335,14 +14335,14 @@
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>NPC 시트 신규 추가 (11종)</t>
+          <t>길드(혈맹) 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -14352,19 +14352,19 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>각성기</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>클래스별 Lv.40 각성기 5종 추가 (천개의칼날/대지가르기/불멸의수호자/시간정지/신의은총)</t>
+          <t>점쟁이/감정사/수집가 3종 추가 (운세/감정/희귀품 매입)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
@@ -14374,19 +14374,19 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>대사 시스템</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>스킬 시트 전면 갱신 (12종→30종, 클레릭 포함)</t>
+          <t>신규 NPC 상황별 대사 (밤/카르마/레벨/골드 연동)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -14396,19 +14396,19 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>v1.9~v1.13 컨텐츠 연계 업적 5종 추가 (폭풍 정복자/연금술사/그림자/전설 동반자/이국 상인)</t>
+          <t>NPC 시트 신규 추가 (11종)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
@@ -14418,19 +14418,19 @@
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>각성기</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>퀘스트 시트 전면 갱신 (9종→64종 반영)</t>
+          <t>클래스별 Lv.40 각성기 5종 추가 (천개의칼날/대지가르기/불멸의수호자/시간정지/신의은총)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -14440,19 +14440,19 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>월드 보스</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>폭풍의 거인 / 시간의 수호자 2종 추가 (최대 HP / 최강 ATK)</t>
+          <t>스킬 시트 전면 갱신 (12종→30종, 클레릭 포함)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
@@ -14462,19 +14462,19 @@
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>교역</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>이국의 사치품 3종 추가 (불사조 깃털/공허의 정수/천공의 비단)</t>
+          <t>v1.9~v1.13 컨텐츠 연계 업적 5종 추가 (폭풍 정복자/연금술사/그림자/전설 동반자/이국 상인)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -14489,14 +14489,14 @@
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>월드 보스 시트 신규 추가, 교역 시트 갱신</t>
+          <t>퀘스트 시트 전면 갱신 (9종→64종 반영)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
@@ -14506,19 +14506,19 @@
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>월드 보스</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>엘릭서 5종 추가 (타이탄/강철/질풍/지혜/행운, 15~30분 강력 버프)</t>
+          <t>폭풍의 거인 / 시간의 수호자 2종 추가 (최대 HP / 최강 ATK)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -14528,19 +14528,19 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>교역</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>연금술 시트 신규 추가</t>
+          <t>이국의 사치품 3종 추가 (불사조 깃털/공허의 정수/천공의 비단)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
@@ -14550,19 +14550,19 @@
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>신규 펫</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>불사조 (화염 +20%) / 유니콘 (회피 +10%) + 진화형</t>
+          <t>월드 보스 시트 신규 추가, 교역 시트 갱신</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -14572,19 +14572,19 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>신규 탈것</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>페가수스 (이동 +85%, 비행)</t>
+          <t>엘릭서 5종 추가 (타이탄/강철/질풍/지혜/행운, 15~30분 강력 버프)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
@@ -14594,19 +14594,19 @@
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>신규 던전</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>그림자 미궁 (Lv.38, 8인 파티, 7스테이지, 전설 드롭)</t>
+          <t>연금술 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -14616,19 +14616,19 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>신규 펫</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>던전 시트 신규 추가 (7종 던전 정리)</t>
+          <t>불사조 (화염 +20%) / 유니콘 (회피 +10%) + 진화형</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
@@ -14638,19 +14638,19 @@
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 탈것</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>공허의 방랑자/불멸자/천공의 군주 3종 추가 (엔드게임)</t>
+          <t>페가수스 (이동 +85%, 비행)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -14660,78 +14660,78 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>신규 던전</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>51개 지역, 16종 칭호, 출석/세트/등급 시트 추가</t>
+          <t>그림자 미궁 (Lv.38, 8인 파티, 7스테이지, 전설 드롭)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>패치 노트 갱신, 낮/밤 시계 + 진행 시간 표시</t>
+          <t>던전 시트 신규 추가 (7종 던전 정리)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>자동화</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>자동 스킬 시전 (인간 플레이어용), 자동 스킬 토글 버튼</t>
+          <t>공허의 방랑자/불멸자/천공의 군주 3종 추가 (엔드게임)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>미니맵 친구 위치 표시, 보스 표시 강화, DPS 미터 스파크라인</t>
+          <t>51개 지역, 16종 칭호, 출석/세트/등급 시트 추가</t>
         </is>
       </c>
     </row>
@@ -14748,19 +14748,19 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>시스템</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>혈맹 창고 UI 패널, 보스 신규 디버프 적용</t>
+          <t>패치 노트 갱신, 낮/밤 시계 + 진행 시간 표시</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
@@ -14770,19 +14770,19 @@
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>상태이상</t>
+          <t>자동화</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>신규 디버프 5종 (빙결/감전/출혈/약화/공포)</t>
+          <t>자동 스킬 시전 (인간 플레이어용), 자동 스킬 토글 버튼</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -14797,14 +14797,14 @@
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>포션 단축키 (1/2/3/4), 레벨별 추천 활동 가이드</t>
+          <t>미니맵 친구 위치 표시, 보스 표시 강화, DPS 미터 스파크라인</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
@@ -14819,7 +14819,7 @@
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>장비 자동 최적화 (auto_equip_best), 알림 센터</t>
+          <t>혈맹 창고 UI 패널, 보스 신규 디버프 적용</t>
         </is>
       </c>
     </row>
@@ -14836,12 +14836,12 @@
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>컨텐츠</t>
+          <t>상태이상</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>신규 업적 10종 (30→40), 신규 몬스터 존 3개</t>
+          <t>신규 디버프 5종 (빙결/감전/출혈/약화/공포)</t>
         </is>
       </c>
     </row>
@@ -14863,27 +14863,93 @@
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>인벤토리 검색 + 정렬, PvP 시즌 보드 시각화</t>
+          <t>포션 단축키 (1/2/3/4), 레벨별 추천 활동 가이드</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>시스템</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>장비 자동 최적화 (auto_equip_best), 알림 센터</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
+        <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>컨텐츠</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>신규 업적 10종 (30→40), 신규 몬스터 존 3개</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>인벤토리 검색 + 정렬, PvP 시즌 보드 시각화</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
+        <is>
           <t>v1.6 이전</t>
         </is>
       </c>
-      <c r="B56" s="7" t="inlineStr">
+      <c r="B59" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C56" s="7" t="inlineStr">
+      <c r="C59" s="8" t="inlineStr">
         <is>
           <t>기반</t>
         </is>
       </c>
-      <c r="D56" s="7" t="inlineStr">
+      <c r="D59" s="8" t="inlineStr">
         <is>
           <t>마을/사냥/PvP/카르마/펫/탈것/제작/교역/길드/공성/투기장 등</t>
         </is>
@@ -14903,7 +14969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E73"/>
+  <dimension ref="A1:E77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -14950,378 +15016,378 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>game/auction.js 신규</t>
+          <t>lottery → server.js</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>입찰식 / 3기간 / 5% 인상 / 스나이핑 방지</t>
+          <t>require + 소켓 핸들러 3종</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>등록 2% + 낙찰 5%</t>
+          <t>첫 모듈 통합 마일스톤</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>소켓 이벤트</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>활성 한도</t>
+          <t>lottery_status</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>플레이어당 10개</t>
+          <t>상태/가격/상품 풀 조회</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>자기 입찰 금지</t>
+          <t>클라이언트 표시용</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>소켓 이벤트</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>game/fishing.js 신규</t>
+          <t>lottery_free_spin</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>11종 어종 / 5등급 낚싯대 / 4종 미끼</t>
+          <t>매일 무료 1회 스핀</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>신화 크라켄 = 20000G + 칭호</t>
+          <t>자정 초기화</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>소켓 이벤트</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>전설의 비단잉어</t>
+          <t>lottery_paid_spin</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>드래곤 낚싯대 + 가중치 1</t>
+          <t>유료 1회 / 10연속</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>5000G + 평생 행운 +5%</t>
+          <t>count: 1 또는 10</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>game/boss_rush.js 신규</t>
+          <t>game/auction.js 신규</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>20웨이브 / HP ×1.35 스케일링</t>
+          <t>입찰식 / 3기간 / 5% 인상 / 스나이핑 방지</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>최종 보상: 200💎 + 용재료 ×5</t>
+          <t>등록 2% + 낙찰 5%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>입장</t>
+          <t>활성 한도</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>매일 무료 3회 / 1000G / 30💎</t>
+          <t>플레이어당 10개</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>랭킹 시스템</t>
+          <t>자기 입찰 금지</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>챔피언 보상</t>
+          <t>game/fishing.js 신규</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>1위: 500💎 + 칭호 / 2위: 300💎 / 3위: 200💎</t>
+          <t>11종 어종 / 5등급 낚싯대 / 4종 미끼</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>신화 크라켄 = 20000G + 칭호</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>행운의 룰렛</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>game/lottery.js 신규</t>
+          <t>전설의 비단잉어</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>10종 보상 / 가중치 1000</t>
+          <t>드래곤 낚싯대 + 가중치 1</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>매일 무료 1회 + 유료</t>
+          <t>5000G + 평생 행운 +5%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>룰렛 (전설)</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>영웅 장비 상자</t>
+          <t>game/boss_rush.js 신규</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>확률 0.2% (가장 희귀)</t>
+          <t>20웨이브 / HP ×1.35 스케일링</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>전설 보상</t>
+          <t>최종 보상: 200💎 + 용재료 ×5</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>룰렛 (전설)</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>200 다이아</t>
+          <t>입장</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>확률 0.8%</t>
+          <t>매일 무료 3회 / 1000G / 30💎</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>잭팟</t>
+          <t>랭킹 시스템</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>신년 축제</t>
+          <t>챔피언 보상</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>1/1 ~ 1/7</t>
+          <t>1위: 500💎 + 칭호 / 2위: 300💎 / 3위: 200💎</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>골드 +50% / EXP +30%</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>행운의 룰렛</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>봄꽃 축제</t>
+          <t>game/lottery.js 신규</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>4/1 ~ 4/14</t>
+          <t>10종 보상 / 가중치 1000</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>HP재생 +30% / 드롭 +20%</t>
+          <t>매일 무료 1회 + 유료</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>룰렛 (전설)</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>한여름 밤의 축제</t>
+          <t>영웅 장비 상자</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>7/15 ~ 8/15</t>
+          <t>확률 0.2% (가장 희귀)</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>화염 +30% / PvP 보상 +50%</t>
+          <t>전설 보상</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>룰렛 (전설)</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>할로윈 축제</t>
+          <t>200 다이아</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>10/25 ~ 11/1</t>
+          <t>확률 0.8%</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>크리 +10% / 언데드 +50%</t>
+          <t>잭팟</t>
         </is>
       </c>
     </row>
@@ -15338,206 +15404,206 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>겨울 축제</t>
+          <t>신년 축제</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>12/20 ~ 12/31</t>
+          <t>1/1 ~ 1/7</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>골드 +30% / EXP +30% / 드롭 +30%</t>
+          <t>골드 +50% / EXP +30%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>game/season.js 신규</t>
+          <t>봄꽃 축제</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>15티어 / 30일 / 무료+프리미엄</t>
+          <t>4/1 ~ 4/14</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>만렙 보상: 태초 반지 + 시즌 칭호</t>
+          <t>HP재생 +30% / 드롭 +20%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>XP 획득 7종</t>
+          <t>한여름 밤의 축제</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>퀘/보스/PvP/월드보스/던전/제작</t>
+          <t>7/15 ~ 8/15</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>일일 +200 ~ 월드보스 +500</t>
+          <t>화염 +30% / PvP 보상 +50%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>프리미엄 가격</t>
+          <t>할로윈 축제</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>1500 다이아</t>
+          <t>10/25 ~ 11/1</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>시즌 당 1회</t>
+          <t>크리 +10% / 언데드 +50%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Lv.40 달성</t>
+          <t>겨울 축제</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>각성기 해금 마일스톤</t>
+          <t>12/20 ~ 12/31</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>150💎</t>
+          <t>골드 +30% / EXP +30% / 드롭 +30%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Lv.50 달성</t>
+          <t>game/season.js 신규</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>환생 가능 마일스톤</t>
+          <t>15티어 / 30일 / 무료+프리미엄</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>250💎</t>
+          <t>만렙 보상: 태초 반지 + 시즌 칭호</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>첫 환생</t>
+          <t>XP 획득 7종</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>prestige 1차</t>
+          <t>퀘/보스/PvP/월드보스/던전/제작</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>500💎</t>
+          <t>일일 +200 ~ 월드보스 +500</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>첫 월드 보스</t>
+          <t>프리미엄 가격</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>월드 보스 처치 보너스</t>
+          <t>1500 다이아</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>100💎</t>
+          <t>시즌 당 1회</t>
         </is>
       </c>
     </row>
@@ -15554,125 +15620,125 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>업적 50개</t>
+          <t>Lv.40 달성</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>업적 마일스톤</t>
+          <t>각성기 해금 마일스톤</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>200💎</t>
+          <t>150💎</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>상점 (스킨)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>불사조 스킨</t>
+          <t>Lv.50 달성</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>1200 다이아</t>
+          <t>환생 가능 마일스톤</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>불사조 깃털 이펙트 (영구)</t>
+          <t>250💎</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>상점 (스킨)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>폭풍 스킨</t>
+          <t>첫 환생</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>1200 다이아</t>
+          <t>prestige 1차</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>번개 오라 이펙트 (영구)</t>
+          <t>500💎</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>상점 (편의)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>프리미엄 자동물약</t>
+          <t>첫 월드 보스</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>500 다이아</t>
+          <t>월드 보스 처치 보너스</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>24시간 자동물약 무한</t>
+          <t>100💎</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>상점 (상자)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>프리미엄 보물 상자</t>
+          <t>업적 50개</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>300 다이아</t>
+          <t>업적 마일스톤</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>전설 장비 확정 + 다이아</t>
+          <t>200💎</t>
         </is>
       </c>
     </row>
@@ -15684,130 +15750,130 @@
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>상점 (재료)</t>
+          <t>상점 (스킨)</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>전설 재료 패키지</t>
+          <t>불사조 스킨</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>600 다이아</t>
+          <t>1200 다이아</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>용재료×10 + 영혼석×20 + 마법재료×20</t>
+          <t>불사조 깃털 이펙트 (영구)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>혈맹 Lv.6</t>
+          <t>상점 (스킨)</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>혈맹의 분노</t>
+          <t>폭풍 스킨</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>크리티컬 +5%</t>
+          <t>1200 다이아</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>60명 정원</t>
+          <t>번개 오라 이펙트 (영구)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>혈맹 Lv.7</t>
+          <t>상점 (편의)</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>혈맹의 신속</t>
+          <t>프리미엄 자동물약</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>이동속도 +10%</t>
+          <t>500 다이아</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>70명 정원</t>
+          <t>24시간 자동물약 무한</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>혈맹 Lv.8</t>
+          <t>상점 (상자)</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>혈맹의 회복</t>
+          <t>프리미엄 보물 상자</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>HP 재생 +50%</t>
+          <t>300 다이아</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>80명 정원</t>
+          <t>전설 장비 확정 + 다이아</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>혈맹 Lv.9</t>
+          <t>상점 (재료)</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>혈맹의 운명</t>
+          <t>전설 재료 패키지</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>회피 +5%</t>
+          <t>600 다이아</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>90명 정원</t>
+          <t>용재료×10 + 영혼석×20 + 마법재료×20</t>
         </is>
       </c>
     </row>
@@ -15819,211 +15885,211 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>혈맹 Lv.10</t>
+          <t>혈맹 Lv.6</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>혈맹의 전설</t>
+          <t>혈맹의 분노</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>전 스탯 +5%</t>
+          <t>크리티컬 +5%</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>100명 정원 — 최종</t>
+          <t>60명 정원</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>혈맹 Lv.7</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>점쟁이</t>
+          <t>혈맹의 신속</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>운세 / 행운 버프 (밤·카르마 반응)</t>
+          <t>이동속도 +10%</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>상황 대사 4종</t>
+          <t>70명 정원</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>혈맹 Lv.8</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>감정사</t>
+          <t>혈맹의 회복</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>미감정 장비 감정 (Lv.30+ 특수)</t>
+          <t>HP 재생 +50%</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>상황 대사 4종</t>
+          <t>80명 정원</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>혈맹 Lv.9</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>수집가</t>
+          <t>혈맹의 운명</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>희귀 아이템 매입 (골드 50000+ 특별)</t>
+          <t>회피 +5%</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>상황 대사 4종</t>
+          <t>90명 정원</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>각성기 (어쌔신)</t>
+          <t>혈맹 Lv.10</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>천 개의 칼날</t>
+          <t>혈맹의 전설</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>3.5배 × 7타 / 광역 / 쿨150초</t>
+          <t>전 스탯 +5%</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>100명 정원 — 최종</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>각성기 (워리어)</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>대지 가르기</t>
+          <t>점쟁이</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>6.0배 / 광역 5범위 / 스턴 2초</t>
+          <t>운세 / 행운 버프 (밤·카르마 반응)</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>상황 대사 4종</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>각성기 (나이트)</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>불멸의 수호자</t>
+          <t>감정사</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>피해 90% 감소 / 도발 / 10초</t>
+          <t>미감정 장비 감정 (Lv.30+ 특수)</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>상황 대사 4종</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>각성기 (메이지)</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>시간 정지</t>
+          <t>수집가</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>12.0배 / 광역 6범위 / 슬로우 90%</t>
+          <t>희귀 아이템 매입 (골드 50000+ 특별)</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>상황 대사 4종</t>
         </is>
       </c>
     </row>
@@ -16035,17 +16101,17 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>각성기 (클레릭)</t>
+          <t>각성기 (어쌔신)</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>신의 은총</t>
+          <t>천 개의 칼날</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>HP 100% 회복 / 전스탯 +50%</t>
+          <t>3.5배 × 7타 / 광역 / 쿨150초</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
@@ -16057,108 +16123,108 @@
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (워리어)</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>폭풍 정복자</t>
+          <t>대지 가르기</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>폭풍의 거인 처치</t>
+          <t>6.0배 / 광역 5범위 / 스턴 2초</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>10,000G + 150다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (나이트)</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>연금술사</t>
+          <t>불멸의 수호자</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>엘릭서 10회 제작</t>
+          <t>피해 90% 감소 / 도발 / 10초</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>5,000G + 80다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (메이지)</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>그림자 정복자</t>
+          <t>시간 정지</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>그림자 미궁 클리어</t>
+          <t>12.0배 / 광역 6범위 / 슬로우 90%</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>8,000G + 120다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (클레릭)</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>전설의 동반자</t>
+          <t>신의 은총</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>전설급 펫 진화</t>
+          <t>HP 100% 회복 / 전스탯 +50%</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>6,000G + 100다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
@@ -16175,206 +16241,206 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>이국의 상인</t>
+          <t>폭풍 정복자</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>사치품 교역 5회</t>
+          <t>폭풍의 거인 처치</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>4,000G + 60다이아</t>
+          <t>10,000G + 150다이아</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>월드 보스</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>폭풍의 거인</t>
+          <t>연금술사</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>HP 100,000 / ATK 140 / DEF 90</t>
+          <t>엘릭서 10회 제작</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>EXP 10000 + 6000G</t>
+          <t>5,000G + 80다이아</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>월드 보스</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>시간의 수호자</t>
+          <t>그림자 정복자</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>HP 70,000 / ATK 170 / DEF 60</t>
+          <t>그림자 미궁 클리어</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t>EXP 9000 + 7000G</t>
+          <t>8,000G + 120다이아</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>교역품</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>불사조 깃털 / 공허의 정수 / 천공의 비단</t>
+          <t>전설의 동반자</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>이국의 사치품 3종</t>
+          <t>전설급 펫 진화</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>기본가 600~900G</t>
+          <t>6,000G + 100다이아</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>타이탄의 엘릭서</t>
+          <t>이국의 상인</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>용재료×3 + 마법재료×10</t>
+          <t>사치품 교역 5회</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
         <is>
-          <t>ATK ×1.5 / 30분</t>
+          <t>4,000G + 60다이아</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>월드 보스</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>강철 엘릭서</t>
+          <t>폭풍의 거인</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>철광석×30 + 마법재료×10</t>
+          <t>HP 100,000 / ATK 140 / DEF 90</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>DEF ×1.5 / 30분</t>
+          <t>EXP 10000 + 6000G</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>월드 보스</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>질풍 엘릭서</t>
+          <t>시간의 수호자</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>약초×20 + 마법재료×8</t>
+          <t>HP 70,000 / ATK 170 / DEF 60</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t>SPD ×1.4 / 20분</t>
+          <t>EXP 9000 + 7000G</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>교역품</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>지혜 엘릭서</t>
+          <t>불사조 깃털 / 공허의 정수 / 천공의 비단</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>마법수정×5 + 영혼재료×5</t>
+          <t>이국의 사치품 3종</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>EXP ×2.5 / 15분</t>
+          <t>기본가 600~900G</t>
         </is>
       </c>
     </row>
@@ -16391,260 +16457,260 @@
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>행운 엘릭서</t>
+          <t>타이탄의 엘릭서</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>보석×10 + 마법재료×5</t>
+          <t>용재료×3 + 마법재료×10</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t>GOLD ×2.0 / 15분</t>
+          <t>ATK ×1.5 / 30분</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>신규 펫</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>불사조 (pet_phoenix)</t>
+          <t>강철 엘릭서</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>불꽃산 보스 50처치</t>
+          <t>철광석×30 + 마법재료×10</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>화염 DMG +20% (진화 +40%)</t>
+          <t>DEF ×1.5 / 30분</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>신규 펫</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>유니콘 (pet_unicorn)</t>
+          <t>질풍 엘릭서</t>
         </is>
       </c>
       <c r="D59" s="8" t="inlineStr">
         <is>
-          <t>다이아 800개</t>
+          <t>약초×20 + 마법재료×8</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t>회피 +10% (진화 +20%)</t>
+          <t>SPD ×1.4 / 20분</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>신규 탈것</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>페가수스 (mount_pegasus)</t>
+          <t>지혜 엘릭서</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>다이아 1200개</t>
+          <t>마법수정×5 + 영혼재료×5</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>이동속도 +85% / 비행</t>
+          <t>EXP ×2.5 / 15분</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>신규 던전</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>그림자 미궁</t>
+          <t>행운 엘릭서</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>Lv.38 / 8인 파티 / 7스테이지</t>
+          <t>보석×10 + 마법재료×5</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t>22000G + 32000EXP</t>
+          <t>GOLD ×2.0 / 15분</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>드롭</t>
+          <t>신규 펫</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>드래곤 검/망토/투구/장갑</t>
+          <t>불사조 (pet_phoenix)</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>그림자 미궁 보스 드롭</t>
+          <t>불꽃산 보스 50처치</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>전설급</t>
+          <t>화염 DMG +20% (진화 +40%)</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 펫</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>공허의 방랑자</t>
+          <t>유니콘 (pet_unicorn)</t>
         </is>
       </c>
       <c r="D63" s="8" t="inlineStr">
         <is>
-          <t>몬스터 10,000 처치</t>
+          <t>다이아 800개</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t>ATK +7%</t>
+          <t>회피 +10% (진화 +20%)</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 탈것</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>불멸자</t>
+          <t>페가수스 (mount_pegasus)</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>환생 5회</t>
+          <t>다이아 1200개</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>EXP +25%</t>
+          <t>이동속도 +85% / 비행</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 던전</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>천공의 군주</t>
+          <t>그림자 미궁</t>
         </is>
       </c>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>월드 보스 10회 처치</t>
+          <t>Lv.38 / 8인 파티 / 7스테이지</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>보스DMG +15%</t>
+          <t>22000G + 32000EXP</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>드롭</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>지역 시트 갱신</t>
+          <t>드래곤 검/망토/투구/장갑</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>25→51개 지역 반영</t>
+          <t>그림자 미궁 보스 드롭</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>전설급</t>
         </is>
       </c>
     </row>
@@ -16656,22 +16722,22 @@
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>칭호 시트 갱신</t>
+          <t>공허의 방랑자</t>
         </is>
       </c>
       <c r="D67" s="8" t="inlineStr">
         <is>
-          <t>7→16종 + 효과/색상 추가</t>
+          <t>몬스터 10,000 처치</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ATK +7%</t>
         </is>
       </c>
     </row>
@@ -16683,22 +16749,22 @@
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>출석 캘린더 시트</t>
+          <t>불멸자</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>신규 추가 (28일 사이클)</t>
+          <t>환생 5회</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EXP +25%</t>
         </is>
       </c>
     </row>
@@ -16710,22 +16776,22 @@
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>장비 세트 시트</t>
+          <t>천공의 군주</t>
         </is>
       </c>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>신규 추가 (드래곤/영웅/태초)</t>
+          <t>월드 보스 10회 처치</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>보스DMG +15%</t>
         </is>
       </c>
     </row>
@@ -16742,12 +16808,12 @@
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>장비 등급 시트</t>
+          <t>지역 시트 갱신</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>신규 추가 (5등급 + 랜덤 옵션 7종)</t>
+          <t>25→51개 지역 반영</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
@@ -16769,12 +16835,12 @@
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>디버프 시트</t>
+          <t>칭호 시트 갱신</t>
         </is>
       </c>
       <c r="D71" s="8" t="inlineStr">
         <is>
-          <t>신규 추가 (10종, v1.7 5종 포함)</t>
+          <t>7→16종 + 효과/색상 추가</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
@@ -16796,12 +16862,12 @@
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>패치 노트 시트</t>
+          <t>출석 캘린더 시트</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>신규 추가 (히스토리)</t>
+          <t>신규 추가 (28일 사이클)</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
@@ -16813,25 +16879,133 @@
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B73" s="8" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>장비 세트 시트</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>신규 추가 (드래곤/영웅/태초)</t>
+        </is>
+      </c>
+      <c r="E73" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>장비 등급 시트</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>신규 추가 (5등급 + 랜덤 옵션 7종)</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B75" s="8" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>디버프 시트</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>신규 추가 (10종, v1.7 5종 포함)</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="7" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>패치 노트 시트</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>신규 추가 (히스토리)</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="8" t="inlineStr">
+        <is>
           <t>v1.10</t>
         </is>
       </c>
-      <c r="B73" s="8" t="inlineStr">
+      <c r="B77" s="8" t="inlineStr">
         <is>
           <t>기획서</t>
         </is>
       </c>
-      <c r="C73" s="8" t="inlineStr">
+      <c r="C77" s="8" t="inlineStr">
         <is>
           <t>던전 시트</t>
         </is>
       </c>
-      <c r="D73" s="8" t="inlineStr">
+      <c r="D77" s="8" t="inlineStr">
         <is>
           <t>신규 추가 (7종 던전)</t>
         </is>
       </c>
-      <c r="E73" s="8" t="inlineStr">
+      <c r="E77" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
feat: v1.27 — game/fishing.js를 server.js에 통합 (두 번째 모듈 통합)
- require('./game/fishing') 추가
- 소켓 핸들러 3종:
  * fishing_status — 지역/낚싯대/미끼/시간대 조회
  * fishing_cast — 낚시 시도 (지역+낚싯대+미끼+시간대 검증)
  * fishing_buy_rod — 낚싯대 구매 (골드/다이아)
- 낚시 가능 지역: 낚시 만 / 강변 평야 / 산호초 해안
- 낚싯대 미보유 시 거부, 미끼는 사용 시 자동 차감
- 시간대(밤) 컨텍스트 전달 → 신화 크라켄 출현 가능
- 전설/신화 어종 낚시 시 전 서버 알림
- ach_fish50 업적 자동 추적 (fish_catch)

v1.20부터 만든 6개 신규 모듈 중 두 번째 통합.

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutoBattle_io_기획서.xlsx
+++ b/AutoBattle_io_기획서.xlsx
@@ -40,7 +40,7 @@
     <sheet name="월드 보스" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="연금술" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="패치 노트" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="v1.9 ~ v1.26" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="v1.9 ~ v1.27" sheetId="34" state="visible" r:id="rId34"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -13685,7 +13685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13726,7 +13726,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -13741,14 +13741,14 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>game/lottery.js → server.js 통합 (require + 소켓 핸들러 3종)</t>
+          <t>game/fishing.js → server.js 통합 (소켓 핸들러 3종)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -13758,19 +13758,19 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>룰렛</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>lottery_status / lottery_free_spin / lottery_paid_spin 이벤트 추가</t>
+          <t>fishing_status / fishing_cast / fishing_buy_rod 이벤트</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
@@ -13780,19 +13780,19 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>룰렛</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>전설/영웅 보상 획득 시 전 서버 알림 + ach_lucky 업적 추적</t>
+          <t>지역 검증 (낚시 만/강변/산호초), 낚싯대 보유 검증, 미끼 소비</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -13802,19 +13802,19 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>입찰식 경매 시스템 (game/auction.js 신규 모듈)</t>
+          <t>전설/신화 어종 낚시 시 전 서버 알림 + ach_fish50 추적</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -13824,19 +13824,19 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>3가지 기간(1h/6h/24h) + 등록2% + 낙찰5% + 스나이핑 방지</t>
+          <t>game/lottery.js → server.js 통합 (require + 소켓 핸들러 3종)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -13846,19 +13846,19 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>룰렛</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>경매장 시트 신규 추가</t>
+          <t>lottery_status / lottery_free_spin / lottery_paid_spin 이벤트 추가</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -13868,19 +13868,19 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>룰렛</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>11종 어종 + 5등급 낚싯대 + 4종 미끼 (game/fishing.js 신규 모듈)</t>
+          <t>전설/영웅 보상 획득 시 전 서버 알림 + ach_lucky 업적 추적</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -13890,19 +13890,19 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>신화 크라켄 (밤+낚시터+드래곤대 한정), 바다의 군주 칭호 연계</t>
+          <t>입찰식 경매 시스템 (game/auction.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -13912,19 +13912,19 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>낚시 시트 신규 추가</t>
+          <t>3가지 기간(1h/6h/24h) + 등록2% + 낙찰5% + 스나이핑 방지</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -13934,19 +13934,19 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>20웨이브 엔드리스 보스 러시 모드 (game/boss_rush.js 신규 모듈)</t>
+          <t>경매장 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -13956,19 +13956,19 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>매일 무료 3회 + 랭킹 1위 챔피언 칭호</t>
+          <t>11종 어종 + 5등급 낚싯대 + 4종 미끼 (game/fishing.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -13978,19 +13978,19 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>보스 러시 시트 신규 추가</t>
+          <t>신화 크라켄 (밤+낚시터+드래곤대 한정), 바다의 군주 칭호 연계</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
@@ -14000,19 +14000,19 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>행운의 룰렛</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>10종 보상 + 가중치 시스템 (game/lottery.js 신규 모듈)</t>
+          <t>낚시 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
@@ -14022,19 +14022,19 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>룰렛</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>매일 무료 1회 / 유료 50💎 / 10연속 450💎 (10% 할인)</t>
+          <t>20웨이브 엔드리스 보스 러시 모드 (game/boss_rush.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -14044,19 +14044,19 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>행운의 룰렛 시트 신규 추가</t>
+          <t>매일 무료 3회 + 랭킹 1위 챔피언 칭호</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
@@ -14066,19 +14066,19 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>5종 시즌 축제 추가 (신년/봄꽃/한여름/할로윈/겨울)</t>
+          <t>보스 러시 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -14088,19 +14088,19 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>모듈화</t>
+          <t>행운의 룰렛</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>game/event.js 신규 파일 (실제 달력 기반 자동 활성화)</t>
+          <t>10종 보상 + 가중치 시스템 (game/lottery.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
@@ -14110,19 +14110,19 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>룰렛</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트 시트 신규 추가</t>
+          <t>매일 무료 1회 / 유료 50💎 / 10연속 450💎 (10% 할인)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -14132,19 +14132,19 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>15티어 배틀 패스 시스템 추가 (game/season.js 신규 모듈)</t>
+          <t>행운의 룰렛 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
@@ -14154,19 +14154,19 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>30일 사이클, 무료+프리미엄(1500💎) 트랙</t>
+          <t>5종 시즌 축제 추가 (신년/봄꽃/한여름/할로윈/겨울)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -14176,19 +14176,19 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>모듈화</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>시즌 패스 시트 신규 추가</t>
+          <t>game/event.js 신규 파일 (실제 달력 기반 자동 활성화)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
@@ -14198,19 +14198,19 @@
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>마일스톤 5종 추가 (Lv.40/50, 첫 환생, 첫 월드 보스, 업적 50)</t>
+          <t>축제 이벤트 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -14220,19 +14220,19 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>무료 다이아 시트 신규 추가</t>
+          <t>15티어 배틀 패스 시스템 추가 (game/season.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
@@ -14242,19 +14242,19 @@
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>상점</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>프리미엄 5종 추가 (불사조/폭풍 스킨, 자동물약 24h, 보물상자, 재료 패키지)</t>
+          <t>30일 사이클, 무료+프리미엄(1500💎) 트랙</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -14269,14 +14269,14 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>상점 시트 갱신</t>
+          <t>시즌 패스 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
@@ -14286,19 +14286,19 @@
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>혈맹</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>혈맹 Lv.6-10 + 신규 스킬 5종 (분노/신속/회복/운명/전설)</t>
+          <t>마일스톤 5종 추가 (Lv.40/50, 첫 환생, 첫 월드 보스, 업적 50)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -14308,19 +14308,19 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>혈맹</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>최대 인원 50→100명 (Lv.10 기준)</t>
+          <t>무료 다이아 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
@@ -14330,19 +14330,19 @@
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>상점</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>길드(혈맹) 시트 신규 추가</t>
+          <t>프리미엄 5종 추가 (불사조/폭풍 스킨, 자동물약 24h, 보물상자, 재료 패키지)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -14352,19 +14352,19 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>점쟁이/감정사/수집가 3종 추가 (운세/감정/희귀품 매입)</t>
+          <t>상점 시트 갱신</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
@@ -14374,19 +14374,19 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>대사 시스템</t>
+          <t>혈맹</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>신규 NPC 상황별 대사 (밤/카르마/레벨/골드 연동)</t>
+          <t>혈맹 Lv.6-10 + 신규 스킬 5종 (분노/신속/회복/운명/전설)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -14396,19 +14396,19 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>혈맹</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>NPC 시트 신규 추가 (11종)</t>
+          <t>최대 인원 50→100명 (Lv.10 기준)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
@@ -14418,19 +14418,19 @@
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>각성기</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>클래스별 Lv.40 각성기 5종 추가 (천개의칼날/대지가르기/불멸의수호자/시간정지/신의은총)</t>
+          <t>길드(혈맹) 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -14440,19 +14440,19 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>스킬 시트 전면 갱신 (12종→30종, 클레릭 포함)</t>
+          <t>점쟁이/감정사/수집가 3종 추가 (운세/감정/희귀품 매입)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
@@ -14462,19 +14462,19 @@
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>대사 시스템</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>v1.9~v1.13 컨텐츠 연계 업적 5종 추가 (폭풍 정복자/연금술사/그림자/전설 동반자/이국 상인)</t>
+          <t>신규 NPC 상황별 대사 (밤/카르마/레벨/골드 연동)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -14489,14 +14489,14 @@
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>퀘스트 시트 전면 갱신 (9종→64종 반영)</t>
+          <t>NPC 시트 신규 추가 (11종)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
@@ -14506,19 +14506,19 @@
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>월드 보스</t>
+          <t>각성기</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>폭풍의 거인 / 시간의 수호자 2종 추가 (최대 HP / 최강 ATK)</t>
+          <t>클래스별 Lv.40 각성기 5종 추가 (천개의칼날/대지가르기/불멸의수호자/시간정지/신의은총)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -14528,19 +14528,19 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>교역</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>이국의 사치품 3종 추가 (불사조 깃털/공허의 정수/천공의 비단)</t>
+          <t>스킬 시트 전면 갱신 (12종→30종, 클레릭 포함)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
@@ -14550,19 +14550,19 @@
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>월드 보스 시트 신규 추가, 교역 시트 갱신</t>
+          <t>v1.9~v1.13 컨텐츠 연계 업적 5종 추가 (폭풍 정복자/연금술사/그림자/전설 동반자/이국 상인)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -14572,19 +14572,19 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>엘릭서 5종 추가 (타이탄/강철/질풍/지혜/행운, 15~30분 강력 버프)</t>
+          <t>퀘스트 시트 전면 갱신 (9종→64종 반영)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
@@ -14594,19 +14594,19 @@
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>월드 보스</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>연금술 시트 신규 추가</t>
+          <t>폭풍의 거인 / 시간의 수호자 2종 추가 (최대 HP / 최강 ATK)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -14616,19 +14616,19 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>신규 펫</t>
+          <t>교역</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>불사조 (화염 +20%) / 유니콘 (회피 +10%) + 진화형</t>
+          <t>이국의 사치품 3종 추가 (불사조 깃털/공허의 정수/천공의 비단)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
@@ -14638,19 +14638,19 @@
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>신규 탈것</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>페가수스 (이동 +85%, 비행)</t>
+          <t>월드 보스 시트 신규 추가, 교역 시트 갱신</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -14660,19 +14660,19 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>신규 던전</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>그림자 미궁 (Lv.38, 8인 파티, 7스테이지, 전설 드롭)</t>
+          <t>엘릭서 5종 추가 (타이탄/강철/질풍/지혜/행운, 15~30분 강력 버프)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
@@ -14687,14 +14687,14 @@
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>던전 시트 신규 추가 (7종 던전 정리)</t>
+          <t>연금술 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -14704,19 +14704,19 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 펫</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>공허의 방랑자/불멸자/천공의 군주 3종 추가 (엔드게임)</t>
+          <t>불사조 (화염 +20%) / 유니콘 (회피 +10%) + 진화형</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
@@ -14726,107 +14726,107 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>신규 탈것</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>51개 지역, 16종 칭호, 출석/세트/등급 시트 추가</t>
+          <t>페가수스 (이동 +85%, 비행)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>신규 던전</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>패치 노트 갱신, 낮/밤 시계 + 진행 시간 표시</t>
+          <t>그림자 미궁 (Lv.38, 8인 파티, 7스테이지, 전설 드롭)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>자동화</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>자동 스킬 시전 (인간 플레이어용), 자동 스킬 토글 버튼</t>
+          <t>던전 시트 신규 추가 (7종 던전 정리)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>미니맵 친구 위치 표시, 보스 표시 강화, DPS 미터 스파크라인</t>
+          <t>공허의 방랑자/불멸자/천공의 군주 3종 추가 (엔드게임)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>시스템</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>혈맹 창고 UI 패널, 보스 신규 디버프 적용</t>
+          <t>51개 지역, 16종 칭호, 출석/세트/등급 시트 추가</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -14836,19 +14836,19 @@
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>상태이상</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>신규 디버프 5종 (빙결/감전/출혈/약화/공포)</t>
+          <t>패치 노트 갱신, 낮/밤 시계 + 진행 시간 표시</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
@@ -14858,19 +14858,19 @@
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>자동화</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>포션 단축키 (1/2/3/4), 레벨별 추천 활동 가이드</t>
+          <t>자동 스킬 시전 (인간 플레이어용), 자동 스킬 토글 버튼</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -14880,19 +14880,19 @@
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>시스템</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>장비 자동 최적화 (auto_equip_best), 알림 센터</t>
+          <t>미니맵 친구 위치 표시, 보스 표시 강화, DPS 미터 스파크라인</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
@@ -14902,12 +14902,12 @@
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>컨텐츠</t>
+          <t>시스템</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>신규 업적 10종 (30→40), 신규 몬스터 존 3개</t>
+          <t>혈맹 창고 UI 패널, 보스 신규 디버프 적용</t>
         </is>
       </c>
     </row>
@@ -14924,32 +14924,120 @@
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>상태이상</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>인벤토리 검색 + 정렬, PvP 시즌 보드 시각화</t>
+          <t>신규 디버프 5종 (빙결/감전/출혈/약화/공포)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B59" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>포션 단축키 (1/2/3/4), 레벨별 추천 활동 가이드</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>시스템</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>장비 자동 최적화 (auto_equip_best), 알림 센터</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
+        <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B61" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>컨텐츠</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>신규 업적 10종 (30→40), 신규 몬스터 존 3개</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>인벤토리 검색 + 정렬, PvP 시즌 보드 시각화</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
+        <is>
           <t>v1.6 이전</t>
         </is>
       </c>
-      <c r="B59" s="8" t="inlineStr">
+      <c r="B63" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C59" s="8" t="inlineStr">
+      <c r="C63" s="8" t="inlineStr">
         <is>
           <t>기반</t>
         </is>
       </c>
-      <c r="D59" s="8" t="inlineStr">
+      <c r="D63" s="8" t="inlineStr">
         <is>
           <t>마을/사냥/PvP/카르마/펫/탈것/제작/교역/길드/공성/투기장 등</t>
         </is>
@@ -14969,7 +15057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -15016,7 +15104,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -15026,7 +15114,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>lottery → server.js</t>
+          <t>fishing → server.js</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -15036,29 +15124,29 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>첫 모듈 통합 마일스톤</t>
+          <t>두 번째 모듈 통합</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>소켓 이벤트</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>lottery_status</t>
+          <t>fishing_status</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>상태/가격/상품 풀 조회</t>
+          <t>지역/낚싯대/미끼/시간대 조회</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -15070,432 +15158,432 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>소켓 이벤트</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>lottery_free_spin</t>
+          <t>fishing_cast</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>매일 무료 1회 스핀</t>
+          <t>낚시 시도 (지역+낚싯대+미끼 검증)</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>자정 초기화</t>
+          <t>전설/신화 → 서버 알림</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>소켓 이벤트</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>lottery_paid_spin</t>
+          <t>fishing_buy_rod</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>유료 1회 / 10연속</t>
+          <t>낚싯대 구매 (골드/다이아)</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>count: 1 또는 10</t>
+          <t>5등급 모두</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>game/auction.js 신규</t>
+          <t>lottery → server.js</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>입찰식 / 3기간 / 5% 인상 / 스나이핑 방지</t>
+          <t>require + 소켓 핸들러 3종</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>등록 2% + 낙찰 5%</t>
+          <t>첫 모듈 통합 마일스톤</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>소켓 이벤트</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>활성 한도</t>
+          <t>lottery_status</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>플레이어당 10개</t>
+          <t>상태/가격/상품 풀 조회</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>자기 입찰 금지</t>
+          <t>클라이언트 표시용</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>소켓 이벤트</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>game/fishing.js 신규</t>
+          <t>lottery_free_spin</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>11종 어종 / 5등급 낚싯대 / 4종 미끼</t>
+          <t>매일 무료 1회 스핀</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>신화 크라켄 = 20000G + 칭호</t>
+          <t>자정 초기화</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>소켓 이벤트</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>전설의 비단잉어</t>
+          <t>lottery_paid_spin</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>드래곤 낚싯대 + 가중치 1</t>
+          <t>유료 1회 / 10연속</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>5000G + 평생 행운 +5%</t>
+          <t>count: 1 또는 10</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>game/boss_rush.js 신규</t>
+          <t>game/auction.js 신규</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>20웨이브 / HP ×1.35 스케일링</t>
+          <t>입찰식 / 3기간 / 5% 인상 / 스나이핑 방지</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>최종 보상: 200💎 + 용재료 ×5</t>
+          <t>등록 2% + 낙찰 5%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>입장</t>
+          <t>활성 한도</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>매일 무료 3회 / 1000G / 30💎</t>
+          <t>플레이어당 10개</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>랭킹 시스템</t>
+          <t>자기 입찰 금지</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>챔피언 보상</t>
+          <t>game/fishing.js 신규</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>1위: 500💎 + 칭호 / 2위: 300💎 / 3위: 200💎</t>
+          <t>11종 어종 / 5등급 낚싯대 / 4종 미끼</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>신화 크라켄 = 20000G + 칭호</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>행운의 룰렛</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>game/lottery.js 신규</t>
+          <t>전설의 비단잉어</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>10종 보상 / 가중치 1000</t>
+          <t>드래곤 낚싯대 + 가중치 1</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>매일 무료 1회 + 유료</t>
+          <t>5000G + 평생 행운 +5%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>룰렛 (전설)</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>영웅 장비 상자</t>
+          <t>game/boss_rush.js 신규</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>확률 0.2% (가장 희귀)</t>
+          <t>20웨이브 / HP ×1.35 스케일링</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>전설 보상</t>
+          <t>최종 보상: 200💎 + 용재료 ×5</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>룰렛 (전설)</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>200 다이아</t>
+          <t>입장</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>확률 0.8%</t>
+          <t>매일 무료 3회 / 1000G / 30💎</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>잭팟</t>
+          <t>랭킹 시스템</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>신년 축제</t>
+          <t>챔피언 보상</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>1/1 ~ 1/7</t>
+          <t>1위: 500💎 + 칭호 / 2위: 300💎 / 3위: 200💎</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>골드 +50% / EXP +30%</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>행운의 룰렛</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>봄꽃 축제</t>
+          <t>game/lottery.js 신규</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>4/1 ~ 4/14</t>
+          <t>10종 보상 / 가중치 1000</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>HP재생 +30% / 드롭 +20%</t>
+          <t>매일 무료 1회 + 유료</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>룰렛 (전설)</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>한여름 밤의 축제</t>
+          <t>영웅 장비 상자</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>7/15 ~ 8/15</t>
+          <t>확률 0.2% (가장 희귀)</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>화염 +30% / PvP 보상 +50%</t>
+          <t>전설 보상</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>룰렛 (전설)</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>할로윈 축제</t>
+          <t>200 다이아</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>10/25 ~ 11/1</t>
+          <t>확률 0.8%</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>크리 +10% / 언데드 +50%</t>
+          <t>잭팟</t>
         </is>
       </c>
     </row>
@@ -15512,206 +15600,206 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>겨울 축제</t>
+          <t>신년 축제</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>12/20 ~ 12/31</t>
+          <t>1/1 ~ 1/7</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>골드 +30% / EXP +30% / 드롭 +30%</t>
+          <t>골드 +50% / EXP +30%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>game/season.js 신규</t>
+          <t>봄꽃 축제</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>15티어 / 30일 / 무료+프리미엄</t>
+          <t>4/1 ~ 4/14</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>만렙 보상: 태초 반지 + 시즌 칭호</t>
+          <t>HP재생 +30% / 드롭 +20%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>XP 획득 7종</t>
+          <t>한여름 밤의 축제</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>퀘/보스/PvP/월드보스/던전/제작</t>
+          <t>7/15 ~ 8/15</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>일일 +200 ~ 월드보스 +500</t>
+          <t>화염 +30% / PvP 보상 +50%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>프리미엄 가격</t>
+          <t>할로윈 축제</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>1500 다이아</t>
+          <t>10/25 ~ 11/1</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>시즌 당 1회</t>
+          <t>크리 +10% / 언데드 +50%</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Lv.40 달성</t>
+          <t>겨울 축제</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>각성기 해금 마일스톤</t>
+          <t>12/20 ~ 12/31</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>150💎</t>
+          <t>골드 +30% / EXP +30% / 드롭 +30%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Lv.50 달성</t>
+          <t>game/season.js 신규</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>환생 가능 마일스톤</t>
+          <t>15티어 / 30일 / 무료+프리미엄</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>250💎</t>
+          <t>만렙 보상: 태초 반지 + 시즌 칭호</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>첫 환생</t>
+          <t>XP 획득 7종</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>prestige 1차</t>
+          <t>퀘/보스/PvP/월드보스/던전/제작</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>500💎</t>
+          <t>일일 +200 ~ 월드보스 +500</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>첫 월드 보스</t>
+          <t>프리미엄 가격</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>월드 보스 처치 보너스</t>
+          <t>1500 다이아</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>100💎</t>
+          <t>시즌 당 1회</t>
         </is>
       </c>
     </row>
@@ -15728,125 +15816,125 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>업적 50개</t>
+          <t>Lv.40 달성</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>업적 마일스톤</t>
+          <t>각성기 해금 마일스톤</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>200💎</t>
+          <t>150💎</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>상점 (스킨)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>불사조 스킨</t>
+          <t>Lv.50 달성</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>1200 다이아</t>
+          <t>환생 가능 마일스톤</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>불사조 깃털 이펙트 (영구)</t>
+          <t>250💎</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>상점 (스킨)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>폭풍 스킨</t>
+          <t>첫 환생</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>1200 다이아</t>
+          <t>prestige 1차</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>번개 오라 이펙트 (영구)</t>
+          <t>500💎</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>상점 (편의)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>프리미엄 자동물약</t>
+          <t>첫 월드 보스</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>500 다이아</t>
+          <t>월드 보스 처치 보너스</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>24시간 자동물약 무한</t>
+          <t>100💎</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>상점 (상자)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>프리미엄 보물 상자</t>
+          <t>업적 50개</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>300 다이아</t>
+          <t>업적 마일스톤</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>전설 장비 확정 + 다이아</t>
+          <t>200💎</t>
         </is>
       </c>
     </row>
@@ -15858,130 +15946,130 @@
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>상점 (재료)</t>
+          <t>상점 (스킨)</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>전설 재료 패키지</t>
+          <t>불사조 스킨</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>600 다이아</t>
+          <t>1200 다이아</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>용재료×10 + 영혼석×20 + 마법재료×20</t>
+          <t>불사조 깃털 이펙트 (영구)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>혈맹 Lv.6</t>
+          <t>상점 (스킨)</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>혈맹의 분노</t>
+          <t>폭풍 스킨</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>크리티컬 +5%</t>
+          <t>1200 다이아</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>60명 정원</t>
+          <t>번개 오라 이펙트 (영구)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>혈맹 Lv.7</t>
+          <t>상점 (편의)</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>혈맹의 신속</t>
+          <t>프리미엄 자동물약</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>이동속도 +10%</t>
+          <t>500 다이아</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>70명 정원</t>
+          <t>24시간 자동물약 무한</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>혈맹 Lv.8</t>
+          <t>상점 (상자)</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>혈맹의 회복</t>
+          <t>프리미엄 보물 상자</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>HP 재생 +50%</t>
+          <t>300 다이아</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>80명 정원</t>
+          <t>전설 장비 확정 + 다이아</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>혈맹 Lv.9</t>
+          <t>상점 (재료)</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>혈맹의 운명</t>
+          <t>전설 재료 패키지</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>회피 +5%</t>
+          <t>600 다이아</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>90명 정원</t>
+          <t>용재료×10 + 영혼석×20 + 마법재료×20</t>
         </is>
       </c>
     </row>
@@ -15993,211 +16081,211 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>혈맹 Lv.10</t>
+          <t>혈맹 Lv.6</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>혈맹의 전설</t>
+          <t>혈맹의 분노</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>전 스탯 +5%</t>
+          <t>크리티컬 +5%</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>100명 정원 — 최종</t>
+          <t>60명 정원</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>혈맹 Lv.7</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>점쟁이</t>
+          <t>혈맹의 신속</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>운세 / 행운 버프 (밤·카르마 반응)</t>
+          <t>이동속도 +10%</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>상황 대사 4종</t>
+          <t>70명 정원</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>혈맹 Lv.8</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>감정사</t>
+          <t>혈맹의 회복</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>미감정 장비 감정 (Lv.30+ 특수)</t>
+          <t>HP 재생 +50%</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>상황 대사 4종</t>
+          <t>80명 정원</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>혈맹 Lv.9</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>수집가</t>
+          <t>혈맹의 운명</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>희귀 아이템 매입 (골드 50000+ 특별)</t>
+          <t>회피 +5%</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>상황 대사 4종</t>
+          <t>90명 정원</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>각성기 (어쌔신)</t>
+          <t>혈맹 Lv.10</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>천 개의 칼날</t>
+          <t>혈맹의 전설</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>3.5배 × 7타 / 광역 / 쿨150초</t>
+          <t>전 스탯 +5%</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>100명 정원 — 최종</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>각성기 (워리어)</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>대지 가르기</t>
+          <t>점쟁이</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>6.0배 / 광역 5범위 / 스턴 2초</t>
+          <t>운세 / 행운 버프 (밤·카르마 반응)</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>상황 대사 4종</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>각성기 (나이트)</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>불멸의 수호자</t>
+          <t>감정사</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>피해 90% 감소 / 도발 / 10초</t>
+          <t>미감정 장비 감정 (Lv.30+ 특수)</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>상황 대사 4종</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>각성기 (메이지)</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>시간 정지</t>
+          <t>수집가</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>12.0배 / 광역 6범위 / 슬로우 90%</t>
+          <t>희귀 아이템 매입 (골드 50000+ 특별)</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>상황 대사 4종</t>
         </is>
       </c>
     </row>
@@ -16209,17 +16297,17 @@
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>각성기 (클레릭)</t>
+          <t>각성기 (어쌔신)</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>신의 은총</t>
+          <t>천 개의 칼날</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>HP 100% 회복 / 전스탯 +50%</t>
+          <t>3.5배 × 7타 / 광역 / 쿨150초</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
@@ -16231,108 +16319,108 @@
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (워리어)</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>폭풍 정복자</t>
+          <t>대지 가르기</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>폭풍의 거인 처치</t>
+          <t>6.0배 / 광역 5범위 / 스턴 2초</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>10,000G + 150다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (나이트)</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>연금술사</t>
+          <t>불멸의 수호자</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>엘릭서 10회 제작</t>
+          <t>피해 90% 감소 / 도발 / 10초</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>5,000G + 80다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (메이지)</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>그림자 정복자</t>
+          <t>시간 정지</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>그림자 미궁 클리어</t>
+          <t>12.0배 / 광역 6범위 / 슬로우 90%</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t>8,000G + 120다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (클레릭)</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>전설의 동반자</t>
+          <t>신의 은총</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>전설급 펫 진화</t>
+          <t>HP 100% 회복 / 전스탯 +50%</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>6,000G + 100다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
@@ -16349,206 +16437,206 @@
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>이국의 상인</t>
+          <t>폭풍 정복자</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>사치품 교역 5회</t>
+          <t>폭풍의 거인 처치</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
         <is>
-          <t>4,000G + 60다이아</t>
+          <t>10,000G + 150다이아</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>월드 보스</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>폭풍의 거인</t>
+          <t>연금술사</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>HP 100,000 / ATK 140 / DEF 90</t>
+          <t>엘릭서 10회 제작</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>EXP 10000 + 6000G</t>
+          <t>5,000G + 80다이아</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>월드 보스</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>시간의 수호자</t>
+          <t>그림자 정복자</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>HP 70,000 / ATK 170 / DEF 60</t>
+          <t>그림자 미궁 클리어</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t>EXP 9000 + 7000G</t>
+          <t>8,000G + 120다이아</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>교역품</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>불사조 깃털 / 공허의 정수 / 천공의 비단</t>
+          <t>전설의 동반자</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>이국의 사치품 3종</t>
+          <t>전설급 펫 진화</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>기본가 600~900G</t>
+          <t>6,000G + 100다이아</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>타이탄의 엘릭서</t>
+          <t>이국의 상인</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>용재료×3 + 마법재료×10</t>
+          <t>사치품 교역 5회</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t>ATK ×1.5 / 30분</t>
+          <t>4,000G + 60다이아</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>월드 보스</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>강철 엘릭서</t>
+          <t>폭풍의 거인</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>철광석×30 + 마법재료×10</t>
+          <t>HP 100,000 / ATK 140 / DEF 90</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>DEF ×1.5 / 30분</t>
+          <t>EXP 10000 + 6000G</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>월드 보스</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>질풍 엘릭서</t>
+          <t>시간의 수호자</t>
         </is>
       </c>
       <c r="D59" s="8" t="inlineStr">
         <is>
-          <t>약초×20 + 마법재료×8</t>
+          <t>HP 70,000 / ATK 170 / DEF 60</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t>SPD ×1.4 / 20분</t>
+          <t>EXP 9000 + 7000G</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>교역품</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>지혜 엘릭서</t>
+          <t>불사조 깃털 / 공허의 정수 / 천공의 비단</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>마법수정×5 + 영혼재료×5</t>
+          <t>이국의 사치품 3종</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>EXP ×2.5 / 15분</t>
+          <t>기본가 600~900G</t>
         </is>
       </c>
     </row>
@@ -16565,260 +16653,260 @@
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>행운 엘릭서</t>
+          <t>타이탄의 엘릭서</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>보석×10 + 마법재료×5</t>
+          <t>용재료×3 + 마법재료×10</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t>GOLD ×2.0 / 15분</t>
+          <t>ATK ×1.5 / 30분</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>신규 펫</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>불사조 (pet_phoenix)</t>
+          <t>강철 엘릭서</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>불꽃산 보스 50처치</t>
+          <t>철광석×30 + 마법재료×10</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>화염 DMG +20% (진화 +40%)</t>
+          <t>DEF ×1.5 / 30분</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>신규 펫</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>유니콘 (pet_unicorn)</t>
+          <t>질풍 엘릭서</t>
         </is>
       </c>
       <c r="D63" s="8" t="inlineStr">
         <is>
-          <t>다이아 800개</t>
+          <t>약초×20 + 마법재료×8</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t>회피 +10% (진화 +20%)</t>
+          <t>SPD ×1.4 / 20분</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>신규 탈것</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>페가수스 (mount_pegasus)</t>
+          <t>지혜 엘릭서</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>다이아 1200개</t>
+          <t>마법수정×5 + 영혼재료×5</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>이동속도 +85% / 비행</t>
+          <t>EXP ×2.5 / 15분</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>신규 던전</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>그림자 미궁</t>
+          <t>행운 엘릭서</t>
         </is>
       </c>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>Lv.38 / 8인 파티 / 7스테이지</t>
+          <t>보석×10 + 마법재료×5</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>22000G + 32000EXP</t>
+          <t>GOLD ×2.0 / 15분</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>드롭</t>
+          <t>신규 펫</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>드래곤 검/망토/투구/장갑</t>
+          <t>불사조 (pet_phoenix)</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>그림자 미궁 보스 드롭</t>
+          <t>불꽃산 보스 50처치</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>전설급</t>
+          <t>화염 DMG +20% (진화 +40%)</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 펫</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>공허의 방랑자</t>
+          <t>유니콘 (pet_unicorn)</t>
         </is>
       </c>
       <c r="D67" s="8" t="inlineStr">
         <is>
-          <t>몬스터 10,000 처치</t>
+          <t>다이아 800개</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t>ATK +7%</t>
+          <t>회피 +10% (진화 +20%)</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 탈것</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>불멸자</t>
+          <t>페가수스 (mount_pegasus)</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>환생 5회</t>
+          <t>다이아 1200개</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>EXP +25%</t>
+          <t>이동속도 +85% / 비행</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 던전</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>천공의 군주</t>
+          <t>그림자 미궁</t>
         </is>
       </c>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>월드 보스 10회 처치</t>
+          <t>Lv.38 / 8인 파티 / 7스테이지</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>보스DMG +15%</t>
+          <t>22000G + 32000EXP</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>드롭</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>지역 시트 갱신</t>
+          <t>드래곤 검/망토/투구/장갑</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>25→51개 지역 반영</t>
+          <t>그림자 미궁 보스 드롭</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>전설급</t>
         </is>
       </c>
     </row>
@@ -16830,22 +16918,22 @@
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>칭호 시트 갱신</t>
+          <t>공허의 방랑자</t>
         </is>
       </c>
       <c r="D71" s="8" t="inlineStr">
         <is>
-          <t>7→16종 + 효과/색상 추가</t>
+          <t>몬스터 10,000 처치</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ATK +7%</t>
         </is>
       </c>
     </row>
@@ -16857,22 +16945,22 @@
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>출석 캘린더 시트</t>
+          <t>불멸자</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>신규 추가 (28일 사이클)</t>
+          <t>환생 5회</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EXP +25%</t>
         </is>
       </c>
     </row>
@@ -16884,22 +16972,22 @@
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>장비 세트 시트</t>
+          <t>천공의 군주</t>
         </is>
       </c>
       <c r="D73" s="8" t="inlineStr">
         <is>
-          <t>신규 추가 (드래곤/영웅/태초)</t>
+          <t>월드 보스 10회 처치</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>보스DMG +15%</t>
         </is>
       </c>
     </row>
@@ -16916,12 +17004,12 @@
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>장비 등급 시트</t>
+          <t>지역 시트 갱신</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>신규 추가 (5등급 + 랜덤 옵션 7종)</t>
+          <t>25→51개 지역 반영</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
@@ -16943,12 +17031,12 @@
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t>디버프 시트</t>
+          <t>칭호 시트 갱신</t>
         </is>
       </c>
       <c r="D75" s="8" t="inlineStr">
         <is>
-          <t>신규 추가 (10종, v1.7 5종 포함)</t>
+          <t>7→16종 + 효과/색상 추가</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
@@ -16970,12 +17058,12 @@
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>패치 노트 시트</t>
+          <t>출석 캘린더 시트</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>신규 추가 (히스토리)</t>
+          <t>신규 추가 (28일 사이클)</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
@@ -16987,25 +17075,133 @@
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B77" s="8" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>장비 세트 시트</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="inlineStr">
+        <is>
+          <t>신규 추가 (드래곤/영웅/태초)</t>
+        </is>
+      </c>
+      <c r="E77" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="7" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>장비 등급 시트</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>신규 추가 (5등급 + 랜덤 옵션 7종)</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B79" s="8" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>디버프 시트</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="inlineStr">
+        <is>
+          <t>신규 추가 (10종, v1.7 5종 포함)</t>
+        </is>
+      </c>
+      <c r="E79" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="7" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B80" s="7" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C80" s="7" t="inlineStr">
+        <is>
+          <t>패치 노트 시트</t>
+        </is>
+      </c>
+      <c r="D80" s="7" t="inlineStr">
+        <is>
+          <t>신규 추가 (히스토리)</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="8" t="inlineStr">
+        <is>
           <t>v1.10</t>
         </is>
       </c>
-      <c r="B77" s="8" t="inlineStr">
+      <c r="B81" s="8" t="inlineStr">
         <is>
           <t>기획서</t>
         </is>
       </c>
-      <c r="C77" s="8" t="inlineStr">
+      <c r="C81" s="8" t="inlineStr">
         <is>
           <t>던전 시트</t>
         </is>
       </c>
-      <c r="D77" s="8" t="inlineStr">
+      <c r="D81" s="8" t="inlineStr">
         <is>
           <t>신규 추가 (7종 던전)</t>
         </is>
       </c>
-      <c r="E77" s="8" t="inlineStr">
+      <c r="E81" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
feat: v1.28 — game/event.js를 server.js에 통합 (3번째 모듈 통합)
축제 이벤트 시스템 활성화:
- require('./game/event') 추가 (festival 별칭)
- 소켓 핸들러: event_status — 현재 활성 축제 조회
  (이름/기간/글로벌 버프/한정 보상/NPC 인사 반환)
- /status JSON 엔드포인트에 festival 필드 추가
  (대시보드/모니터링용)
- getNpcMsg(): 축제 기간 중 30% 확률로 축제 인사 출력
  (모든 NPC 자동 적용)

검증: 오늘(2026-04-08) 봄꽃 축제 자동 활성 확인
"active event today: 봄꽃 축제"

5종 축제 자동 활성:
- 신년 (1/1~1/7) / 봄꽃 (4/1~4/14) / 한여름 (7/15~8/15)
  / 할로윈 (10/25~11/1) / 겨울 (12/20~12/31)

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutoBattle_io_기획서.xlsx
+++ b/AutoBattle_io_기획서.xlsx
@@ -40,7 +40,7 @@
     <sheet name="월드 보스" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="연금술" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="패치 노트" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="v1.9 ~ v1.27" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="v1.9 ~ v1.28" sheetId="34" state="visible" r:id="rId34"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -13685,7 +13685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13726,7 +13726,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -13741,14 +13741,14 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>game/fishing.js → server.js 통합 (소켓 핸들러 3종)</t>
+          <t>game/event.js → server.js 통합 (3번째 모듈 통합)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -13758,19 +13758,19 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>축제</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>fishing_status / fishing_cast / fishing_buy_rod 이벤트</t>
+          <t>event_status 소켓 + /status 엔드포인트 노출</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
@@ -13780,19 +13780,19 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>축제</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>지역 검증 (낚시 만/강변/산호초), 낚싯대 보유 검증, 미끼 소비</t>
+          <t>NPC 대사 30% 확률로 축제 인사 (getNpcMsg 통합)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -13802,19 +13802,19 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>검증</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>전설/신화 어종 낚시 시 전 서버 알림 + ach_fish50 추적</t>
+          <t>오늘(4/8) 봄꽃 축제 활성 동작 확인</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -13829,14 +13829,14 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>game/lottery.js → server.js 통합 (require + 소켓 핸들러 3종)</t>
+          <t>game/fishing.js → server.js 통합 (소켓 핸들러 3종)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -13846,19 +13846,19 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>룰렛</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>lottery_status / lottery_free_spin / lottery_paid_spin 이벤트 추가</t>
+          <t>fishing_status / fishing_cast / fishing_buy_rod 이벤트</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -13868,19 +13868,19 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>룰렛</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>전설/영웅 보상 획득 시 전 서버 알림 + ach_lucky 업적 추적</t>
+          <t>지역 검증 (낚시 만/강변/산호초), 낚싯대 보유 검증, 미끼 소비</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -13890,19 +13890,19 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>입찰식 경매 시스템 (game/auction.js 신규 모듈)</t>
+          <t>전설/신화 어종 낚시 시 전 서버 알림 + ach_fish50 추적</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -13912,19 +13912,19 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>3가지 기간(1h/6h/24h) + 등록2% + 낙찰5% + 스나이핑 방지</t>
+          <t>game/lottery.js → server.js 통합 (require + 소켓 핸들러 3종)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -13934,19 +13934,19 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>룰렛</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>경매장 시트 신규 추가</t>
+          <t>lottery_status / lottery_free_spin / lottery_paid_spin 이벤트 추가</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -13956,19 +13956,19 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>룰렛</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>11종 어종 + 5등급 낚싯대 + 4종 미끼 (game/fishing.js 신규 모듈)</t>
+          <t>전설/영웅 보상 획득 시 전 서버 알림 + ach_lucky 업적 추적</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -13978,19 +13978,19 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>신화 크라켄 (밤+낚시터+드래곤대 한정), 바다의 군주 칭호 연계</t>
+          <t>입찰식 경매 시스템 (game/auction.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
@@ -14000,19 +14000,19 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>낚시 시트 신규 추가</t>
+          <t>3가지 기간(1h/6h/24h) + 등록2% + 낙찰5% + 스나이핑 방지</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
@@ -14022,19 +14022,19 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>20웨이브 엔드리스 보스 러시 모드 (game/boss_rush.js 신규 모듈)</t>
+          <t>경매장 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -14044,19 +14044,19 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>매일 무료 3회 + 랭킹 1위 챔피언 칭호</t>
+          <t>11종 어종 + 5등급 낚싯대 + 4종 미끼 (game/fishing.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
@@ -14066,19 +14066,19 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>보스 러시 시트 신규 추가</t>
+          <t>신화 크라켄 (밤+낚시터+드래곤대 한정), 바다의 군주 칭호 연계</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -14088,19 +14088,19 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>행운의 룰렛</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>10종 보상 + 가중치 시스템 (game/lottery.js 신규 모듈)</t>
+          <t>낚시 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
@@ -14110,19 +14110,19 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>룰렛</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>매일 무료 1회 / 유료 50💎 / 10연속 450💎 (10% 할인)</t>
+          <t>20웨이브 엔드리스 보스 러시 모드 (game/boss_rush.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -14132,19 +14132,19 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>행운의 룰렛 시트 신규 추가</t>
+          <t>매일 무료 3회 + 랭킹 1위 챔피언 칭호</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
@@ -14154,19 +14154,19 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>5종 시즌 축제 추가 (신년/봄꽃/한여름/할로윈/겨울)</t>
+          <t>보스 러시 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -14176,19 +14176,19 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>모듈화</t>
+          <t>행운의 룰렛</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>game/event.js 신규 파일 (실제 달력 기반 자동 활성화)</t>
+          <t>10종 보상 + 가중치 시스템 (game/lottery.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
@@ -14198,19 +14198,19 @@
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>룰렛</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트 시트 신규 추가</t>
+          <t>매일 무료 1회 / 유료 50💎 / 10연속 450💎 (10% 할인)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -14220,19 +14220,19 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>15티어 배틀 패스 시스템 추가 (game/season.js 신규 모듈)</t>
+          <t>행운의 룰렛 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
@@ -14242,19 +14242,19 @@
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>30일 사이클, 무료+프리미엄(1500💎) 트랙</t>
+          <t>5종 시즌 축제 추가 (신년/봄꽃/한여름/할로윈/겨울)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -14264,19 +14264,19 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>모듈화</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>시즌 패스 시트 신규 추가</t>
+          <t>game/event.js 신규 파일 (실제 달력 기반 자동 활성화)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
@@ -14286,19 +14286,19 @@
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>마일스톤 5종 추가 (Lv.40/50, 첫 환생, 첫 월드 보스, 업적 50)</t>
+          <t>축제 이벤트 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -14308,19 +14308,19 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>무료 다이아 시트 신규 추가</t>
+          <t>15티어 배틀 패스 시스템 추가 (game/season.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
@@ -14330,19 +14330,19 @@
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>상점</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>프리미엄 5종 추가 (불사조/폭풍 스킨, 자동물약 24h, 보물상자, 재료 패키지)</t>
+          <t>30일 사이클, 무료+프리미엄(1500💎) 트랙</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -14357,14 +14357,14 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>상점 시트 갱신</t>
+          <t>시즌 패스 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
@@ -14374,19 +14374,19 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>혈맹</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>혈맹 Lv.6-10 + 신규 스킬 5종 (분노/신속/회복/운명/전설)</t>
+          <t>마일스톤 5종 추가 (Lv.40/50, 첫 환생, 첫 월드 보스, 업적 50)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -14396,19 +14396,19 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>혈맹</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>최대 인원 50→100명 (Lv.10 기준)</t>
+          <t>무료 다이아 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
@@ -14418,19 +14418,19 @@
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>상점</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>길드(혈맹) 시트 신규 추가</t>
+          <t>프리미엄 5종 추가 (불사조/폭풍 스킨, 자동물약 24h, 보물상자, 재료 패키지)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -14440,19 +14440,19 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>점쟁이/감정사/수집가 3종 추가 (운세/감정/희귀품 매입)</t>
+          <t>상점 시트 갱신</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
@@ -14462,19 +14462,19 @@
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>대사 시스템</t>
+          <t>혈맹</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>신규 NPC 상황별 대사 (밤/카르마/레벨/골드 연동)</t>
+          <t>혈맹 Lv.6-10 + 신규 스킬 5종 (분노/신속/회복/운명/전설)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -14484,19 +14484,19 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>혈맹</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>NPC 시트 신규 추가 (11종)</t>
+          <t>최대 인원 50→100명 (Lv.10 기준)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
@@ -14506,19 +14506,19 @@
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>각성기</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>클래스별 Lv.40 각성기 5종 추가 (천개의칼날/대지가르기/불멸의수호자/시간정지/신의은총)</t>
+          <t>길드(혈맹) 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -14528,19 +14528,19 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>스킬 시트 전면 갱신 (12종→30종, 클레릭 포함)</t>
+          <t>점쟁이/감정사/수집가 3종 추가 (운세/감정/희귀품 매입)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
@@ -14550,19 +14550,19 @@
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>대사 시스템</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>v1.9~v1.13 컨텐츠 연계 업적 5종 추가 (폭풍 정복자/연금술사/그림자/전설 동반자/이국 상인)</t>
+          <t>신규 NPC 상황별 대사 (밤/카르마/레벨/골드 연동)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -14577,14 +14577,14 @@
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>퀘스트 시트 전면 갱신 (9종→64종 반영)</t>
+          <t>NPC 시트 신규 추가 (11종)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
@@ -14594,19 +14594,19 @@
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>월드 보스</t>
+          <t>각성기</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>폭풍의 거인 / 시간의 수호자 2종 추가 (최대 HP / 최강 ATK)</t>
+          <t>클래스별 Lv.40 각성기 5종 추가 (천개의칼날/대지가르기/불멸의수호자/시간정지/신의은총)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -14616,19 +14616,19 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>교역</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>이국의 사치품 3종 추가 (불사조 깃털/공허의 정수/천공의 비단)</t>
+          <t>스킬 시트 전면 갱신 (12종→30종, 클레릭 포함)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
@@ -14638,19 +14638,19 @@
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>월드 보스 시트 신규 추가, 교역 시트 갱신</t>
+          <t>v1.9~v1.13 컨텐츠 연계 업적 5종 추가 (폭풍 정복자/연금술사/그림자/전설 동반자/이국 상인)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -14660,19 +14660,19 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>엘릭서 5종 추가 (타이탄/강철/질풍/지혜/행운, 15~30분 강력 버프)</t>
+          <t>퀘스트 시트 전면 갱신 (9종→64종 반영)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
@@ -14682,19 +14682,19 @@
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>월드 보스</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>연금술 시트 신규 추가</t>
+          <t>폭풍의 거인 / 시간의 수호자 2종 추가 (최대 HP / 최강 ATK)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -14704,19 +14704,19 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>신규 펫</t>
+          <t>교역</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>불사조 (화염 +20%) / 유니콘 (회피 +10%) + 진화형</t>
+          <t>이국의 사치품 3종 추가 (불사조 깃털/공허의 정수/천공의 비단)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
@@ -14726,19 +14726,19 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>신규 탈것</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>페가수스 (이동 +85%, 비행)</t>
+          <t>월드 보스 시트 신규 추가, 교역 시트 갱신</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -14748,19 +14748,19 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>신규 던전</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>그림자 미궁 (Lv.38, 8인 파티, 7스테이지, 전설 드롭)</t>
+          <t>엘릭서 5종 추가 (타이탄/강철/질풍/지혜/행운, 15~30분 강력 버프)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
@@ -14775,14 +14775,14 @@
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>던전 시트 신규 추가 (7종 던전 정리)</t>
+          <t>연금술 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -14792,19 +14792,19 @@
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 펫</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>공허의 방랑자/불멸자/천공의 군주 3종 추가 (엔드게임)</t>
+          <t>불사조 (화염 +20%) / 유니콘 (회피 +10%) + 진화형</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
@@ -14814,107 +14814,107 @@
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>신규 탈것</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>51개 지역, 16종 칭호, 출석/세트/등급 시트 추가</t>
+          <t>페가수스 (이동 +85%, 비행)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>신규 던전</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>패치 노트 갱신, 낮/밤 시계 + 진행 시간 표시</t>
+          <t>그림자 미궁 (Lv.38, 8인 파티, 7스테이지, 전설 드롭)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>자동화</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>자동 스킬 시전 (인간 플레이어용), 자동 스킬 토글 버튼</t>
+          <t>던전 시트 신규 추가 (7종 던전 정리)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>미니맵 친구 위치 표시, 보스 표시 강화, DPS 미터 스파크라인</t>
+          <t>공허의 방랑자/불멸자/천공의 군주 3종 추가 (엔드게임)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>시스템</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>혈맹 창고 UI 패널, 보스 신규 디버프 적용</t>
+          <t>51개 지역, 16종 칭호, 출석/세트/등급 시트 추가</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -14924,19 +14924,19 @@
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>상태이상</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>신규 디버프 5종 (빙결/감전/출혈/약화/공포)</t>
+          <t>패치 노트 갱신, 낮/밤 시계 + 진행 시간 표시</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
@@ -14946,19 +14946,19 @@
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>자동화</t>
         </is>
       </c>
       <c r="D59" s="8" t="inlineStr">
         <is>
-          <t>포션 단축키 (1/2/3/4), 레벨별 추천 활동 가이드</t>
+          <t>자동 스킬 시전 (인간 플레이어용), 자동 스킬 토글 버튼</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -14968,19 +14968,19 @@
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>시스템</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>장비 자동 최적화 (auto_equip_best), 알림 센터</t>
+          <t>미니맵 친구 위치 표시, 보스 표시 강화, DPS 미터 스파크라인</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
@@ -14990,12 +14990,12 @@
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>컨텐츠</t>
+          <t>시스템</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>신규 업적 10종 (30→40), 신규 몬스터 존 3개</t>
+          <t>혈맹 창고 UI 패널, 보스 신규 디버프 적용</t>
         </is>
       </c>
     </row>
@@ -15012,32 +15012,120 @@
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>상태이상</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>인벤토리 검색 + 정렬, PvP 시즌 보드 시각화</t>
+          <t>신규 디버프 5종 (빙결/감전/출혈/약화/공포)</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B63" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>포션 단축키 (1/2/3/4), 레벨별 추천 활동 가이드</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>시스템</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>장비 자동 최적화 (auto_equip_best), 알림 센터</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="inlineStr">
+        <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>컨텐츠</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>신규 업적 10종 (30→40), 신규 몬스터 존 3개</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="inlineStr">
+        <is>
+          <t>인벤토리 검색 + 정렬, PvP 시즌 보드 시각화</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
+        <is>
           <t>v1.6 이전</t>
         </is>
       </c>
-      <c r="B63" s="8" t="inlineStr">
+      <c r="B67" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C63" s="8" t="inlineStr">
+      <c r="C67" s="8" t="inlineStr">
         <is>
           <t>기반</t>
         </is>
       </c>
-      <c r="D63" s="8" t="inlineStr">
+      <c r="D67" s="8" t="inlineStr">
         <is>
           <t>마을/사냥/PvP/카르마/펫/탈것/제작/교역/길드/공성/투기장 등</t>
         </is>
@@ -15057,7 +15145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -15104,7 +15192,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -15114,24 +15202,24 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>fishing → server.js</t>
+          <t>event → server.js</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>require + 소켓 핸들러 3종</t>
+          <t>3번째 모듈 통합</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>두 번째 모듈 통합</t>
+          <t>축제 시스템 활성화</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -15141,78 +15229,78 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>fishing_status</t>
+          <t>event_status</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>지역/낚싯대/미끼/시간대 조회</t>
+          <t>현재 활성 축제 조회</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>클라이언트 표시용</t>
+          <t>이름/기간/버프/한정 보상</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>소켓</t>
+          <t>API</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>fishing_cast</t>
+          <t>/status JSON</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>낚시 시도 (지역+낚싯대+미끼 검증)</t>
+          <t>festival 필드 추가</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>전설/신화 → 서버 알림</t>
+          <t>대시보드 확인용</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>소켓</t>
+          <t>NPC</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>fishing_buy_rod</t>
+          <t>축제 인사</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>낚싯대 구매 (골드/다이아)</t>
+          <t>30% 확률로 NPC가 축제 대사 출력</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>5등급 모두</t>
+          <t>spring_blossom 등 5종</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -15222,7 +15310,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>lottery → server.js</t>
+          <t>fishing → server.js</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -15232,29 +15320,29 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>첫 모듈 통합 마일스톤</t>
+          <t>두 번째 모듈 통합</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>소켓 이벤트</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>lottery_status</t>
+          <t>fishing_status</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>상태/가격/상품 풀 조회</t>
+          <t>지역/낚싯대/미끼/시간대 조회</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -15266,432 +15354,432 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>소켓 이벤트</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>lottery_free_spin</t>
+          <t>fishing_cast</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>매일 무료 1회 스핀</t>
+          <t>낚시 시도 (지역+낚싯대+미끼 검증)</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>자정 초기화</t>
+          <t>전설/신화 → 서버 알림</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>소켓 이벤트</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>lottery_paid_spin</t>
+          <t>fishing_buy_rod</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>유료 1회 / 10연속</t>
+          <t>낚싯대 구매 (골드/다이아)</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>count: 1 또는 10</t>
+          <t>5등급 모두</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>game/auction.js 신규</t>
+          <t>lottery → server.js</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>입찰식 / 3기간 / 5% 인상 / 스나이핑 방지</t>
+          <t>require + 소켓 핸들러 3종</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>등록 2% + 낙찰 5%</t>
+          <t>첫 모듈 통합 마일스톤</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>소켓 이벤트</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>활성 한도</t>
+          <t>lottery_status</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>플레이어당 10개</t>
+          <t>상태/가격/상품 풀 조회</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>자기 입찰 금지</t>
+          <t>클라이언트 표시용</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>소켓 이벤트</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>game/fishing.js 신규</t>
+          <t>lottery_free_spin</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>11종 어종 / 5등급 낚싯대 / 4종 미끼</t>
+          <t>매일 무료 1회 스핀</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>신화 크라켄 = 20000G + 칭호</t>
+          <t>자정 초기화</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>소켓 이벤트</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>전설의 비단잉어</t>
+          <t>lottery_paid_spin</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>드래곤 낚싯대 + 가중치 1</t>
+          <t>유료 1회 / 10연속</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>5000G + 평생 행운 +5%</t>
+          <t>count: 1 또는 10</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>game/boss_rush.js 신규</t>
+          <t>game/auction.js 신규</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>20웨이브 / HP ×1.35 스케일링</t>
+          <t>입찰식 / 3기간 / 5% 인상 / 스나이핑 방지</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>최종 보상: 200💎 + 용재료 ×5</t>
+          <t>등록 2% + 낙찰 5%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>입장</t>
+          <t>활성 한도</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>매일 무료 3회 / 1000G / 30💎</t>
+          <t>플레이어당 10개</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>랭킹 시스템</t>
+          <t>자기 입찰 금지</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>챔피언 보상</t>
+          <t>game/fishing.js 신규</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>1위: 500💎 + 칭호 / 2위: 300💎 / 3위: 200💎</t>
+          <t>11종 어종 / 5등급 낚싯대 / 4종 미끼</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>신화 크라켄 = 20000G + 칭호</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>행운의 룰렛</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>game/lottery.js 신규</t>
+          <t>전설의 비단잉어</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>10종 보상 / 가중치 1000</t>
+          <t>드래곤 낚싯대 + 가중치 1</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>매일 무료 1회 + 유료</t>
+          <t>5000G + 평생 행운 +5%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>룰렛 (전설)</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>영웅 장비 상자</t>
+          <t>game/boss_rush.js 신규</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>확률 0.2% (가장 희귀)</t>
+          <t>20웨이브 / HP ×1.35 스케일링</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>전설 보상</t>
+          <t>최종 보상: 200💎 + 용재료 ×5</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>룰렛 (전설)</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>200 다이아</t>
+          <t>입장</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>확률 0.8%</t>
+          <t>매일 무료 3회 / 1000G / 30💎</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>잭팟</t>
+          <t>랭킹 시스템</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>신년 축제</t>
+          <t>챔피언 보상</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>1/1 ~ 1/7</t>
+          <t>1위: 500💎 + 칭호 / 2위: 300💎 / 3위: 200💎</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>골드 +50% / EXP +30%</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>행운의 룰렛</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>봄꽃 축제</t>
+          <t>game/lottery.js 신규</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>4/1 ~ 4/14</t>
+          <t>10종 보상 / 가중치 1000</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>HP재생 +30% / 드롭 +20%</t>
+          <t>매일 무료 1회 + 유료</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>룰렛 (전설)</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>한여름 밤의 축제</t>
+          <t>영웅 장비 상자</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>7/15 ~ 8/15</t>
+          <t>확률 0.2% (가장 희귀)</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>화염 +30% / PvP 보상 +50%</t>
+          <t>전설 보상</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>룰렛 (전설)</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>할로윈 축제</t>
+          <t>200 다이아</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>10/25 ~ 11/1</t>
+          <t>확률 0.8%</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>크리 +10% / 언데드 +50%</t>
+          <t>잭팟</t>
         </is>
       </c>
     </row>
@@ -15708,206 +15796,206 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>겨울 축제</t>
+          <t>신년 축제</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>12/20 ~ 12/31</t>
+          <t>1/1 ~ 1/7</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>골드 +30% / EXP +30% / 드롭 +30%</t>
+          <t>골드 +50% / EXP +30%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>game/season.js 신규</t>
+          <t>봄꽃 축제</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>15티어 / 30일 / 무료+프리미엄</t>
+          <t>4/1 ~ 4/14</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>만렙 보상: 태초 반지 + 시즌 칭호</t>
+          <t>HP재생 +30% / 드롭 +20%</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>XP 획득 7종</t>
+          <t>한여름 밤의 축제</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>퀘/보스/PvP/월드보스/던전/제작</t>
+          <t>7/15 ~ 8/15</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>일일 +200 ~ 월드보스 +500</t>
+          <t>화염 +30% / PvP 보상 +50%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>프리미엄 가격</t>
+          <t>할로윈 축제</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>1500 다이아</t>
+          <t>10/25 ~ 11/1</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>시즌 당 1회</t>
+          <t>크리 +10% / 언데드 +50%</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Lv.40 달성</t>
+          <t>겨울 축제</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>각성기 해금 마일스톤</t>
+          <t>12/20 ~ 12/31</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>150💎</t>
+          <t>골드 +30% / EXP +30% / 드롭 +30%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>Lv.50 달성</t>
+          <t>game/season.js 신규</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>환생 가능 마일스톤</t>
+          <t>15티어 / 30일 / 무료+프리미엄</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>250💎</t>
+          <t>만렙 보상: 태초 반지 + 시즌 칭호</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>첫 환생</t>
+          <t>XP 획득 7종</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>prestige 1차</t>
+          <t>퀘/보스/PvP/월드보스/던전/제작</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>500💎</t>
+          <t>일일 +200 ~ 월드보스 +500</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>첫 월드 보스</t>
+          <t>프리미엄 가격</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>월드 보스 처치 보너스</t>
+          <t>1500 다이아</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>100💎</t>
+          <t>시즌 당 1회</t>
         </is>
       </c>
     </row>
@@ -15924,125 +16012,125 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>업적 50개</t>
+          <t>Lv.40 달성</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>업적 마일스톤</t>
+          <t>각성기 해금 마일스톤</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>200💎</t>
+          <t>150💎</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>상점 (스킨)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>불사조 스킨</t>
+          <t>Lv.50 달성</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>1200 다이아</t>
+          <t>환생 가능 마일스톤</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>불사조 깃털 이펙트 (영구)</t>
+          <t>250💎</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>상점 (스킨)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>폭풍 스킨</t>
+          <t>첫 환생</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>1200 다이아</t>
+          <t>prestige 1차</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>번개 오라 이펙트 (영구)</t>
+          <t>500💎</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>상점 (편의)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>프리미엄 자동물약</t>
+          <t>첫 월드 보스</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>500 다이아</t>
+          <t>월드 보스 처치 보너스</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>24시간 자동물약 무한</t>
+          <t>100💎</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>상점 (상자)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>프리미엄 보물 상자</t>
+          <t>업적 50개</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>300 다이아</t>
+          <t>업적 마일스톤</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>전설 장비 확정 + 다이아</t>
+          <t>200💎</t>
         </is>
       </c>
     </row>
@@ -16054,130 +16142,130 @@
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>상점 (재료)</t>
+          <t>상점 (스킨)</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>전설 재료 패키지</t>
+          <t>불사조 스킨</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>600 다이아</t>
+          <t>1200 다이아</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>용재료×10 + 영혼석×20 + 마법재료×20</t>
+          <t>불사조 깃털 이펙트 (영구)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>혈맹 Lv.6</t>
+          <t>상점 (스킨)</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>혈맹의 분노</t>
+          <t>폭풍 스킨</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>크리티컬 +5%</t>
+          <t>1200 다이아</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>60명 정원</t>
+          <t>번개 오라 이펙트 (영구)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>혈맹 Lv.7</t>
+          <t>상점 (편의)</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>혈맹의 신속</t>
+          <t>프리미엄 자동물약</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>이동속도 +10%</t>
+          <t>500 다이아</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>70명 정원</t>
+          <t>24시간 자동물약 무한</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>혈맹 Lv.8</t>
+          <t>상점 (상자)</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>혈맹의 회복</t>
+          <t>프리미엄 보물 상자</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>HP 재생 +50%</t>
+          <t>300 다이아</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>80명 정원</t>
+          <t>전설 장비 확정 + 다이아</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>혈맹 Lv.9</t>
+          <t>상점 (재료)</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>혈맹의 운명</t>
+          <t>전설 재료 패키지</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>회피 +5%</t>
+          <t>600 다이아</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>90명 정원</t>
+          <t>용재료×10 + 영혼석×20 + 마법재료×20</t>
         </is>
       </c>
     </row>
@@ -16189,211 +16277,211 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>혈맹 Lv.10</t>
+          <t>혈맹 Lv.6</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>혈맹의 전설</t>
+          <t>혈맹의 분노</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>전 스탯 +5%</t>
+          <t>크리티컬 +5%</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>100명 정원 — 최종</t>
+          <t>60명 정원</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>혈맹 Lv.7</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>점쟁이</t>
+          <t>혈맹의 신속</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>운세 / 행운 버프 (밤·카르마 반응)</t>
+          <t>이동속도 +10%</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>상황 대사 4종</t>
+          <t>70명 정원</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>혈맹 Lv.8</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>감정사</t>
+          <t>혈맹의 회복</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>미감정 장비 감정 (Lv.30+ 특수)</t>
+          <t>HP 재생 +50%</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>상황 대사 4종</t>
+          <t>80명 정원</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>혈맹 Lv.9</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>수집가</t>
+          <t>혈맹의 운명</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>희귀 아이템 매입 (골드 50000+ 특별)</t>
+          <t>회피 +5%</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>상황 대사 4종</t>
+          <t>90명 정원</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>각성기 (어쌔신)</t>
+          <t>혈맹 Lv.10</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>천 개의 칼날</t>
+          <t>혈맹의 전설</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>3.5배 × 7타 / 광역 / 쿨150초</t>
+          <t>전 스탯 +5%</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>100명 정원 — 최종</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>각성기 (워리어)</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>대지 가르기</t>
+          <t>점쟁이</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>6.0배 / 광역 5범위 / 스턴 2초</t>
+          <t>운세 / 행운 버프 (밤·카르마 반응)</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>상황 대사 4종</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>각성기 (나이트)</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>불멸의 수호자</t>
+          <t>감정사</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>피해 90% 감소 / 도발 / 10초</t>
+          <t>미감정 장비 감정 (Lv.30+ 특수)</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>상황 대사 4종</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>각성기 (메이지)</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>시간 정지</t>
+          <t>수집가</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>12.0배 / 광역 6범위 / 슬로우 90%</t>
+          <t>희귀 아이템 매입 (골드 50000+ 특별)</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>상황 대사 4종</t>
         </is>
       </c>
     </row>
@@ -16405,17 +16493,17 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>각성기 (클레릭)</t>
+          <t>각성기 (어쌔신)</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>신의 은총</t>
+          <t>천 개의 칼날</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>HP 100% 회복 / 전스탯 +50%</t>
+          <t>3.5배 × 7타 / 광역 / 쿨150초</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
@@ -16427,108 +16515,108 @@
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (워리어)</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>폭풍 정복자</t>
+          <t>대지 가르기</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>폭풍의 거인 처치</t>
+          <t>6.0배 / 광역 5범위 / 스턴 2초</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
         <is>
-          <t>10,000G + 150다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (나이트)</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>연금술사</t>
+          <t>불멸의 수호자</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>엘릭서 10회 제작</t>
+          <t>피해 90% 감소 / 도발 / 10초</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>5,000G + 80다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (메이지)</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>그림자 정복자</t>
+          <t>시간 정지</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>그림자 미궁 클리어</t>
+          <t>12.0배 / 광역 6범위 / 슬로우 90%</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t>8,000G + 120다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (클레릭)</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>전설의 동반자</t>
+          <t>신의 은총</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>전설급 펫 진화</t>
+          <t>HP 100% 회복 / 전스탯 +50%</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>6,000G + 100다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
@@ -16545,206 +16633,206 @@
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>이국의 상인</t>
+          <t>폭풍 정복자</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>사치품 교역 5회</t>
+          <t>폭풍의 거인 처치</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t>4,000G + 60다이아</t>
+          <t>10,000G + 150다이아</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>월드 보스</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>폭풍의 거인</t>
+          <t>연금술사</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>HP 100,000 / ATK 140 / DEF 90</t>
+          <t>엘릭서 10회 제작</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>EXP 10000 + 6000G</t>
+          <t>5,000G + 80다이아</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>월드 보스</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>시간의 수호자</t>
+          <t>그림자 정복자</t>
         </is>
       </c>
       <c r="D59" s="8" t="inlineStr">
         <is>
-          <t>HP 70,000 / ATK 170 / DEF 60</t>
+          <t>그림자 미궁 클리어</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t>EXP 9000 + 7000G</t>
+          <t>8,000G + 120다이아</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>교역품</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>불사조 깃털 / 공허의 정수 / 천공의 비단</t>
+          <t>전설의 동반자</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>이국의 사치품 3종</t>
+          <t>전설급 펫 진화</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>기본가 600~900G</t>
+          <t>6,000G + 100다이아</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>타이탄의 엘릭서</t>
+          <t>이국의 상인</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>용재료×3 + 마법재료×10</t>
+          <t>사치품 교역 5회</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t>ATK ×1.5 / 30분</t>
+          <t>4,000G + 60다이아</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>월드 보스</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>강철 엘릭서</t>
+          <t>폭풍의 거인</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>철광석×30 + 마법재료×10</t>
+          <t>HP 100,000 / ATK 140 / DEF 90</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>DEF ×1.5 / 30분</t>
+          <t>EXP 10000 + 6000G</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>월드 보스</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>질풍 엘릭서</t>
+          <t>시간의 수호자</t>
         </is>
       </c>
       <c r="D63" s="8" t="inlineStr">
         <is>
-          <t>약초×20 + 마법재료×8</t>
+          <t>HP 70,000 / ATK 170 / DEF 60</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t>SPD ×1.4 / 20분</t>
+          <t>EXP 9000 + 7000G</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>교역품</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>지혜 엘릭서</t>
+          <t>불사조 깃털 / 공허의 정수 / 천공의 비단</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>마법수정×5 + 영혼재료×5</t>
+          <t>이국의 사치품 3종</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>EXP ×2.5 / 15분</t>
+          <t>기본가 600~900G</t>
         </is>
       </c>
     </row>
@@ -16761,260 +16849,260 @@
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>행운 엘릭서</t>
+          <t>타이탄의 엘릭서</t>
         </is>
       </c>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>보석×10 + 마법재료×5</t>
+          <t>용재료×3 + 마법재료×10</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>GOLD ×2.0 / 15분</t>
+          <t>ATK ×1.5 / 30분</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>신규 펫</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>불사조 (pet_phoenix)</t>
+          <t>강철 엘릭서</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>불꽃산 보스 50처치</t>
+          <t>철광석×30 + 마법재료×10</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>화염 DMG +20% (진화 +40%)</t>
+          <t>DEF ×1.5 / 30분</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>신규 펫</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>유니콘 (pet_unicorn)</t>
+          <t>질풍 엘릭서</t>
         </is>
       </c>
       <c r="D67" s="8" t="inlineStr">
         <is>
-          <t>다이아 800개</t>
+          <t>약초×20 + 마법재료×8</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t>회피 +10% (진화 +20%)</t>
+          <t>SPD ×1.4 / 20분</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>신규 탈것</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>페가수스 (mount_pegasus)</t>
+          <t>지혜 엘릭서</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>다이아 1200개</t>
+          <t>마법수정×5 + 영혼재료×5</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>이동속도 +85% / 비행</t>
+          <t>EXP ×2.5 / 15분</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>신규 던전</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>그림자 미궁</t>
+          <t>행운 엘릭서</t>
         </is>
       </c>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>Lv.38 / 8인 파티 / 7스테이지</t>
+          <t>보석×10 + 마법재료×5</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>22000G + 32000EXP</t>
+          <t>GOLD ×2.0 / 15분</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>드롭</t>
+          <t>신규 펫</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>드래곤 검/망토/투구/장갑</t>
+          <t>불사조 (pet_phoenix)</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>그림자 미궁 보스 드롭</t>
+          <t>불꽃산 보스 50처치</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>전설급</t>
+          <t>화염 DMG +20% (진화 +40%)</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 펫</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>공허의 방랑자</t>
+          <t>유니콘 (pet_unicorn)</t>
         </is>
       </c>
       <c r="D71" s="8" t="inlineStr">
         <is>
-          <t>몬스터 10,000 처치</t>
+          <t>다이아 800개</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t>ATK +7%</t>
+          <t>회피 +10% (진화 +20%)</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 탈것</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>불멸자</t>
+          <t>페가수스 (mount_pegasus)</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>환생 5회</t>
+          <t>다이아 1200개</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>EXP +25%</t>
+          <t>이동속도 +85% / 비행</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 던전</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>천공의 군주</t>
+          <t>그림자 미궁</t>
         </is>
       </c>
       <c r="D73" s="8" t="inlineStr">
         <is>
-          <t>월드 보스 10회 처치</t>
+          <t>Lv.38 / 8인 파티 / 7스테이지</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t>보스DMG +15%</t>
+          <t>22000G + 32000EXP</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>드롭</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>지역 시트 갱신</t>
+          <t>드래곤 검/망토/투구/장갑</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>25→51개 지역 반영</t>
+          <t>그림자 미궁 보스 드롭</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>전설급</t>
         </is>
       </c>
     </row>
@@ -17026,22 +17114,22 @@
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t>칭호 시트 갱신</t>
+          <t>공허의 방랑자</t>
         </is>
       </c>
       <c r="D75" s="8" t="inlineStr">
         <is>
-          <t>7→16종 + 효과/색상 추가</t>
+          <t>몬스터 10,000 처치</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ATK +7%</t>
         </is>
       </c>
     </row>
@@ -17053,22 +17141,22 @@
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>출석 캘린더 시트</t>
+          <t>불멸자</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>신규 추가 (28일 사이클)</t>
+          <t>환생 5회</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EXP +25%</t>
         </is>
       </c>
     </row>
@@ -17080,22 +17168,22 @@
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t>장비 세트 시트</t>
+          <t>천공의 군주</t>
         </is>
       </c>
       <c r="D77" s="8" t="inlineStr">
         <is>
-          <t>신규 추가 (드래곤/영웅/태초)</t>
+          <t>월드 보스 10회 처치</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>보스DMG +15%</t>
         </is>
       </c>
     </row>
@@ -17112,12 +17200,12 @@
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>장비 등급 시트</t>
+          <t>지역 시트 갱신</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>신규 추가 (5등급 + 랜덤 옵션 7종)</t>
+          <t>25→51개 지역 반영</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
@@ -17139,12 +17227,12 @@
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>디버프 시트</t>
+          <t>칭호 시트 갱신</t>
         </is>
       </c>
       <c r="D79" s="8" t="inlineStr">
         <is>
-          <t>신규 추가 (10종, v1.7 5종 포함)</t>
+          <t>7→16종 + 효과/색상 추가</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
@@ -17166,12 +17254,12 @@
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>패치 노트 시트</t>
+          <t>출석 캘린더 시트</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>신규 추가 (히스토리)</t>
+          <t>신규 추가 (28일 사이클)</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
@@ -17183,25 +17271,133 @@
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>장비 세트 시트</t>
+        </is>
+      </c>
+      <c r="D81" s="8" t="inlineStr">
+        <is>
+          <t>신규 추가 (드래곤/영웅/태초)</t>
+        </is>
+      </c>
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="7" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C82" s="7" t="inlineStr">
+        <is>
+          <t>장비 등급 시트</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="inlineStr">
+        <is>
+          <t>신규 추가 (5등급 + 랜덤 옵션 7종)</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="8" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B83" s="8" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>디버프 시트</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="inlineStr">
+        <is>
+          <t>신규 추가 (10종, v1.7 5종 포함)</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="7" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="inlineStr">
+        <is>
+          <t>패치 노트 시트</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="inlineStr">
+        <is>
+          <t>신규 추가 (히스토리)</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="inlineStr">
+        <is>
           <t>v1.10</t>
         </is>
       </c>
-      <c r="B81" s="8" t="inlineStr">
+      <c r="B85" s="8" t="inlineStr">
         <is>
           <t>기획서</t>
         </is>
       </c>
-      <c r="C81" s="8" t="inlineStr">
+      <c r="C85" s="8" t="inlineStr">
         <is>
           <t>던전 시트</t>
         </is>
       </c>
-      <c r="D81" s="8" t="inlineStr">
+      <c r="D85" s="8" t="inlineStr">
         <is>
           <t>신규 추가 (7종 던전)</t>
         </is>
       </c>
-      <c r="E81" s="8" t="inlineStr">
+      <c r="E85" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
feat: v1.29 — game/season.js를 server.js에 통합 (4번째 모듈 통합)
시즌 패스 시스템 활성화:
- require('./game/season') (seasonPass 별칭)
- SEASON_XP_MAP: trackQuest target → 시즌 XP source 매핑
  pvp_win / kill_boss / worldboss_kill / dungeon_clear / craft_count
- trackQuest() 훅: 기존 퀘스트 추적 시 시즌 XP 자동 적립
- 티어 승급 감지 → season_tier_up 이벤트 송출
- 소켓 핸들러 3종:
  * season_status — XP/티어/구매여부/수령내역/15티어 전체 조회
  * season_buy_pass — 프리미엄 패스 구매 (1500💎)
  * season_claim — 티어 보상 수령 (free/premium 트랙)
- 보상 자동 지급: 골드/다이아/재료/칭호 인벤토리 적용
- 프리미엄 패스 구매 시 전 서버 알림

기존 PvP/보스/던전/제작 활동이 자동으로 시즌 XP에 적립되어
별도 학습 없이 즉시 동작.

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutoBattle_io_기획서.xlsx
+++ b/AutoBattle_io_기획서.xlsx
@@ -40,7 +40,7 @@
     <sheet name="월드 보스" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="연금술" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="패치 노트" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="v1.9 ~ v1.28" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="v1.9 ~ v1.29" sheetId="34" state="visible" r:id="rId34"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -13685,7 +13685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D67"/>
+  <dimension ref="A1:D71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13726,7 +13726,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -13741,14 +13741,14 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>game/event.js → server.js 통합 (3번째 모듈 통합)</t>
+          <t>game/season.js → server.js 통합 (4번째 모듈 통합)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -13758,19 +13758,19 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>축제</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>event_status 소켓 + /status 엔드포인트 노출</t>
+          <t>trackQuest 자동 XP 적립 (PvP/보스/월드보스/던전/제작)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
@@ -13780,19 +13780,19 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>축제</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>NPC 대사 30% 확률로 축제 인사 (getNpcMsg 통합)</t>
+          <t>season_status / season_buy_pass / season_claim</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -13802,19 +13802,19 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>검증</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>오늘(4/8) 봄꽃 축제 활성 동작 확인</t>
+          <t>티어 승급 시 server_msg + season_tier_up 알림</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -13829,14 +13829,14 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>game/fishing.js → server.js 통합 (소켓 핸들러 3종)</t>
+          <t>game/event.js → server.js 통합 (3번째 모듈 통합)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -13846,19 +13846,19 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>축제</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>fishing_status / fishing_cast / fishing_buy_rod 이벤트</t>
+          <t>event_status 소켓 + /status 엔드포인트 노출</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -13868,19 +13868,19 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>축제</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>지역 검증 (낚시 만/강변/산호초), 낚싯대 보유 검증, 미끼 소비</t>
+          <t>NPC 대사 30% 확률로 축제 인사 (getNpcMsg 통합)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -13890,19 +13890,19 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>검증</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>전설/신화 어종 낚시 시 전 서버 알림 + ach_fish50 추적</t>
+          <t>오늘(4/8) 봄꽃 축제 활성 동작 확인</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -13917,14 +13917,14 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>game/lottery.js → server.js 통합 (require + 소켓 핸들러 3종)</t>
+          <t>game/fishing.js → server.js 통합 (소켓 핸들러 3종)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -13934,19 +13934,19 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>룰렛</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>lottery_status / lottery_free_spin / lottery_paid_spin 이벤트 추가</t>
+          <t>fishing_status / fishing_cast / fishing_buy_rod 이벤트</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -13956,19 +13956,19 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>룰렛</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>전설/영웅 보상 획득 시 전 서버 알림 + ach_lucky 업적 추적</t>
+          <t>지역 검증 (낚시 만/강변/산호초), 낚싯대 보유 검증, 미끼 소비</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -13978,19 +13978,19 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>입찰식 경매 시스템 (game/auction.js 신규 모듈)</t>
+          <t>전설/신화 어종 낚시 시 전 서버 알림 + ach_fish50 추적</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
@@ -14000,19 +14000,19 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>3가지 기간(1h/6h/24h) + 등록2% + 낙찰5% + 스나이핑 방지</t>
+          <t>game/lottery.js → server.js 통합 (require + 소켓 핸들러 3종)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
@@ -14022,19 +14022,19 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>룰렛</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>경매장 시트 신규 추가</t>
+          <t>lottery_status / lottery_free_spin / lottery_paid_spin 이벤트 추가</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -14044,19 +14044,19 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>룰렛</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>11종 어종 + 5등급 낚싯대 + 4종 미끼 (game/fishing.js 신규 모듈)</t>
+          <t>전설/영웅 보상 획득 시 전 서버 알림 + ach_lucky 업적 추적</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
@@ -14066,19 +14066,19 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>신화 크라켄 (밤+낚시터+드래곤대 한정), 바다의 군주 칭호 연계</t>
+          <t>입찰식 경매 시스템 (game/auction.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -14088,19 +14088,19 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>낚시 시트 신규 추가</t>
+          <t>3가지 기간(1h/6h/24h) + 등록2% + 낙찰5% + 스나이핑 방지</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
@@ -14110,19 +14110,19 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>20웨이브 엔드리스 보스 러시 모드 (game/boss_rush.js 신규 모듈)</t>
+          <t>경매장 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -14132,19 +14132,19 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>매일 무료 3회 + 랭킹 1위 챔피언 칭호</t>
+          <t>11종 어종 + 5등급 낚싯대 + 4종 미끼 (game/fishing.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
@@ -14154,19 +14154,19 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>보스 러시 시트 신규 추가</t>
+          <t>신화 크라켄 (밤+낚시터+드래곤대 한정), 바다의 군주 칭호 연계</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -14176,19 +14176,19 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>행운의 룰렛</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>10종 보상 + 가중치 시스템 (game/lottery.js 신규 모듈)</t>
+          <t>낚시 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
@@ -14198,19 +14198,19 @@
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>룰렛</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>매일 무료 1회 / 유료 50💎 / 10연속 450💎 (10% 할인)</t>
+          <t>20웨이브 엔드리스 보스 러시 모드 (game/boss_rush.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -14220,19 +14220,19 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>행운의 룰렛 시트 신규 추가</t>
+          <t>매일 무료 3회 + 랭킹 1위 챔피언 칭호</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
@@ -14242,19 +14242,19 @@
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>5종 시즌 축제 추가 (신년/봄꽃/한여름/할로윈/겨울)</t>
+          <t>보스 러시 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -14264,19 +14264,19 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>모듈화</t>
+          <t>행운의 룰렛</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>game/event.js 신규 파일 (실제 달력 기반 자동 활성화)</t>
+          <t>10종 보상 + 가중치 시스템 (game/lottery.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
@@ -14286,19 +14286,19 @@
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>룰렛</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트 시트 신규 추가</t>
+          <t>매일 무료 1회 / 유료 50💎 / 10연속 450💎 (10% 할인)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -14308,19 +14308,19 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>15티어 배틀 패스 시스템 추가 (game/season.js 신규 모듈)</t>
+          <t>행운의 룰렛 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
@@ -14330,19 +14330,19 @@
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>30일 사이클, 무료+프리미엄(1500💎) 트랙</t>
+          <t>5종 시즌 축제 추가 (신년/봄꽃/한여름/할로윈/겨울)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -14352,19 +14352,19 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>모듈화</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>시즌 패스 시트 신규 추가</t>
+          <t>game/event.js 신규 파일 (실제 달력 기반 자동 활성화)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
@@ -14374,19 +14374,19 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>마일스톤 5종 추가 (Lv.40/50, 첫 환생, 첫 월드 보스, 업적 50)</t>
+          <t>축제 이벤트 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -14396,19 +14396,19 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>무료 다이아 시트 신규 추가</t>
+          <t>15티어 배틀 패스 시스템 추가 (game/season.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
@@ -14418,19 +14418,19 @@
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>상점</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>프리미엄 5종 추가 (불사조/폭풍 스킨, 자동물약 24h, 보물상자, 재료 패키지)</t>
+          <t>30일 사이클, 무료+프리미엄(1500💎) 트랙</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -14445,14 +14445,14 @@
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>상점 시트 갱신</t>
+          <t>시즌 패스 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
@@ -14462,19 +14462,19 @@
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>혈맹</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>혈맹 Lv.6-10 + 신규 스킬 5종 (분노/신속/회복/운명/전설)</t>
+          <t>마일스톤 5종 추가 (Lv.40/50, 첫 환생, 첫 월드 보스, 업적 50)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -14484,19 +14484,19 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>혈맹</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>최대 인원 50→100명 (Lv.10 기준)</t>
+          <t>무료 다이아 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
@@ -14506,19 +14506,19 @@
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>상점</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>길드(혈맹) 시트 신규 추가</t>
+          <t>프리미엄 5종 추가 (불사조/폭풍 스킨, 자동물약 24h, 보물상자, 재료 패키지)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -14528,19 +14528,19 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>점쟁이/감정사/수집가 3종 추가 (운세/감정/희귀품 매입)</t>
+          <t>상점 시트 갱신</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
@@ -14550,19 +14550,19 @@
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>대사 시스템</t>
+          <t>혈맹</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>신규 NPC 상황별 대사 (밤/카르마/레벨/골드 연동)</t>
+          <t>혈맹 Lv.6-10 + 신규 스킬 5종 (분노/신속/회복/운명/전설)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -14572,19 +14572,19 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>혈맹</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>NPC 시트 신규 추가 (11종)</t>
+          <t>최대 인원 50→100명 (Lv.10 기준)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
@@ -14594,19 +14594,19 @@
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>각성기</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>클래스별 Lv.40 각성기 5종 추가 (천개의칼날/대지가르기/불멸의수호자/시간정지/신의은총)</t>
+          <t>길드(혈맹) 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -14616,19 +14616,19 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>스킬 시트 전면 갱신 (12종→30종, 클레릭 포함)</t>
+          <t>점쟁이/감정사/수집가 3종 추가 (운세/감정/희귀품 매입)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
@@ -14638,19 +14638,19 @@
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>대사 시스템</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>v1.9~v1.13 컨텐츠 연계 업적 5종 추가 (폭풍 정복자/연금술사/그림자/전설 동반자/이국 상인)</t>
+          <t>신규 NPC 상황별 대사 (밤/카르마/레벨/골드 연동)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -14665,14 +14665,14 @@
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>퀘스트 시트 전면 갱신 (9종→64종 반영)</t>
+          <t>NPC 시트 신규 추가 (11종)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
@@ -14682,19 +14682,19 @@
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>월드 보스</t>
+          <t>각성기</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>폭풍의 거인 / 시간의 수호자 2종 추가 (최대 HP / 최강 ATK)</t>
+          <t>클래스별 Lv.40 각성기 5종 추가 (천개의칼날/대지가르기/불멸의수호자/시간정지/신의은총)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -14704,19 +14704,19 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>교역</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>이국의 사치품 3종 추가 (불사조 깃털/공허의 정수/천공의 비단)</t>
+          <t>스킬 시트 전면 갱신 (12종→30종, 클레릭 포함)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
@@ -14726,19 +14726,19 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>월드 보스 시트 신규 추가, 교역 시트 갱신</t>
+          <t>v1.9~v1.13 컨텐츠 연계 업적 5종 추가 (폭풍 정복자/연금술사/그림자/전설 동반자/이국 상인)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -14748,19 +14748,19 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>엘릭서 5종 추가 (타이탄/강철/질풍/지혜/행운, 15~30분 강력 버프)</t>
+          <t>퀘스트 시트 전면 갱신 (9종→64종 반영)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
@@ -14770,19 +14770,19 @@
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>월드 보스</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>연금술 시트 신규 추가</t>
+          <t>폭풍의 거인 / 시간의 수호자 2종 추가 (최대 HP / 최강 ATK)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -14792,19 +14792,19 @@
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>신규 펫</t>
+          <t>교역</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>불사조 (화염 +20%) / 유니콘 (회피 +10%) + 진화형</t>
+          <t>이국의 사치품 3종 추가 (불사조 깃털/공허의 정수/천공의 비단)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
@@ -14814,19 +14814,19 @@
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>신규 탈것</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>페가수스 (이동 +85%, 비행)</t>
+          <t>월드 보스 시트 신규 추가, 교역 시트 갱신</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -14836,19 +14836,19 @@
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>신규 던전</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>그림자 미궁 (Lv.38, 8인 파티, 7스테이지, 전설 드롭)</t>
+          <t>엘릭서 5종 추가 (타이탄/강철/질풍/지혜/행운, 15~30분 강력 버프)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
@@ -14863,14 +14863,14 @@
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>던전 시트 신규 추가 (7종 던전 정리)</t>
+          <t>연금술 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -14880,19 +14880,19 @@
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 펫</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>공허의 방랑자/불멸자/천공의 군주 3종 추가 (엔드게임)</t>
+          <t>불사조 (화염 +20%) / 유니콘 (회피 +10%) + 진화형</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
@@ -14902,107 +14902,107 @@
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>신규 탈것</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>51개 지역, 16종 칭호, 출석/세트/등급 시트 추가</t>
+          <t>페가수스 (이동 +85%, 비행)</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>신규 던전</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>패치 노트 갱신, 낮/밤 시계 + 진행 시간 표시</t>
+          <t>그림자 미궁 (Lv.38, 8인 파티, 7스테이지, 전설 드롭)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>자동화</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D59" s="8" t="inlineStr">
         <is>
-          <t>자동 스킬 시전 (인간 플레이어용), 자동 스킬 토글 버튼</t>
+          <t>던전 시트 신규 추가 (7종 던전 정리)</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>미니맵 친구 위치 표시, 보스 표시 강화, DPS 미터 스파크라인</t>
+          <t>공허의 방랑자/불멸자/천공의 군주 3종 추가 (엔드게임)</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>시스템</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>혈맹 창고 UI 패널, 보스 신규 디버프 적용</t>
+          <t>51개 지역, 16종 칭호, 출석/세트/등급 시트 추가</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -15012,19 +15012,19 @@
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>상태이상</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>신규 디버프 5종 (빙결/감전/출혈/약화/공포)</t>
+          <t>패치 노트 갱신, 낮/밤 시계 + 진행 시간 표시</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
@@ -15034,19 +15034,19 @@
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>자동화</t>
         </is>
       </c>
       <c r="D63" s="8" t="inlineStr">
         <is>
-          <t>포션 단축키 (1/2/3/4), 레벨별 추천 활동 가이드</t>
+          <t>자동 스킬 시전 (인간 플레이어용), 자동 스킬 토글 버튼</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
@@ -15056,19 +15056,19 @@
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>시스템</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>장비 자동 최적화 (auto_equip_best), 알림 센터</t>
+          <t>미니맵 친구 위치 표시, 보스 표시 강화, DPS 미터 스파크라인</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
@@ -15078,12 +15078,12 @@
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>컨텐츠</t>
+          <t>시스템</t>
         </is>
       </c>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>신규 업적 10종 (30→40), 신규 몬스터 존 3개</t>
+          <t>혈맹 창고 UI 패널, 보스 신규 디버프 적용</t>
         </is>
       </c>
     </row>
@@ -15100,32 +15100,120 @@
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>상태이상</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>인벤토리 검색 + 정렬, PvP 시즌 보드 시각화</t>
+          <t>신규 디버프 5종 (빙결/감전/출혈/약화/공포)</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B67" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>포션 단축키 (1/2/3/4), 레벨별 추천 활동 가이드</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>시스템</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>장비 자동 최적화 (auto_equip_best), 알림 센터</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="inlineStr">
+        <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B69" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>컨텐츠</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="inlineStr">
+        <is>
+          <t>신규 업적 10종 (30→40), 신규 몬스터 존 3개</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="7" t="inlineStr">
+        <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>인벤토리 검색 + 정렬, PvP 시즌 보드 시각화</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
+        <is>
           <t>v1.6 이전</t>
         </is>
       </c>
-      <c r="B67" s="8" t="inlineStr">
+      <c r="B71" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C67" s="8" t="inlineStr">
+      <c r="C71" s="8" t="inlineStr">
         <is>
           <t>기반</t>
         </is>
       </c>
-      <c r="D67" s="8" t="inlineStr">
+      <c r="D71" s="8" t="inlineStr">
         <is>
           <t>마을/사냥/PvP/카르마/펫/탈것/제작/교역/길드/공성/투기장 등</t>
         </is>
@@ -15145,7 +15233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E85"/>
+  <dimension ref="A1:E90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -15192,7 +15280,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -15202,159 +15290,159 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>event → server.js</t>
+          <t>season → server.js</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>3번째 모듈 통합</t>
+          <t>4번째 모듈 통합</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>축제 시스템 활성화</t>
+          <t>XP 자동 적립 + 보상 수령</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>소켓</t>
+          <t>자동화</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>event_status</t>
+          <t>trackQuest 훅</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>현재 활성 축제 조회</t>
+          <t>PvP/보스/월드보스/던전/제작 → 시즌 XP</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>이름/기간/버프/한정 보상</t>
+          <t>SEASON_XP_MAP 매핑</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>/status JSON</t>
+          <t>season_status</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>festival 필드 추가</t>
+          <t>XP/티어/구매여부/수령내역 조회</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>대시보드 확인용</t>
+          <t>15티어 전체</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>NPC</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>축제 인사</t>
+          <t>season_buy_pass</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>30% 확률로 NPC가 축제 대사 출력</t>
+          <t>프리미엄 패스 구매 (1500💎)</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>spring_blossom 등 5종</t>
+          <t>전 서버 알림</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>통합</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>fishing → server.js</t>
+          <t>season_claim</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>require + 소켓 핸들러 3종</t>
+          <t>티어 보상 수령 (free/premium)</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>두 번째 모듈 통합</t>
+          <t>자동 인벤토리 적용</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>소켓</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>fishing_status</t>
+          <t>event → server.js</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>지역/낚싯대/미끼/시간대 조회</t>
+          <t>3번째 모듈 통합</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>클라이언트 표시용</t>
+          <t>축제 시스템 활성화</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -15364,1880 +15452,1880 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>fishing_cast</t>
+          <t>event_status</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>낚시 시도 (지역+낚싯대+미끼 검증)</t>
+          <t>현재 활성 축제 조회</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>전설/신화 → 서버 알림</t>
+          <t>이름/기간/버프/한정 보상</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>소켓</t>
+          <t>API</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>fishing_buy_rod</t>
+          <t>/status JSON</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>낚싯대 구매 (골드/다이아)</t>
+          <t>festival 필드 추가</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>5등급 모두</t>
+          <t>대시보드 확인용</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>통합</t>
+          <t>NPC</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>lottery → server.js</t>
+          <t>축제 인사</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>require + 소켓 핸들러 3종</t>
+          <t>30% 확률로 NPC가 축제 대사 출력</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>첫 모듈 통합 마일스톤</t>
+          <t>spring_blossom 등 5종</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>소켓 이벤트</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>lottery_status</t>
+          <t>fishing → server.js</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>상태/가격/상품 풀 조회</t>
+          <t>require + 소켓 핸들러 3종</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>클라이언트 표시용</t>
+          <t>두 번째 모듈 통합</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>소켓 이벤트</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>lottery_free_spin</t>
+          <t>fishing_status</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>매일 무료 1회 스핀</t>
+          <t>지역/낚싯대/미끼/시간대 조회</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>자정 초기화</t>
+          <t>클라이언트 표시용</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>소켓 이벤트</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>lottery_paid_spin</t>
+          <t>fishing_cast</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>유료 1회 / 10연속</t>
+          <t>낚시 시도 (지역+낚싯대+미끼 검증)</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>count: 1 또는 10</t>
+          <t>전설/신화 → 서버 알림</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>game/auction.js 신규</t>
+          <t>fishing_buy_rod</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>입찰식 / 3기간 / 5% 인상 / 스나이핑 방지</t>
+          <t>낚싯대 구매 (골드/다이아)</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>등록 2% + 낙찰 5%</t>
+          <t>5등급 모두</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>활성 한도</t>
+          <t>lottery → server.js</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>플레이어당 10개</t>
+          <t>require + 소켓 핸들러 3종</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>자기 입찰 금지</t>
+          <t>첫 모듈 통합 마일스톤</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>소켓 이벤트</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>game/fishing.js 신규</t>
+          <t>lottery_status</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>11종 어종 / 5등급 낚싯대 / 4종 미끼</t>
+          <t>상태/가격/상품 풀 조회</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>신화 크라켄 = 20000G + 칭호</t>
+          <t>클라이언트 표시용</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>소켓 이벤트</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>전설의 비단잉어</t>
+          <t>lottery_free_spin</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>드래곤 낚싯대 + 가중치 1</t>
+          <t>매일 무료 1회 스핀</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>5000G + 평생 행운 +5%</t>
+          <t>자정 초기화</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>소켓 이벤트</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>game/boss_rush.js 신규</t>
+          <t>lottery_paid_spin</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>20웨이브 / HP ×1.35 스케일링</t>
+          <t>유료 1회 / 10연속</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>최종 보상: 200💎 + 용재료 ×5</t>
+          <t>count: 1 또는 10</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>입장</t>
+          <t>game/auction.js 신규</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>매일 무료 3회 / 1000G / 30💎</t>
+          <t>입찰식 / 3기간 / 5% 인상 / 스나이핑 방지</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>랭킹 시스템</t>
+          <t>등록 2% + 낙찰 5%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>챔피언 보상</t>
+          <t>활성 한도</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>1위: 500💎 + 칭호 / 2위: 300💎 / 3위: 200💎</t>
+          <t>플레이어당 10개</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>자기 입찰 금지</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>행운의 룰렛</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>game/lottery.js 신규</t>
+          <t>game/fishing.js 신규</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>10종 보상 / 가중치 1000</t>
+          <t>11종 어종 / 5등급 낚싯대 / 4종 미끼</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>매일 무료 1회 + 유료</t>
+          <t>신화 크라켄 = 20000G + 칭호</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>룰렛 (전설)</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>영웅 장비 상자</t>
+          <t>전설의 비단잉어</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>확률 0.2% (가장 희귀)</t>
+          <t>드래곤 낚싯대 + 가중치 1</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>전설 보상</t>
+          <t>5000G + 평생 행운 +5%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>룰렛 (전설)</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>200 다이아</t>
+          <t>game/boss_rush.js 신규</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>확률 0.8%</t>
+          <t>20웨이브 / HP ×1.35 스케일링</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>잭팟</t>
+          <t>최종 보상: 200💎 + 용재료 ×5</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>신년 축제</t>
+          <t>입장</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>1/1 ~ 1/7</t>
+          <t>매일 무료 3회 / 1000G / 30💎</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>골드 +50% / EXP +30%</t>
+          <t>랭킹 시스템</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>봄꽃 축제</t>
+          <t>챔피언 보상</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>4/1 ~ 4/14</t>
+          <t>1위: 500💎 + 칭호 / 2위: 300💎 / 3위: 200💎</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>HP재생 +30% / 드롭 +20%</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>행운의 룰렛</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>한여름 밤의 축제</t>
+          <t>game/lottery.js 신규</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>7/15 ~ 8/15</t>
+          <t>10종 보상 / 가중치 1000</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>화염 +30% / PvP 보상 +50%</t>
+          <t>매일 무료 1회 + 유료</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>룰렛 (전설)</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>할로윈 축제</t>
+          <t>영웅 장비 상자</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>10/25 ~ 11/1</t>
+          <t>확률 0.2% (가장 희귀)</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>크리 +10% / 언데드 +50%</t>
+          <t>전설 보상</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>룰렛 (전설)</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>겨울 축제</t>
+          <t>200 다이아</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>12/20 ~ 12/31</t>
+          <t>확률 0.8%</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>골드 +30% / EXP +30% / 드롭 +30%</t>
+          <t>잭팟</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>game/season.js 신규</t>
+          <t>신년 축제</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>15티어 / 30일 / 무료+프리미엄</t>
+          <t>1/1 ~ 1/7</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>만렙 보상: 태초 반지 + 시즌 칭호</t>
+          <t>골드 +50% / EXP +30%</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>XP 획득 7종</t>
+          <t>봄꽃 축제</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>퀘/보스/PvP/월드보스/던전/제작</t>
+          <t>4/1 ~ 4/14</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>일일 +200 ~ 월드보스 +500</t>
+          <t>HP재생 +30% / 드롭 +20%</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>프리미엄 가격</t>
+          <t>한여름 밤의 축제</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>1500 다이아</t>
+          <t>7/15 ~ 8/15</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>시즌 당 1회</t>
+          <t>화염 +30% / PvP 보상 +50%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Lv.40 달성</t>
+          <t>할로윈 축제</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>각성기 해금 마일스톤</t>
+          <t>10/25 ~ 11/1</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>150💎</t>
+          <t>크리 +10% / 언데드 +50%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Lv.50 달성</t>
+          <t>겨울 축제</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>환생 가능 마일스톤</t>
+          <t>12/20 ~ 12/31</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>250💎</t>
+          <t>골드 +30% / EXP +30% / 드롭 +30%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>첫 환생</t>
+          <t>game/season.js 신규</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>prestige 1차</t>
+          <t>15티어 / 30일 / 무료+프리미엄</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>500💎</t>
+          <t>만렙 보상: 태초 반지 + 시즌 칭호</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>첫 월드 보스</t>
+          <t>XP 획득 7종</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>월드 보스 처치 보너스</t>
+          <t>퀘/보스/PvP/월드보스/던전/제작</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>100💎</t>
+          <t>일일 +200 ~ 월드보스 +500</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>업적 50개</t>
+          <t>프리미엄 가격</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>업적 마일스톤</t>
+          <t>1500 다이아</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>200💎</t>
+          <t>시즌 당 1회</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>상점 (스킨)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>불사조 스킨</t>
+          <t>Lv.40 달성</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>1200 다이아</t>
+          <t>각성기 해금 마일스톤</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>불사조 깃털 이펙트 (영구)</t>
+          <t>150💎</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>상점 (스킨)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>폭풍 스킨</t>
+          <t>Lv.50 달성</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>1200 다이아</t>
+          <t>환생 가능 마일스톤</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>번개 오라 이펙트 (영구)</t>
+          <t>250💎</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>상점 (편의)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>프리미엄 자동물약</t>
+          <t>첫 환생</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>500 다이아</t>
+          <t>prestige 1차</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>24시간 자동물약 무한</t>
+          <t>500💎</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>상점 (상자)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>프리미엄 보물 상자</t>
+          <t>첫 월드 보스</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>300 다이아</t>
+          <t>월드 보스 처치 보너스</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>전설 장비 확정 + 다이아</t>
+          <t>100💎</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>상점 (재료)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>전설 재료 패키지</t>
+          <t>업적 50개</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>600 다이아</t>
+          <t>업적 마일스톤</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>용재료×10 + 영혼석×20 + 마법재료×20</t>
+          <t>200💎</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>혈맹 Lv.6</t>
+          <t>상점 (스킨)</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>혈맹의 분노</t>
+          <t>불사조 스킨</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>크리티컬 +5%</t>
+          <t>1200 다이아</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>60명 정원</t>
+          <t>불사조 깃털 이펙트 (영구)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>혈맹 Lv.7</t>
+          <t>상점 (스킨)</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>혈맹의 신속</t>
+          <t>폭풍 스킨</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>이동속도 +10%</t>
+          <t>1200 다이아</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>70명 정원</t>
+          <t>번개 오라 이펙트 (영구)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>혈맹 Lv.8</t>
+          <t>상점 (편의)</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>혈맹의 회복</t>
+          <t>프리미엄 자동물약</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>HP 재생 +50%</t>
+          <t>500 다이아</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>80명 정원</t>
+          <t>24시간 자동물약 무한</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>혈맹 Lv.9</t>
+          <t>상점 (상자)</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>혈맹의 운명</t>
+          <t>프리미엄 보물 상자</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>회피 +5%</t>
+          <t>300 다이아</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>90명 정원</t>
+          <t>전설 장비 확정 + 다이아</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>혈맹 Lv.10</t>
+          <t>상점 (재료)</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>혈맹의 전설</t>
+          <t>전설 재료 패키지</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>전 스탯 +5%</t>
+          <t>600 다이아</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>100명 정원 — 최종</t>
+          <t>용재료×10 + 영혼석×20 + 마법재료×20</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>혈맹 Lv.6</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>점쟁이</t>
+          <t>혈맹의 분노</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>운세 / 행운 버프 (밤·카르마 반응)</t>
+          <t>크리티컬 +5%</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>상황 대사 4종</t>
+          <t>60명 정원</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>혈맹 Lv.7</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>감정사</t>
+          <t>혈맹의 신속</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>미감정 장비 감정 (Lv.30+ 특수)</t>
+          <t>이동속도 +10%</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>상황 대사 4종</t>
+          <t>70명 정원</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>혈맹 Lv.8</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>수집가</t>
+          <t>혈맹의 회복</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>희귀 아이템 매입 (골드 50000+ 특별)</t>
+          <t>HP 재생 +50%</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t>상황 대사 4종</t>
+          <t>80명 정원</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>각성기 (어쌔신)</t>
+          <t>혈맹 Lv.9</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>천 개의 칼날</t>
+          <t>혈맹의 운명</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>3.5배 × 7타 / 광역 / 쿨150초</t>
+          <t>회피 +5%</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>90명 정원</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>각성기 (워리어)</t>
+          <t>혈맹 Lv.10</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>대지 가르기</t>
+          <t>혈맹의 전설</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>6.0배 / 광역 5범위 / 스턴 2초</t>
+          <t>전 스탯 +5%</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>100명 정원 — 최종</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>각성기 (나이트)</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>불멸의 수호자</t>
+          <t>점쟁이</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>피해 90% 감소 / 도발 / 10초</t>
+          <t>운세 / 행운 버프 (밤·카르마 반응)</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>상황 대사 4종</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>각성기 (메이지)</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>시간 정지</t>
+          <t>감정사</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>12.0배 / 광역 6범위 / 슬로우 90%</t>
+          <t>미감정 장비 감정 (Lv.30+ 특수)</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>상황 대사 4종</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>각성기 (클레릭)</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>신의 은총</t>
+          <t>수집가</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>HP 100% 회복 / 전스탯 +50%</t>
+          <t>희귀 아이템 매입 (골드 50000+ 특별)</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>상황 대사 4종</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (어쌔신)</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>폭풍 정복자</t>
+          <t>천 개의 칼날</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>폭풍의 거인 처치</t>
+          <t>3.5배 × 7타 / 광역 / 쿨150초</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t>10,000G + 150다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (워리어)</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>연금술사</t>
+          <t>대지 가르기</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>엘릭서 10회 제작</t>
+          <t>6.0배 / 광역 5범위 / 스턴 2초</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>5,000G + 80다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (나이트)</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>그림자 정복자</t>
+          <t>불멸의 수호자</t>
         </is>
       </c>
       <c r="D59" s="8" t="inlineStr">
         <is>
-          <t>그림자 미궁 클리어</t>
+          <t>피해 90% 감소 / 도발 / 10초</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t>8,000G + 120다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (메이지)</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>전설의 동반자</t>
+          <t>시간 정지</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>전설급 펫 진화</t>
+          <t>12.0배 / 광역 6범위 / 슬로우 90%</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>6,000G + 100다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (클레릭)</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>이국의 상인</t>
+          <t>신의 은총</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>사치품 교역 5회</t>
+          <t>HP 100% 회복 / 전스탯 +50%</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t>4,000G + 60다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>월드 보스</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>폭풍의 거인</t>
+          <t>폭풍 정복자</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>HP 100,000 / ATK 140 / DEF 90</t>
+          <t>폭풍의 거인 처치</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>EXP 10000 + 6000G</t>
+          <t>10,000G + 150다이아</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>월드 보스</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>시간의 수호자</t>
+          <t>연금술사</t>
         </is>
       </c>
       <c r="D63" s="8" t="inlineStr">
         <is>
-          <t>HP 70,000 / ATK 170 / DEF 60</t>
+          <t>엘릭서 10회 제작</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t>EXP 9000 + 7000G</t>
+          <t>5,000G + 80다이아</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>교역품</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>불사조 깃털 / 공허의 정수 / 천공의 비단</t>
+          <t>그림자 정복자</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>이국의 사치품 3종</t>
+          <t>그림자 미궁 클리어</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>기본가 600~900G</t>
+          <t>8,000G + 120다이아</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>타이탄의 엘릭서</t>
+          <t>전설의 동반자</t>
         </is>
       </c>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>용재료×3 + 마법재료×10</t>
+          <t>전설급 펫 진화</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>ATK ×1.5 / 30분</t>
+          <t>6,000G + 100다이아</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>강철 엘릭서</t>
+          <t>이국의 상인</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>철광석×30 + 마법재료×10</t>
+          <t>사치품 교역 5회</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>DEF ×1.5 / 30분</t>
+          <t>4,000G + 60다이아</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>월드 보스</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>질풍 엘릭서</t>
+          <t>폭풍의 거인</t>
         </is>
       </c>
       <c r="D67" s="8" t="inlineStr">
         <is>
-          <t>약초×20 + 마법재료×8</t>
+          <t>HP 100,000 / ATK 140 / DEF 90</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t>SPD ×1.4 / 20분</t>
+          <t>EXP 10000 + 6000G</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>월드 보스</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>지혜 엘릭서</t>
+          <t>시간의 수호자</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>마법수정×5 + 영혼재료×5</t>
+          <t>HP 70,000 / ATK 170 / DEF 60</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>EXP ×2.5 / 15분</t>
+          <t>EXP 9000 + 7000G</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>교역품</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>행운 엘릭서</t>
+          <t>불사조 깃털 / 공허의 정수 / 천공의 비단</t>
         </is>
       </c>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>보석×10 + 마법재료×5</t>
+          <t>이국의 사치품 3종</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>GOLD ×2.0 / 15분</t>
+          <t>기본가 600~900G</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>신규 펫</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>불사조 (pet_phoenix)</t>
+          <t>타이탄의 엘릭서</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>불꽃산 보스 50처치</t>
+          <t>용재료×3 + 마법재료×10</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>화염 DMG +20% (진화 +40%)</t>
+          <t>ATK ×1.5 / 30분</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>신규 펫</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>유니콘 (pet_unicorn)</t>
+          <t>강철 엘릭서</t>
         </is>
       </c>
       <c r="D71" s="8" t="inlineStr">
         <is>
-          <t>다이아 800개</t>
+          <t>철광석×30 + 마법재료×10</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t>회피 +10% (진화 +20%)</t>
+          <t>DEF ×1.5 / 30분</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>신규 탈것</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>페가수스 (mount_pegasus)</t>
+          <t>질풍 엘릭서</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>다이아 1200개</t>
+          <t>약초×20 + 마법재료×8</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>이동속도 +85% / 비행</t>
+          <t>SPD ×1.4 / 20분</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>신규 던전</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>그림자 미궁</t>
+          <t>지혜 엘릭서</t>
         </is>
       </c>
       <c r="D73" s="8" t="inlineStr">
         <is>
-          <t>Lv.38 / 8인 파티 / 7스테이지</t>
+          <t>마법수정×5 + 영혼재료×5</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t>22000G + 32000EXP</t>
+          <t>EXP ×2.5 / 15분</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>드롭</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>드래곤 검/망토/투구/장갑</t>
+          <t>행운 엘릭서</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>그림자 미궁 보스 드롭</t>
+          <t>보석×10 + 마법재료×5</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>전설급</t>
+          <t>GOLD ×2.0 / 15분</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 펫</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t>공허의 방랑자</t>
+          <t>불사조 (pet_phoenix)</t>
         </is>
       </c>
       <c r="D75" s="8" t="inlineStr">
         <is>
-          <t>몬스터 10,000 처치</t>
+          <t>불꽃산 보스 50처치</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
         <is>
-          <t>ATK +7%</t>
+          <t>화염 DMG +20% (진화 +40%)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 펫</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>불멸자</t>
+          <t>유니콘 (pet_unicorn)</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>환생 5회</t>
+          <t>다이아 800개</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>EXP +25%</t>
+          <t>회피 +10% (진화 +20%)</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 탈것</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t>천공의 군주</t>
+          <t>페가수스 (mount_pegasus)</t>
         </is>
       </c>
       <c r="D77" s="8" t="inlineStr">
         <is>
-          <t>월드 보스 10회 처치</t>
+          <t>다이아 1200개</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
         <is>
-          <t>보스DMG +15%</t>
+          <t>이동속도 +85% / 비행</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>신규 던전</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>지역 시트 갱신</t>
+          <t>그림자 미궁</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>25→51개 지역 반영</t>
+          <t>Lv.38 / 8인 파티 / 7스테이지</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22000G + 32000EXP</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>드롭</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>칭호 시트 갱신</t>
+          <t>드래곤 검/망토/투구/장갑</t>
         </is>
       </c>
       <c r="D79" s="8" t="inlineStr">
         <is>
-          <t>7→16종 + 효과/색상 추가</t>
+          <t>그림자 미궁 보스 드롭</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>전설급</t>
         </is>
       </c>
     </row>
@@ -17249,22 +17337,22 @@
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>출석 캘린더 시트</t>
+          <t>공허의 방랑자</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>신규 추가 (28일 사이클)</t>
+          <t>몬스터 10,000 처치</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ATK +7%</t>
         </is>
       </c>
     </row>
@@ -17276,22 +17364,22 @@
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t>장비 세트 시트</t>
+          <t>불멸자</t>
         </is>
       </c>
       <c r="D81" s="8" t="inlineStr">
         <is>
-          <t>신규 추가 (드래곤/영웅/태초)</t>
+          <t>환생 5회</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EXP +25%</t>
         </is>
       </c>
     </row>
@@ -17303,22 +17391,22 @@
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>장비 등급 시트</t>
+          <t>천공의 군주</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>신규 추가 (5등급 + 랜덤 옵션 7종)</t>
+          <t>월드 보스 10회 처치</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>보스DMG +15%</t>
         </is>
       </c>
     </row>
@@ -17335,12 +17423,12 @@
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t>디버프 시트</t>
+          <t>지역 시트 갱신</t>
         </is>
       </c>
       <c r="D83" s="8" t="inlineStr">
         <is>
-          <t>신규 추가 (10종, v1.7 5종 포함)</t>
+          <t>25→51개 지역 반영</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
@@ -17362,12 +17450,12 @@
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>패치 노트 시트</t>
+          <t>칭호 시트 갱신</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>신규 추가 (히스토리)</t>
+          <t>7→16종 + 효과/색상 추가</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
@@ -17379,25 +17467,160 @@
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>출석 캘린더 시트</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>신규 추가 (28일 사이클)</t>
+        </is>
+      </c>
+      <c r="E85" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="7" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C86" s="7" t="inlineStr">
+        <is>
+          <t>장비 세트 시트</t>
+        </is>
+      </c>
+      <c r="D86" s="7" t="inlineStr">
+        <is>
+          <t>신규 추가 (드래곤/영웅/태초)</t>
+        </is>
+      </c>
+      <c r="E86" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="8" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>장비 등급 시트</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>신규 추가 (5등급 + 랜덤 옵션 7종)</t>
+        </is>
+      </c>
+      <c r="E87" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="7" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C88" s="7" t="inlineStr">
+        <is>
+          <t>디버프 시트</t>
+        </is>
+      </c>
+      <c r="D88" s="7" t="inlineStr">
+        <is>
+          <t>신규 추가 (10종, v1.7 5종 포함)</t>
+        </is>
+      </c>
+      <c r="E88" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="8" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B89" s="8" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t>패치 노트 시트</t>
+        </is>
+      </c>
+      <c r="D89" s="8" t="inlineStr">
+        <is>
+          <t>신규 추가 (히스토리)</t>
+        </is>
+      </c>
+      <c r="E89" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="7" t="inlineStr">
+        <is>
           <t>v1.10</t>
         </is>
       </c>
-      <c r="B85" s="8" t="inlineStr">
+      <c r="B90" s="7" t="inlineStr">
         <is>
           <t>기획서</t>
         </is>
       </c>
-      <c r="C85" s="8" t="inlineStr">
+      <c r="C90" s="7" t="inlineStr">
         <is>
           <t>던전 시트</t>
         </is>
       </c>
-      <c r="D85" s="8" t="inlineStr">
+      <c r="D90" s="7" t="inlineStr">
         <is>
           <t>신규 추가 (7종 던전)</t>
         </is>
       </c>
-      <c r="E85" s="8" t="inlineStr">
+      <c r="E90" s="7" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
feat: v1.30 — game/boss_rush.js를 server.js에 통합 (5번째 모듈 통합)
보스 러시 모드 활성화:
- require('./game/boss_rush') (bossRush 별칭)
- 메모리 상태:
  * bossRushSessions — 진행 중 세션 (currentWave/시간 추적)
  * bossRushRanking — 글로벌 랭킹 TOP 100
- finishBossRush(playerId, isFullClear) 헬퍼:
  * 누적 보상 자동 지급 (gold/exp/diamonds/mats)
  * 최고 기록 갱신 (p.bossRushBestWave)
  * 랭킹 등재 (웨이브 → 시간 정렬)
  * 풀클리어 시 전 서버 알림 (rare)
  * 10웨이브+ 시 일반 알림
- 소켓 핸들러 4종:
  * boss_rush_status — 입장권/세션/랭킹/베스트 조회
  * boss_rush_enter — 무료/골드/다이아 입장 (동시 1개 제한)
  * boss_rush_advance — 클라이언트 웨이브 클리어 보고
                       (서버에서 시간 초과 검증)
  * boss_rush_abandon — 진행 포기

20웨이브 엔드리스 보스 러시가 실제로 동작 가능한 상태로 통합 완료.

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutoBattle_io_기획서.xlsx
+++ b/AutoBattle_io_기획서.xlsx
@@ -40,7 +40,7 @@
     <sheet name="월드 보스" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="연금술" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="패치 노트" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="v1.9 ~ v1.29" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="v1.9 ~ v1.30" sheetId="34" state="visible" r:id="rId34"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -13685,7 +13685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D71"/>
+  <dimension ref="A1:D75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13726,7 +13726,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>v1.29</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -13741,14 +13741,14 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>game/season.js → server.js 통합 (4번째 모듈 통합)</t>
+          <t>game/boss_rush.js → server.js 통합 (5번째 모듈 통합)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>v1.29</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -13758,19 +13758,19 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>trackQuest 자동 XP 적립 (PvP/보스/월드보스/던전/제작)</t>
+          <t>메모리 세션 + 시간 검증 + 누적 보상 + 랭킹 (TOP 100)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>v1.29</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
@@ -13785,14 +13785,14 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>season_status / season_buy_pass / season_claim</t>
+          <t>boss_rush_status / enter / advance / abandon</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>v1.29</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -13802,19 +13802,19 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>티어 승급 시 server_msg + season_tier_up 알림</t>
+          <t>풀클리어 시 전 서버 알림, 10웨이브+ 일반 알림</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -13829,14 +13829,14 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>game/event.js → server.js 통합 (3번째 모듈 통합)</t>
+          <t>game/season.js → server.js 통합 (4번째 모듈 통합)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -13846,19 +13846,19 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>축제</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>event_status 소켓 + /status 엔드포인트 노출</t>
+          <t>trackQuest 자동 XP 적립 (PvP/보스/월드보스/던전/제작)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -13868,19 +13868,19 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>축제</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>NPC 대사 30% 확률로 축제 인사 (getNpcMsg 통합)</t>
+          <t>season_status / season_buy_pass / season_claim</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -13890,19 +13890,19 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>검증</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>오늘(4/8) 봄꽃 축제 활성 동작 확인</t>
+          <t>티어 승급 시 server_msg + season_tier_up 알림</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -13917,14 +13917,14 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>game/fishing.js → server.js 통합 (소켓 핸들러 3종)</t>
+          <t>game/event.js → server.js 통합 (3번째 모듈 통합)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -13934,19 +13934,19 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>축제</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>fishing_status / fishing_cast / fishing_buy_rod 이벤트</t>
+          <t>event_status 소켓 + /status 엔드포인트 노출</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -13956,19 +13956,19 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>축제</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>지역 검증 (낚시 만/강변/산호초), 낚싯대 보유 검증, 미끼 소비</t>
+          <t>NPC 대사 30% 확률로 축제 인사 (getNpcMsg 통합)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -13978,19 +13978,19 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>검증</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>전설/신화 어종 낚시 시 전 서버 알림 + ach_fish50 추적</t>
+          <t>오늘(4/8) 봄꽃 축제 활성 동작 확인</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
@@ -14005,14 +14005,14 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>game/lottery.js → server.js 통합 (require + 소켓 핸들러 3종)</t>
+          <t>game/fishing.js → server.js 통합 (소켓 핸들러 3종)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
@@ -14022,19 +14022,19 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>룰렛</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>lottery_status / lottery_free_spin / lottery_paid_spin 이벤트 추가</t>
+          <t>fishing_status / fishing_cast / fishing_buy_rod 이벤트</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -14044,19 +14044,19 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>룰렛</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>전설/영웅 보상 획득 시 전 서버 알림 + ach_lucky 업적 추적</t>
+          <t>지역 검증 (낚시 만/강변/산호초), 낚싯대 보유 검증, 미끼 소비</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
@@ -14066,19 +14066,19 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>입찰식 경매 시스템 (game/auction.js 신규 모듈)</t>
+          <t>전설/신화 어종 낚시 시 전 서버 알림 + ach_fish50 추적</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -14088,19 +14088,19 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>3가지 기간(1h/6h/24h) + 등록2% + 낙찰5% + 스나이핑 방지</t>
+          <t>game/lottery.js → server.js 통합 (require + 소켓 핸들러 3종)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
@@ -14110,19 +14110,19 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>룰렛</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>경매장 시트 신규 추가</t>
+          <t>lottery_status / lottery_free_spin / lottery_paid_spin 이벤트 추가</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -14132,19 +14132,19 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>룰렛</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>11종 어종 + 5등급 낚싯대 + 4종 미끼 (game/fishing.js 신규 모듈)</t>
+          <t>전설/영웅 보상 획득 시 전 서버 알림 + ach_lucky 업적 추적</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
@@ -14154,19 +14154,19 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>신화 크라켄 (밤+낚시터+드래곤대 한정), 바다의 군주 칭호 연계</t>
+          <t>입찰식 경매 시스템 (game/auction.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -14176,19 +14176,19 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>낚시 시트 신규 추가</t>
+          <t>3가지 기간(1h/6h/24h) + 등록2% + 낙찰5% + 스나이핑 방지</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
@@ -14198,19 +14198,19 @@
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>20웨이브 엔드리스 보스 러시 모드 (game/boss_rush.js 신규 모듈)</t>
+          <t>경매장 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -14220,19 +14220,19 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>매일 무료 3회 + 랭킹 1위 챔피언 칭호</t>
+          <t>11종 어종 + 5등급 낚싯대 + 4종 미끼 (game/fishing.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
@@ -14242,19 +14242,19 @@
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>보스 러시 시트 신규 추가</t>
+          <t>신화 크라켄 (밤+낚시터+드래곤대 한정), 바다의 군주 칭호 연계</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -14264,19 +14264,19 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>행운의 룰렛</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>10종 보상 + 가중치 시스템 (game/lottery.js 신규 모듈)</t>
+          <t>낚시 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
@@ -14286,19 +14286,19 @@
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>룰렛</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>매일 무료 1회 / 유료 50💎 / 10연속 450💎 (10% 할인)</t>
+          <t>20웨이브 엔드리스 보스 러시 모드 (game/boss_rush.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -14308,19 +14308,19 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>행운의 룰렛 시트 신규 추가</t>
+          <t>매일 무료 3회 + 랭킹 1위 챔피언 칭호</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
@@ -14330,19 +14330,19 @@
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>5종 시즌 축제 추가 (신년/봄꽃/한여름/할로윈/겨울)</t>
+          <t>보스 러시 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -14352,19 +14352,19 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>모듈화</t>
+          <t>행운의 룰렛</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>game/event.js 신규 파일 (실제 달력 기반 자동 활성화)</t>
+          <t>10종 보상 + 가중치 시스템 (game/lottery.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
@@ -14374,19 +14374,19 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>룰렛</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트 시트 신규 추가</t>
+          <t>매일 무료 1회 / 유료 50💎 / 10연속 450💎 (10% 할인)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -14396,19 +14396,19 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>15티어 배틀 패스 시스템 추가 (game/season.js 신규 모듈)</t>
+          <t>행운의 룰렛 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
@@ -14418,19 +14418,19 @@
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>30일 사이클, 무료+프리미엄(1500💎) 트랙</t>
+          <t>5종 시즌 축제 추가 (신년/봄꽃/한여름/할로윈/겨울)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -14440,19 +14440,19 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>모듈화</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>시즌 패스 시트 신규 추가</t>
+          <t>game/event.js 신규 파일 (실제 달력 기반 자동 활성화)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
@@ -14462,19 +14462,19 @@
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>마일스톤 5종 추가 (Lv.40/50, 첫 환생, 첫 월드 보스, 업적 50)</t>
+          <t>축제 이벤트 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -14484,19 +14484,19 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>무료 다이아 시트 신규 추가</t>
+          <t>15티어 배틀 패스 시스템 추가 (game/season.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
@@ -14506,19 +14506,19 @@
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>상점</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>프리미엄 5종 추가 (불사조/폭풍 스킨, 자동물약 24h, 보물상자, 재료 패키지)</t>
+          <t>30일 사이클, 무료+프리미엄(1500💎) 트랙</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -14533,14 +14533,14 @@
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>상점 시트 갱신</t>
+          <t>시즌 패스 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
@@ -14550,19 +14550,19 @@
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>혈맹</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>혈맹 Lv.6-10 + 신규 스킬 5종 (분노/신속/회복/운명/전설)</t>
+          <t>마일스톤 5종 추가 (Lv.40/50, 첫 환생, 첫 월드 보스, 업적 50)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -14572,19 +14572,19 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>혈맹</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>최대 인원 50→100명 (Lv.10 기준)</t>
+          <t>무료 다이아 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
@@ -14594,19 +14594,19 @@
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>상점</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>길드(혈맹) 시트 신규 추가</t>
+          <t>프리미엄 5종 추가 (불사조/폭풍 스킨, 자동물약 24h, 보물상자, 재료 패키지)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -14616,19 +14616,19 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>점쟁이/감정사/수집가 3종 추가 (운세/감정/희귀품 매입)</t>
+          <t>상점 시트 갱신</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
@@ -14638,19 +14638,19 @@
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>대사 시스템</t>
+          <t>혈맹</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>신규 NPC 상황별 대사 (밤/카르마/레벨/골드 연동)</t>
+          <t>혈맹 Lv.6-10 + 신규 스킬 5종 (분노/신속/회복/운명/전설)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -14660,19 +14660,19 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>혈맹</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>NPC 시트 신규 추가 (11종)</t>
+          <t>최대 인원 50→100명 (Lv.10 기준)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
@@ -14682,19 +14682,19 @@
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>각성기</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>클래스별 Lv.40 각성기 5종 추가 (천개의칼날/대지가르기/불멸의수호자/시간정지/신의은총)</t>
+          <t>길드(혈맹) 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -14704,19 +14704,19 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>스킬 시트 전면 갱신 (12종→30종, 클레릭 포함)</t>
+          <t>점쟁이/감정사/수집가 3종 추가 (운세/감정/희귀품 매입)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
@@ -14726,19 +14726,19 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>대사 시스템</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>v1.9~v1.13 컨텐츠 연계 업적 5종 추가 (폭풍 정복자/연금술사/그림자/전설 동반자/이국 상인)</t>
+          <t>신규 NPC 상황별 대사 (밤/카르마/레벨/골드 연동)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -14753,14 +14753,14 @@
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>퀘스트 시트 전면 갱신 (9종→64종 반영)</t>
+          <t>NPC 시트 신규 추가 (11종)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
@@ -14770,19 +14770,19 @@
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>월드 보스</t>
+          <t>각성기</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>폭풍의 거인 / 시간의 수호자 2종 추가 (최대 HP / 최강 ATK)</t>
+          <t>클래스별 Lv.40 각성기 5종 추가 (천개의칼날/대지가르기/불멸의수호자/시간정지/신의은총)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -14792,19 +14792,19 @@
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>교역</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>이국의 사치품 3종 추가 (불사조 깃털/공허의 정수/천공의 비단)</t>
+          <t>스킬 시트 전면 갱신 (12종→30종, 클레릭 포함)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
@@ -14814,19 +14814,19 @@
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>월드 보스 시트 신규 추가, 교역 시트 갱신</t>
+          <t>v1.9~v1.13 컨텐츠 연계 업적 5종 추가 (폭풍 정복자/연금술사/그림자/전설 동반자/이국 상인)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -14836,19 +14836,19 @@
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>엘릭서 5종 추가 (타이탄/강철/질풍/지혜/행운, 15~30분 강력 버프)</t>
+          <t>퀘스트 시트 전면 갱신 (9종→64종 반영)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
@@ -14858,19 +14858,19 @@
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>월드 보스</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>연금술 시트 신규 추가</t>
+          <t>폭풍의 거인 / 시간의 수호자 2종 추가 (최대 HP / 최강 ATK)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -14880,19 +14880,19 @@
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>신규 펫</t>
+          <t>교역</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>불사조 (화염 +20%) / 유니콘 (회피 +10%) + 진화형</t>
+          <t>이국의 사치품 3종 추가 (불사조 깃털/공허의 정수/천공의 비단)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
@@ -14902,19 +14902,19 @@
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>신규 탈것</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>페가수스 (이동 +85%, 비행)</t>
+          <t>월드 보스 시트 신규 추가, 교역 시트 갱신</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -14924,19 +14924,19 @@
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>신규 던전</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>그림자 미궁 (Lv.38, 8인 파티, 7스테이지, 전설 드롭)</t>
+          <t>엘릭서 5종 추가 (타이탄/강철/질풍/지혜/행운, 15~30분 강력 버프)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
@@ -14951,14 +14951,14 @@
       </c>
       <c r="D59" s="8" t="inlineStr">
         <is>
-          <t>던전 시트 신규 추가 (7종 던전 정리)</t>
+          <t>연금술 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -14968,19 +14968,19 @@
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 펫</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>공허의 방랑자/불멸자/천공의 군주 3종 추가 (엔드게임)</t>
+          <t>불사조 (화염 +20%) / 유니콘 (회피 +10%) + 진화형</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
@@ -14990,107 +14990,107 @@
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>신규 탈것</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>51개 지역, 16종 칭호, 출석/세트/등급 시트 추가</t>
+          <t>페가수스 (이동 +85%, 비행)</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>신규 던전</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>패치 노트 갱신, 낮/밤 시계 + 진행 시간 표시</t>
+          <t>그림자 미궁 (Lv.38, 8인 파티, 7스테이지, 전설 드롭)</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>자동화</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D63" s="8" t="inlineStr">
         <is>
-          <t>자동 스킬 시전 (인간 플레이어용), 자동 스킬 토글 버튼</t>
+          <t>던전 시트 신규 추가 (7종 던전 정리)</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>미니맵 친구 위치 표시, 보스 표시 강화, DPS 미터 스파크라인</t>
+          <t>공허의 방랑자/불멸자/천공의 군주 3종 추가 (엔드게임)</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>시스템</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>혈맹 창고 UI 패널, 보스 신규 디버프 적용</t>
+          <t>51개 지역, 16종 칭호, 출석/세트/등급 시트 추가</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -15100,19 +15100,19 @@
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>상태이상</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>신규 디버프 5종 (빙결/감전/출혈/약화/공포)</t>
+          <t>패치 노트 갱신, 낮/밤 시계 + 진행 시간 표시</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
@@ -15122,19 +15122,19 @@
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>자동화</t>
         </is>
       </c>
       <c r="D67" s="8" t="inlineStr">
         <is>
-          <t>포션 단축키 (1/2/3/4), 레벨별 추천 활동 가이드</t>
+          <t>자동 스킬 시전 (인간 플레이어용), 자동 스킬 토글 버튼</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
@@ -15144,19 +15144,19 @@
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>시스템</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>장비 자동 최적화 (auto_equip_best), 알림 센터</t>
+          <t>미니맵 친구 위치 표시, 보스 표시 강화, DPS 미터 스파크라인</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
@@ -15166,12 +15166,12 @@
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>컨텐츠</t>
+          <t>시스템</t>
         </is>
       </c>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>신규 업적 10종 (30→40), 신규 몬스터 존 3개</t>
+          <t>혈맹 창고 UI 패널, 보스 신규 디버프 적용</t>
         </is>
       </c>
     </row>
@@ -15188,32 +15188,120 @@
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>상태이상</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>인벤토리 검색 + 정렬, PvP 시즌 보드 시각화</t>
+          <t>신규 디버프 5종 (빙결/감전/출혈/약화/공포)</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>포션 단축키 (1/2/3/4), 레벨별 추천 활동 가이드</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>시스템</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>장비 자동 최적화 (auto_equip_best), 알림 센터</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="8" t="inlineStr">
+        <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B73" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>컨텐츠</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>신규 업적 10종 (30→40), 신규 몬스터 존 3개</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>인벤토리 검색 + 정렬, PvP 시즌 보드 시각화</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="inlineStr">
+        <is>
           <t>v1.6 이전</t>
         </is>
       </c>
-      <c r="B71" s="8" t="inlineStr">
+      <c r="B75" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C71" s="8" t="inlineStr">
+      <c r="C75" s="8" t="inlineStr">
         <is>
           <t>기반</t>
         </is>
       </c>
-      <c r="D71" s="8" t="inlineStr">
+      <c r="D75" s="8" t="inlineStr">
         <is>
           <t>마을/사냥/PvP/카르마/펫/탈것/제작/교역/길드/공성/투기장 등</t>
         </is>
@@ -15233,7 +15321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E90"/>
+  <dimension ref="A1:E96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -15280,7 +15368,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>v1.29</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -15290,78 +15378,78 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>season → server.js</t>
+          <t>boss_rush → server.js</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>4번째 모듈 통합</t>
+          <t>5번째 모듈 통합</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>XP 자동 적립 + 보상 수령</t>
+          <t>메모리 세션 기반</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>v1.29</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>자동화</t>
+          <t>상태</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>trackQuest 훅</t>
+          <t>bossRushSessions</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>PvP/보스/월드보스/던전/제작 → 시즌 XP</t>
+          <t>진행 중 세션 저장</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>SEASON_XP_MAP 매핑</t>
+          <t>currentWave/시간 추적</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>v1.29</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>소켓</t>
+          <t>상태</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>season_status</t>
+          <t>bossRushRanking</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>XP/티어/구매여부/수령내역 조회</t>
+          <t>글로벌 랭킹 TOP 100</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>15티어 전체</t>
+          <t>웨이브 → 시간 정렬</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>v1.29</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -15371,24 +15459,24 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>season_buy_pass</t>
+          <t>boss_rush_enter</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>프리미엄 패스 구매 (1500💎)</t>
+          <t>무료/유료/다이아 입장</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>전 서버 알림</t>
+          <t>동시 1개 세션 제한</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>v1.29</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -15398,159 +15486,159 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>season_claim</t>
+          <t>boss_rush_advance</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>티어 보상 수령 (free/premium)</t>
+          <t>웨이브 클리어 보고</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>자동 인벤토리 적용</t>
+          <t>시간 초과 검증</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>통합</t>
+          <t>보상</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>event → server.js</t>
+          <t>풀클리어 보상</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>3번째 모듈 통합</t>
+          <t>20웨이브 누적</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>축제 시스템 활성화</t>
+          <t>전 서버 알림</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>소켓</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>event_status</t>
+          <t>season → server.js</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>현재 활성 축제 조회</t>
+          <t>4번째 모듈 통합</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>이름/기간/버프/한정 보상</t>
+          <t>XP 자동 적립 + 보상 수령</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>자동화</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>/status JSON</t>
+          <t>trackQuest 훅</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>festival 필드 추가</t>
+          <t>PvP/보스/월드보스/던전/제작 → 시즌 XP</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>대시보드 확인용</t>
+          <t>SEASON_XP_MAP 매핑</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>NPC</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>축제 인사</t>
+          <t>season_status</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>30% 확률로 NPC가 축제 대사 출력</t>
+          <t>XP/티어/구매여부/수령내역 조회</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>spring_blossom 등 5종</t>
+          <t>15티어 전체</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>통합</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>fishing → server.js</t>
+          <t>season_buy_pass</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>require + 소켓 핸들러 3종</t>
+          <t>프리미엄 패스 구매 (1500💎)</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>두 번째 모듈 통합</t>
+          <t>전 서버 알림</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -15560,51 +15648,51 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>fishing_status</t>
+          <t>season_claim</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>지역/낚싯대/미끼/시간대 조회</t>
+          <t>티어 보상 수령 (free/premium)</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>클라이언트 표시용</t>
+          <t>자동 인벤토리 적용</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>소켓</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>fishing_cast</t>
+          <t>event → server.js</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>낚시 시도 (지역+낚싯대+미끼 검증)</t>
+          <t>3번째 모듈 통합</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>전설/신화 → 서버 알림</t>
+          <t>축제 시스템 활성화</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
@@ -15614,1880 +15702,1880 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>fishing_buy_rod</t>
+          <t>event_status</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>낚싯대 구매 (골드/다이아)</t>
+          <t>현재 활성 축제 조회</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>5등급 모두</t>
+          <t>이름/기간/버프/한정 보상</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>통합</t>
+          <t>API</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>lottery → server.js</t>
+          <t>/status JSON</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>require + 소켓 핸들러 3종</t>
+          <t>festival 필드 추가</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>첫 모듈 통합 마일스톤</t>
+          <t>대시보드 확인용</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>소켓 이벤트</t>
+          <t>NPC</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>lottery_status</t>
+          <t>축제 인사</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>상태/가격/상품 풀 조회</t>
+          <t>30% 확률로 NPC가 축제 대사 출력</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>클라이언트 표시용</t>
+          <t>spring_blossom 등 5종</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>소켓 이벤트</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>lottery_free_spin</t>
+          <t>fishing → server.js</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>매일 무료 1회 스핀</t>
+          <t>require + 소켓 핸들러 3종</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>자정 초기화</t>
+          <t>두 번째 모듈 통합</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>소켓 이벤트</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>lottery_paid_spin</t>
+          <t>fishing_status</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>유료 1회 / 10연속</t>
+          <t>지역/낚싯대/미끼/시간대 조회</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>count: 1 또는 10</t>
+          <t>클라이언트 표시용</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>game/auction.js 신규</t>
+          <t>fishing_cast</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>입찰식 / 3기간 / 5% 인상 / 스나이핑 방지</t>
+          <t>낚시 시도 (지역+낚싯대+미끼 검증)</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>등록 2% + 낙찰 5%</t>
+          <t>전설/신화 → 서버 알림</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>활성 한도</t>
+          <t>fishing_buy_rod</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>플레이어당 10개</t>
+          <t>낚싯대 구매 (골드/다이아)</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>자기 입찰 금지</t>
+          <t>5등급 모두</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>game/fishing.js 신규</t>
+          <t>lottery → server.js</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>11종 어종 / 5등급 낚싯대 / 4종 미끼</t>
+          <t>require + 소켓 핸들러 3종</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>신화 크라켄 = 20000G + 칭호</t>
+          <t>첫 모듈 통합 마일스톤</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>소켓 이벤트</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>전설의 비단잉어</t>
+          <t>lottery_status</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>드래곤 낚싯대 + 가중치 1</t>
+          <t>상태/가격/상품 풀 조회</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>5000G + 평생 행운 +5%</t>
+          <t>클라이언트 표시용</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>소켓 이벤트</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>game/boss_rush.js 신규</t>
+          <t>lottery_free_spin</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>20웨이브 / HP ×1.35 스케일링</t>
+          <t>매일 무료 1회 스핀</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>최종 보상: 200💎 + 용재료 ×5</t>
+          <t>자정 초기화</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>소켓 이벤트</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>입장</t>
+          <t>lottery_paid_spin</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>매일 무료 3회 / 1000G / 30💎</t>
+          <t>유료 1회 / 10연속</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>랭킹 시스템</t>
+          <t>count: 1 또는 10</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>챔피언 보상</t>
+          <t>game/auction.js 신규</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>1위: 500💎 + 칭호 / 2위: 300💎 / 3위: 200💎</t>
+          <t>입찰식 / 3기간 / 5% 인상 / 스나이핑 방지</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>등록 2% + 낙찰 5%</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>행운의 룰렛</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>game/lottery.js 신규</t>
+          <t>활성 한도</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>10종 보상 / 가중치 1000</t>
+          <t>플레이어당 10개</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>매일 무료 1회 + 유료</t>
+          <t>자기 입찰 금지</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>룰렛 (전설)</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>영웅 장비 상자</t>
+          <t>game/fishing.js 신규</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>확률 0.2% (가장 희귀)</t>
+          <t>11종 어종 / 5등급 낚싯대 / 4종 미끼</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>전설 보상</t>
+          <t>신화 크라켄 = 20000G + 칭호</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>룰렛 (전설)</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>200 다이아</t>
+          <t>전설의 비단잉어</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>확률 0.8%</t>
+          <t>드래곤 낚싯대 + 가중치 1</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>잭팟</t>
+          <t>5000G + 평생 행운 +5%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>신년 축제</t>
+          <t>game/boss_rush.js 신규</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>1/1 ~ 1/7</t>
+          <t>20웨이브 / HP ×1.35 스케일링</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>골드 +50% / EXP +30%</t>
+          <t>최종 보상: 200💎 + 용재료 ×5</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>봄꽃 축제</t>
+          <t>입장</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>4/1 ~ 4/14</t>
+          <t>매일 무료 3회 / 1000G / 30💎</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>HP재생 +30% / 드롭 +20%</t>
+          <t>랭킹 시스템</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>한여름 밤의 축제</t>
+          <t>챔피언 보상</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>7/15 ~ 8/15</t>
+          <t>1위: 500💎 + 칭호 / 2위: 300💎 / 3위: 200💎</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>화염 +30% / PvP 보상 +50%</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>행운의 룰렛</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>할로윈 축제</t>
+          <t>game/lottery.js 신규</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>10/25 ~ 11/1</t>
+          <t>10종 보상 / 가중치 1000</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>크리 +10% / 언데드 +50%</t>
+          <t>매일 무료 1회 + 유료</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>룰렛 (전설)</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>겨울 축제</t>
+          <t>영웅 장비 상자</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>12/20 ~ 12/31</t>
+          <t>확률 0.2% (가장 희귀)</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>골드 +30% / EXP +30% / 드롭 +30%</t>
+          <t>전설 보상</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>룰렛 (전설)</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>game/season.js 신규</t>
+          <t>200 다이아</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>15티어 / 30일 / 무료+프리미엄</t>
+          <t>확률 0.8%</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>만렙 보상: 태초 반지 + 시즌 칭호</t>
+          <t>잭팟</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>XP 획득 7종</t>
+          <t>신년 축제</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>퀘/보스/PvP/월드보스/던전/제작</t>
+          <t>1/1 ~ 1/7</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>일일 +200 ~ 월드보스 +500</t>
+          <t>골드 +50% / EXP +30%</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>프리미엄 가격</t>
+          <t>봄꽃 축제</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>1500 다이아</t>
+          <t>4/1 ~ 4/14</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>시즌 당 1회</t>
+          <t>HP재생 +30% / 드롭 +20%</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>Lv.40 달성</t>
+          <t>한여름 밤의 축제</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>각성기 해금 마일스톤</t>
+          <t>7/15 ~ 8/15</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>150💎</t>
+          <t>화염 +30% / PvP 보상 +50%</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Lv.50 달성</t>
+          <t>할로윈 축제</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>환생 가능 마일스톤</t>
+          <t>10/25 ~ 11/1</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>250💎</t>
+          <t>크리 +10% / 언데드 +50%</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>첫 환생</t>
+          <t>겨울 축제</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>prestige 1차</t>
+          <t>12/20 ~ 12/31</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>500💎</t>
+          <t>골드 +30% / EXP +30% / 드롭 +30%</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>첫 월드 보스</t>
+          <t>game/season.js 신규</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>월드 보스 처치 보너스</t>
+          <t>15티어 / 30일 / 무료+프리미엄</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>100💎</t>
+          <t>만렙 보상: 태초 반지 + 시즌 칭호</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>업적 50개</t>
+          <t>XP 획득 7종</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>업적 마일스톤</t>
+          <t>퀘/보스/PvP/월드보스/던전/제작</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>200💎</t>
+          <t>일일 +200 ~ 월드보스 +500</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>상점 (스킨)</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>불사조 스킨</t>
+          <t>프리미엄 가격</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>1200 다이아</t>
+          <t>1500 다이아</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>불사조 깃털 이펙트 (영구)</t>
+          <t>시즌 당 1회</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>상점 (스킨)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>폭풍 스킨</t>
+          <t>Lv.40 달성</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>1200 다이아</t>
+          <t>각성기 해금 마일스톤</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>번개 오라 이펙트 (영구)</t>
+          <t>150💎</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>상점 (편의)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>프리미엄 자동물약</t>
+          <t>Lv.50 달성</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>500 다이아</t>
+          <t>환생 가능 마일스톤</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>24시간 자동물약 무한</t>
+          <t>250💎</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>상점 (상자)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>프리미엄 보물 상자</t>
+          <t>첫 환생</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>300 다이아</t>
+          <t>prestige 1차</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>전설 장비 확정 + 다이아</t>
+          <t>500💎</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>상점 (재료)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>전설 재료 패키지</t>
+          <t>첫 월드 보스</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>600 다이아</t>
+          <t>월드 보스 처치 보너스</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>용재료×10 + 영혼석×20 + 마법재료×20</t>
+          <t>100💎</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>혈맹 Lv.6</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>혈맹의 분노</t>
+          <t>업적 50개</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>크리티컬 +5%</t>
+          <t>업적 마일스톤</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>60명 정원</t>
+          <t>200💎</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>혈맹 Lv.7</t>
+          <t>상점 (스킨)</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>혈맹의 신속</t>
+          <t>불사조 스킨</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>이동속도 +10%</t>
+          <t>1200 다이아</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>70명 정원</t>
+          <t>불사조 깃털 이펙트 (영구)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>혈맹 Lv.8</t>
+          <t>상점 (스킨)</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>혈맹의 회복</t>
+          <t>폭풍 스킨</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>HP 재생 +50%</t>
+          <t>1200 다이아</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t>80명 정원</t>
+          <t>번개 오라 이펙트 (영구)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>혈맹 Lv.9</t>
+          <t>상점 (편의)</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>혈맹의 운명</t>
+          <t>프리미엄 자동물약</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>회피 +5%</t>
+          <t>500 다이아</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>90명 정원</t>
+          <t>24시간 자동물약 무한</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>혈맹 Lv.10</t>
+          <t>상점 (상자)</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>혈맹의 전설</t>
+          <t>프리미엄 보물 상자</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>전 스탯 +5%</t>
+          <t>300 다이아</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
         <is>
-          <t>100명 정원 — 최종</t>
+          <t>전설 장비 확정 + 다이아</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>상점 (재료)</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>점쟁이</t>
+          <t>전설 재료 패키지</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>운세 / 행운 버프 (밤·카르마 반응)</t>
+          <t>600 다이아</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>상황 대사 4종</t>
+          <t>용재료×10 + 영혼석×20 + 마법재료×20</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>혈맹 Lv.6</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>감정사</t>
+          <t>혈맹의 분노</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>미감정 장비 감정 (Lv.30+ 특수)</t>
+          <t>크리티컬 +5%</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t>상황 대사 4종</t>
+          <t>60명 정원</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>혈맹 Lv.7</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>수집가</t>
+          <t>혈맹의 신속</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>희귀 아이템 매입 (골드 50000+ 특별)</t>
+          <t>이동속도 +10%</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>상황 대사 4종</t>
+          <t>70명 정원</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>각성기 (어쌔신)</t>
+          <t>혈맹 Lv.8</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>천 개의 칼날</t>
+          <t>혈맹의 회복</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>3.5배 × 7타 / 광역 / 쿨150초</t>
+          <t>HP 재생 +50%</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>80명 정원</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>각성기 (워리어)</t>
+          <t>혈맹 Lv.9</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>대지 가르기</t>
+          <t>혈맹의 운명</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>6.0배 / 광역 5범위 / 스턴 2초</t>
+          <t>회피 +5%</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>90명 정원</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>각성기 (나이트)</t>
+          <t>혈맹 Lv.10</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>불멸의 수호자</t>
+          <t>혈맹의 전설</t>
         </is>
       </c>
       <c r="D59" s="8" t="inlineStr">
         <is>
-          <t>피해 90% 감소 / 도발 / 10초</t>
+          <t>전 스탯 +5%</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>100명 정원 — 최종</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>각성기 (메이지)</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>시간 정지</t>
+          <t>점쟁이</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>12.0배 / 광역 6범위 / 슬로우 90%</t>
+          <t>운세 / 행운 버프 (밤·카르마 반응)</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>상황 대사 4종</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>각성기 (클레릭)</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>신의 은총</t>
+          <t>감정사</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>HP 100% 회복 / 전스탯 +50%</t>
+          <t>미감정 장비 감정 (Lv.30+ 특수)</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>상황 대사 4종</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>폭풍 정복자</t>
+          <t>수집가</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>폭풍의 거인 처치</t>
+          <t>희귀 아이템 매입 (골드 50000+ 특별)</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>10,000G + 150다이아</t>
+          <t>상황 대사 4종</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (어쌔신)</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>연금술사</t>
+          <t>천 개의 칼날</t>
         </is>
       </c>
       <c r="D63" s="8" t="inlineStr">
         <is>
-          <t>엘릭서 10회 제작</t>
+          <t>3.5배 × 7타 / 광역 / 쿨150초</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t>5,000G + 80다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (워리어)</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>그림자 정복자</t>
+          <t>대지 가르기</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>그림자 미궁 클리어</t>
+          <t>6.0배 / 광역 5범위 / 스턴 2초</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>8,000G + 120다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (나이트)</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>전설의 동반자</t>
+          <t>불멸의 수호자</t>
         </is>
       </c>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>전설급 펫 진화</t>
+          <t>피해 90% 감소 / 도발 / 10초</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>6,000G + 100다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (메이지)</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>이국의 상인</t>
+          <t>시간 정지</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>사치품 교역 5회</t>
+          <t>12.0배 / 광역 6범위 / 슬로우 90%</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>4,000G + 60다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>월드 보스</t>
+          <t>각성기 (클레릭)</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>폭풍의 거인</t>
+          <t>신의 은총</t>
         </is>
       </c>
       <c r="D67" s="8" t="inlineStr">
         <is>
-          <t>HP 100,000 / ATK 140 / DEF 90</t>
+          <t>HP 100% 회복 / 전스탯 +50%</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t>EXP 10000 + 6000G</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>월드 보스</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>시간의 수호자</t>
+          <t>폭풍 정복자</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>HP 70,000 / ATK 170 / DEF 60</t>
+          <t>폭풍의 거인 처치</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>EXP 9000 + 7000G</t>
+          <t>10,000G + 150다이아</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>교역품</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>불사조 깃털 / 공허의 정수 / 천공의 비단</t>
+          <t>연금술사</t>
         </is>
       </c>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>이국의 사치품 3종</t>
+          <t>엘릭서 10회 제작</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>기본가 600~900G</t>
+          <t>5,000G + 80다이아</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>타이탄의 엘릭서</t>
+          <t>그림자 정복자</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>용재료×3 + 마법재료×10</t>
+          <t>그림자 미궁 클리어</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>ATK ×1.5 / 30분</t>
+          <t>8,000G + 120다이아</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>강철 엘릭서</t>
+          <t>전설의 동반자</t>
         </is>
       </c>
       <c r="D71" s="8" t="inlineStr">
         <is>
-          <t>철광석×30 + 마법재료×10</t>
+          <t>전설급 펫 진화</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t>DEF ×1.5 / 30분</t>
+          <t>6,000G + 100다이아</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>질풍 엘릭서</t>
+          <t>이국의 상인</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>약초×20 + 마법재료×8</t>
+          <t>사치품 교역 5회</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>SPD ×1.4 / 20분</t>
+          <t>4,000G + 60다이아</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>월드 보스</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>지혜 엘릭서</t>
+          <t>폭풍의 거인</t>
         </is>
       </c>
       <c r="D73" s="8" t="inlineStr">
         <is>
-          <t>마법수정×5 + 영혼재료×5</t>
+          <t>HP 100,000 / ATK 140 / DEF 90</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t>EXP ×2.5 / 15분</t>
+          <t>EXP 10000 + 6000G</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>월드 보스</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>행운 엘릭서</t>
+          <t>시간의 수호자</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>보석×10 + 마법재료×5</t>
+          <t>HP 70,000 / ATK 170 / DEF 60</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>GOLD ×2.0 / 15분</t>
+          <t>EXP 9000 + 7000G</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>신규 펫</t>
+          <t>교역품</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t>불사조 (pet_phoenix)</t>
+          <t>불사조 깃털 / 공허의 정수 / 천공의 비단</t>
         </is>
       </c>
       <c r="D75" s="8" t="inlineStr">
         <is>
-          <t>불꽃산 보스 50처치</t>
+          <t>이국의 사치품 3종</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
         <is>
-          <t>화염 DMG +20% (진화 +40%)</t>
+          <t>기본가 600~900G</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>신규 펫</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>유니콘 (pet_unicorn)</t>
+          <t>타이탄의 엘릭서</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>다이아 800개</t>
+          <t>용재료×3 + 마법재료×10</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>회피 +10% (진화 +20%)</t>
+          <t>ATK ×1.5 / 30분</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>신규 탈것</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t>페가수스 (mount_pegasus)</t>
+          <t>강철 엘릭서</t>
         </is>
       </c>
       <c r="D77" s="8" t="inlineStr">
         <is>
-          <t>다이아 1200개</t>
+          <t>철광석×30 + 마법재료×10</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
         <is>
-          <t>이동속도 +85% / 비행</t>
+          <t>DEF ×1.5 / 30분</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>신규 던전</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>그림자 미궁</t>
+          <t>질풍 엘릭서</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>Lv.38 / 8인 파티 / 7스테이지</t>
+          <t>약초×20 + 마법재료×8</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>22000G + 32000EXP</t>
+          <t>SPD ×1.4 / 20분</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>드롭</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>드래곤 검/망토/투구/장갑</t>
+          <t>지혜 엘릭서</t>
         </is>
       </c>
       <c r="D79" s="8" t="inlineStr">
         <is>
-          <t>그림자 미궁 보스 드롭</t>
+          <t>마법수정×5 + 영혼재료×5</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
         <is>
-          <t>전설급</t>
+          <t>EXP ×2.5 / 15분</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>공허의 방랑자</t>
+          <t>행운 엘릭서</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>몬스터 10,000 처치</t>
+          <t>보석×10 + 마법재료×5</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>ATK +7%</t>
+          <t>GOLD ×2.0 / 15분</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 펫</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t>불멸자</t>
+          <t>불사조 (pet_phoenix)</t>
         </is>
       </c>
       <c r="D81" s="8" t="inlineStr">
         <is>
-          <t>환생 5회</t>
+          <t>불꽃산 보스 50처치</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr">
         <is>
-          <t>EXP +25%</t>
+          <t>화염 DMG +20% (진화 +40%)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 펫</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>천공의 군주</t>
+          <t>유니콘 (pet_unicorn)</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>월드 보스 10회 처치</t>
+          <t>다이아 800개</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>보스DMG +15%</t>
+          <t>회피 +10% (진화 +20%)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>신규 탈것</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t>지역 시트 갱신</t>
+          <t>페가수스 (mount_pegasus)</t>
         </is>
       </c>
       <c r="D83" s="8" t="inlineStr">
         <is>
-          <t>25→51개 지역 반영</t>
+          <t>다이아 1200개</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>이동속도 +85% / 비행</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>신규 던전</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>칭호 시트 갱신</t>
+          <t>그림자 미궁</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>7→16종 + 효과/색상 추가</t>
+          <t>Lv.38 / 8인 파티 / 7스테이지</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22000G + 32000EXP</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B85" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>드롭</t>
         </is>
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t>출석 캘린더 시트</t>
+          <t>드래곤 검/망토/투구/장갑</t>
         </is>
       </c>
       <c r="D85" s="8" t="inlineStr">
         <is>
-          <t>신규 추가 (28일 사이클)</t>
+          <t>그림자 미궁 보스 드롭</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>전설급</t>
         </is>
       </c>
     </row>
@@ -17499,22 +17587,22 @@
       </c>
       <c r="B86" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>장비 세트 시트</t>
+          <t>공허의 방랑자</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>신규 추가 (드래곤/영웅/태초)</t>
+          <t>몬스터 10,000 처치</t>
         </is>
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ATK +7%</t>
         </is>
       </c>
     </row>
@@ -17526,22 +17614,22 @@
       </c>
       <c r="B87" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t>장비 등급 시트</t>
+          <t>불멸자</t>
         </is>
       </c>
       <c r="D87" s="8" t="inlineStr">
         <is>
-          <t>신규 추가 (5등급 + 랜덤 옵션 7종)</t>
+          <t>환생 5회</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EXP +25%</t>
         </is>
       </c>
     </row>
@@ -17553,22 +17641,22 @@
       </c>
       <c r="B88" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>디버프 시트</t>
+          <t>천공의 군주</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>신규 추가 (10종, v1.7 5종 포함)</t>
+          <t>월드 보스 10회 처치</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>보스DMG +15%</t>
         </is>
       </c>
     </row>
@@ -17585,12 +17673,12 @@
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t>패치 노트 시트</t>
+          <t>지역 시트 갱신</t>
         </is>
       </c>
       <c r="D89" s="8" t="inlineStr">
         <is>
-          <t>신규 추가 (히스토리)</t>
+          <t>25→51개 지역 반영</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr">
@@ -17602,25 +17690,187 @@
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
         <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B90" s="7" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C90" s="7" t="inlineStr">
+        <is>
+          <t>칭호 시트 갱신</t>
+        </is>
+      </c>
+      <c r="D90" s="7" t="inlineStr">
+        <is>
+          <t>7→16종 + 효과/색상 추가</t>
+        </is>
+      </c>
+      <c r="E90" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="8" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B91" s="8" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C91" s="8" t="inlineStr">
+        <is>
+          <t>출석 캘린더 시트</t>
+        </is>
+      </c>
+      <c r="D91" s="8" t="inlineStr">
+        <is>
+          <t>신규 추가 (28일 사이클)</t>
+        </is>
+      </c>
+      <c r="E91" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="7" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B92" s="7" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C92" s="7" t="inlineStr">
+        <is>
+          <t>장비 세트 시트</t>
+        </is>
+      </c>
+      <c r="D92" s="7" t="inlineStr">
+        <is>
+          <t>신규 추가 (드래곤/영웅/태초)</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="8" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B93" s="8" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C93" s="8" t="inlineStr">
+        <is>
+          <t>장비 등급 시트</t>
+        </is>
+      </c>
+      <c r="D93" s="8" t="inlineStr">
+        <is>
+          <t>신규 추가 (5등급 + 랜덤 옵션 7종)</t>
+        </is>
+      </c>
+      <c r="E93" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="7" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B94" s="7" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C94" s="7" t="inlineStr">
+        <is>
+          <t>디버프 시트</t>
+        </is>
+      </c>
+      <c r="D94" s="7" t="inlineStr">
+        <is>
+          <t>신규 추가 (10종, v1.7 5종 포함)</t>
+        </is>
+      </c>
+      <c r="E94" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="8" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B95" s="8" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>패치 노트 시트</t>
+        </is>
+      </c>
+      <c r="D95" s="8" t="inlineStr">
+        <is>
+          <t>신규 추가 (히스토리)</t>
+        </is>
+      </c>
+      <c r="E95" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="7" t="inlineStr">
+        <is>
           <t>v1.10</t>
         </is>
       </c>
-      <c r="B90" s="7" t="inlineStr">
+      <c r="B96" s="7" t="inlineStr">
         <is>
           <t>기획서</t>
         </is>
       </c>
-      <c r="C90" s="7" t="inlineStr">
+      <c r="C96" s="7" t="inlineStr">
         <is>
           <t>던전 시트</t>
         </is>
       </c>
-      <c r="D90" s="7" t="inlineStr">
+      <c r="D96" s="7" t="inlineStr">
         <is>
           <t>신규 추가 (7종 던전)</t>
         </is>
       </c>
-      <c r="E90" s="7" t="inlineStr">
+      <c r="E96" s="7" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
feat: v1.31 — game/auction.js를 server.js에 통합 (6번째 = 마지막 모듈)
🎉 v1.20~v1.25 신규 모듈 6개 100% 통합 완료

경매장 시스템 활성화:
- require('./game/auction')
- 소켓 핸들러 4종:
  * auction_list — 활성 경매 목록 (필터 가능)
  * auction_create — 경매 등록 (이름 자동 매핑, 등록 수수료 차감)
  * auction_bid — 입찰 (이전 입찰자 자동 환불 + 스나이핑 방지)
  * auction_my — 내 등록/입찰 내역
- 자동 정산 틱: 메인 setInterval에 10초마다 tickAuctions() 호출
  * 낙찰 성공: 판매자에게 (낙찰가 - 5%수수료) 골드 지급
              + 구매자에게 아이템 지급
              + auction_sold / auction_won 이벤트
  * 유찰: 판매자에게 아이템 반환 + auction_failed 이벤트
- 입찰 시 이전 최고 입찰자 골드 환불 + auction_outbid 알림
- 스나이핑 방지 연장 시 auction_extended 이벤트

통합 진척:
- v1.26 lottery   ✅
- v1.27 fishing   ✅
- v1.28 event     ✅
- v1.29 season    ✅
- v1.30 boss_rush ✅
- v1.31 auction   ✅ (마지막)

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutoBattle_io_기획서.xlsx
+++ b/AutoBattle_io_기획서.xlsx
@@ -40,7 +40,7 @@
     <sheet name="월드 보스" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="연금술" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="패치 노트" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="v1.9 ~ v1.30" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="v1.9 ~ v1.31" sheetId="34" state="visible" r:id="rId34"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -13685,7 +13685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D75"/>
+  <dimension ref="A1:D80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13726,7 +13726,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>v1.30</t>
+          <t>v1.31</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -13741,14 +13741,14 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>game/boss_rush.js → server.js 통합 (5번째 모듈 통합)</t>
+          <t>game/auction.js → server.js 통합 (6번째 = 마지막 모듈 통합)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>v1.30</t>
+          <t>v1.31</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -13758,19 +13758,19 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>메모리 세션 + 시간 검증 + 누적 보상 + 랭킹 (TOP 100)</t>
+          <t>자동 정산 틱 (10초마다 tickAuctions())</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>v1.30</t>
+          <t>v1.31</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
@@ -13780,19 +13780,19 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>소켓</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>boss_rush_status / enter / advance / abandon</t>
+          <t>이전 입찰자 자동 환불, 낙찰 시 아이템/골드 양방향 지급</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>v1.30</t>
+          <t>v1.31</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -13802,19 +13802,19 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>풀클리어 시 전 서버 알림, 10웨이브+ 일반 알림</t>
+          <t>auction_list / create / bid / my</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>v1.29</t>
+          <t>v1.31</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -13824,19 +13824,19 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>통합</t>
+          <t>마일스톤</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>game/season.js → server.js 통합 (4번째 모듈 통합)</t>
+          <t>🎉 v1.20~v1.25 신규 모듈 6개 모두 통합 완료</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>v1.29</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -13846,19 +13846,19 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>trackQuest 자동 XP 적립 (PvP/보스/월드보스/던전/제작)</t>
+          <t>game/boss_rush.js → server.js 통합 (5번째 모듈 통합)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>v1.29</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -13868,19 +13868,19 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>소켓</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>season_status / season_buy_pass / season_claim</t>
+          <t>메모리 세션 + 시간 검증 + 누적 보상 + 랭킹 (TOP 100)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>v1.29</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -13890,19 +13890,19 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>티어 승급 시 server_msg + season_tier_up 알림</t>
+          <t>boss_rush_status / enter / advance / abandon</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -13912,19 +13912,19 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>통합</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>game/event.js → server.js 통합 (3번째 모듈 통합)</t>
+          <t>풀클리어 시 전 서버 알림, 10웨이브+ 일반 알림</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -13934,19 +13934,19 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>축제</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>event_status 소켓 + /status 엔드포인트 노출</t>
+          <t>game/season.js → server.js 통합 (4번째 모듈 통합)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -13956,19 +13956,19 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>축제</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>NPC 대사 30% 확률로 축제 인사 (getNpcMsg 통합)</t>
+          <t>trackQuest 자동 XP 적립 (PvP/보스/월드보스/던전/제작)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -13978,19 +13978,19 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>검증</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>오늘(4/8) 봄꽃 축제 활성 동작 확인</t>
+          <t>season_status / season_buy_pass / season_claim</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
@@ -14000,19 +14000,19 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>통합</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>game/fishing.js → server.js 통합 (소켓 핸들러 3종)</t>
+          <t>티어 승급 시 server_msg + season_tier_up 알림</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
@@ -14022,19 +14022,19 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>fishing_status / fishing_cast / fishing_buy_rod 이벤트</t>
+          <t>game/event.js → server.js 통합 (3번째 모듈 통합)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -14044,19 +14044,19 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>축제</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>지역 검증 (낚시 만/강변/산호초), 낚싯대 보유 검증, 미끼 소비</t>
+          <t>event_status 소켓 + /status 엔드포인트 노출</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
@@ -14066,19 +14066,19 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>축제</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>전설/신화 어종 낚시 시 전 서버 알림 + ach_fish50 추적</t>
+          <t>NPC 대사 30% 확률로 축제 인사 (getNpcMsg 통합)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -14088,19 +14088,19 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>통합</t>
+          <t>검증</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>game/lottery.js → server.js 통합 (require + 소켓 핸들러 3종)</t>
+          <t>오늘(4/8) 봄꽃 축제 활성 동작 확인</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
@@ -14110,19 +14110,19 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>룰렛</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>lottery_status / lottery_free_spin / lottery_paid_spin 이벤트 추가</t>
+          <t>game/fishing.js → server.js 통합 (소켓 핸들러 3종)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -14132,19 +14132,19 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>룰렛</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>전설/영웅 보상 획득 시 전 서버 알림 + ach_lucky 업적 추적</t>
+          <t>fishing_status / fishing_cast / fishing_buy_rod 이벤트</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
@@ -14154,19 +14154,19 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>입찰식 경매 시스템 (game/auction.js 신규 모듈)</t>
+          <t>지역 검증 (낚시 만/강변/산호초), 낚싯대 보유 검증, 미끼 소비</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -14176,19 +14176,19 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>3가지 기간(1h/6h/24h) + 등록2% + 낙찰5% + 스나이핑 방지</t>
+          <t>전설/신화 어종 낚시 시 전 서버 알림 + ach_fish50 추적</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
@@ -14198,19 +14198,19 @@
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>경매장 시트 신규 추가</t>
+          <t>game/lottery.js → server.js 통합 (require + 소켓 핸들러 3종)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -14220,19 +14220,19 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>룰렛</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>11종 어종 + 5등급 낚싯대 + 4종 미끼 (game/fishing.js 신규 모듈)</t>
+          <t>lottery_status / lottery_free_spin / lottery_paid_spin 이벤트 추가</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
@@ -14242,19 +14242,19 @@
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>룰렛</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>신화 크라켄 (밤+낚시터+드래곤대 한정), 바다의 군주 칭호 연계</t>
+          <t>전설/영웅 보상 획득 시 전 서버 알림 + ach_lucky 업적 추적</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -14264,19 +14264,19 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>낚시 시트 신규 추가</t>
+          <t>입찰식 경매 시스템 (game/auction.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
@@ -14286,19 +14286,19 @@
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>20웨이브 엔드리스 보스 러시 모드 (game/boss_rush.js 신규 모듈)</t>
+          <t>3가지 기간(1h/6h/24h) + 등록2% + 낙찰5% + 스나이핑 방지</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -14308,19 +14308,19 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>매일 무료 3회 + 랭킹 1위 챔피언 칭호</t>
+          <t>경매장 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
@@ -14330,19 +14330,19 @@
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>보스 러시 시트 신규 추가</t>
+          <t>11종 어종 + 5등급 낚싯대 + 4종 미끼 (game/fishing.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -14352,19 +14352,19 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>행운의 룰렛</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>10종 보상 + 가중치 시스템 (game/lottery.js 신규 모듈)</t>
+          <t>신화 크라켄 (밤+낚시터+드래곤대 한정), 바다의 군주 칭호 연계</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
@@ -14374,19 +14374,19 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>룰렛</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>매일 무료 1회 / 유료 50💎 / 10연속 450💎 (10% 할인)</t>
+          <t>낚시 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -14396,19 +14396,19 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>행운의 룰렛 시트 신규 추가</t>
+          <t>20웨이브 엔드리스 보스 러시 모드 (game/boss_rush.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
@@ -14418,19 +14418,19 @@
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>5종 시즌 축제 추가 (신년/봄꽃/한여름/할로윈/겨울)</t>
+          <t>매일 무료 3회 + 랭킹 1위 챔피언 칭호</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -14440,19 +14440,19 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>모듈화</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>game/event.js 신규 파일 (실제 달력 기반 자동 활성화)</t>
+          <t>보스 러시 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
@@ -14462,19 +14462,19 @@
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>행운의 룰렛</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트 시트 신규 추가</t>
+          <t>10종 보상 + 가중치 시스템 (game/lottery.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -14484,19 +14484,19 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>룰렛</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>15티어 배틀 패스 시스템 추가 (game/season.js 신규 모듈)</t>
+          <t>매일 무료 1회 / 유료 50💎 / 10연속 450💎 (10% 할인)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
@@ -14506,19 +14506,19 @@
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>30일 사이클, 무료+프리미엄(1500💎) 트랙</t>
+          <t>행운의 룰렛 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -14528,19 +14528,19 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>시즌 패스 시트 신규 추가</t>
+          <t>5종 시즌 축제 추가 (신년/봄꽃/한여름/할로윈/겨울)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
@@ -14550,19 +14550,19 @@
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>모듈화</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>마일스톤 5종 추가 (Lv.40/50, 첫 환생, 첫 월드 보스, 업적 50)</t>
+          <t>game/event.js 신규 파일 (실제 달력 기반 자동 활성화)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -14577,14 +14577,14 @@
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>무료 다이아 시트 신규 추가</t>
+          <t>축제 이벤트 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
@@ -14594,19 +14594,19 @@
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>상점</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>프리미엄 5종 추가 (불사조/폭풍 스킨, 자동물약 24h, 보물상자, 재료 패키지)</t>
+          <t>15티어 배틀 패스 시스템 추가 (game/season.js 신규 모듈)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -14616,19 +14616,19 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>상점 시트 갱신</t>
+          <t>30일 사이클, 무료+프리미엄(1500💎) 트랙</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
@@ -14638,19 +14638,19 @@
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>혈맹</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>혈맹 Lv.6-10 + 신규 스킬 5종 (분노/신속/회복/운명/전설)</t>
+          <t>시즌 패스 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -14660,19 +14660,19 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>혈맹</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>최대 인원 50→100명 (Lv.10 기준)</t>
+          <t>마일스톤 5종 추가 (Lv.40/50, 첫 환생, 첫 월드 보스, 업적 50)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
@@ -14687,14 +14687,14 @@
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>길드(혈맹) 시트 신규 추가</t>
+          <t>무료 다이아 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -14704,19 +14704,19 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>상점</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>점쟁이/감정사/수집가 3종 추가 (운세/감정/희귀품 매입)</t>
+          <t>프리미엄 5종 추가 (불사조/폭풍 스킨, 자동물약 24h, 보물상자, 재료 패키지)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
@@ -14726,19 +14726,19 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>대사 시스템</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>신규 NPC 상황별 대사 (밤/카르마/레벨/골드 연동)</t>
+          <t>상점 시트 갱신</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -14748,19 +14748,19 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>혈맹</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>NPC 시트 신규 추가 (11종)</t>
+          <t>혈맹 Lv.6-10 + 신규 스킬 5종 (분노/신속/회복/운명/전설)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
@@ -14770,19 +14770,19 @@
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>각성기</t>
+          <t>혈맹</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>클래스별 Lv.40 각성기 5종 추가 (천개의칼날/대지가르기/불멸의수호자/시간정지/신의은총)</t>
+          <t>최대 인원 50→100명 (Lv.10 기준)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -14797,14 +14797,14 @@
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>스킬 시트 전면 갱신 (12종→30종, 클레릭 포함)</t>
+          <t>길드(혈맹) 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
@@ -14814,19 +14814,19 @@
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>v1.9~v1.13 컨텐츠 연계 업적 5종 추가 (폭풍 정복자/연금술사/그림자/전설 동반자/이국 상인)</t>
+          <t>점쟁이/감정사/수집가 3종 추가 (운세/감정/희귀품 매입)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -14836,19 +14836,19 @@
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>대사 시스템</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>퀘스트 시트 전면 갱신 (9종→64종 반영)</t>
+          <t>신규 NPC 상황별 대사 (밤/카르마/레벨/골드 연동)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
@@ -14858,19 +14858,19 @@
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>월드 보스</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>폭풍의 거인 / 시간의 수호자 2종 추가 (최대 HP / 최강 ATK)</t>
+          <t>NPC 시트 신규 추가 (11종)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -14880,19 +14880,19 @@
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>교역</t>
+          <t>각성기</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>이국의 사치품 3종 추가 (불사조 깃털/공허의 정수/천공의 비단)</t>
+          <t>클래스별 Lv.40 각성기 5종 추가 (천개의칼날/대지가르기/불멸의수호자/시간정지/신의은총)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
@@ -14907,14 +14907,14 @@
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>월드 보스 시트 신규 추가, 교역 시트 갱신</t>
+          <t>스킬 시트 전면 갱신 (12종→30종, 클레릭 포함)</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -14924,19 +14924,19 @@
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>엘릭서 5종 추가 (타이탄/강철/질풍/지혜/행운, 15~30분 강력 버프)</t>
+          <t>v1.9~v1.13 컨텐츠 연계 업적 5종 추가 (폭풍 정복자/연금술사/그림자/전설 동반자/이국 상인)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
@@ -14951,14 +14951,14 @@
       </c>
       <c r="D59" s="8" t="inlineStr">
         <is>
-          <t>연금술 시트 신규 추가</t>
+          <t>퀘스트 시트 전면 갱신 (9종→64종 반영)</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -14968,19 +14968,19 @@
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>신규 펫</t>
+          <t>월드 보스</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>불사조 (화염 +20%) / 유니콘 (회피 +10%) + 진화형</t>
+          <t>폭풍의 거인 / 시간의 수호자 2종 추가 (최대 HP / 최강 ATK)</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
@@ -14990,19 +14990,19 @@
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>신규 탈것</t>
+          <t>교역</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>페가수스 (이동 +85%, 비행)</t>
+          <t>이국의 사치품 3종 추가 (불사조 깃털/공허의 정수/천공의 비단)</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -15012,19 +15012,19 @@
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>신규 던전</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>그림자 미궁 (Lv.38, 8인 파티, 7스테이지, 전설 드롭)</t>
+          <t>월드 보스 시트 신규 추가, 교역 시트 갱신</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
@@ -15034,19 +15034,19 @@
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="D63" s="8" t="inlineStr">
         <is>
-          <t>던전 시트 신규 추가 (7종 던전 정리)</t>
+          <t>엘릭서 5종 추가 (타이탄/강철/질풍/지혜/행운, 15~30분 강력 버프)</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
@@ -15056,19 +15056,19 @@
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>공허의 방랑자/불멸자/천공의 군주 3종 추가 (엔드게임)</t>
+          <t>연금술 시트 신규 추가</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
@@ -15078,129 +15078,129 @@
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>신규 펫</t>
         </is>
       </c>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>51개 지역, 16종 칭호, 출석/세트/등급 시트 추가</t>
+          <t>불사조 (화염 +20%) / 유니콘 (회피 +10%) + 진화형</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>신규 탈것</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>패치 노트 갱신, 낮/밤 시계 + 진행 시간 표시</t>
+          <t>페가수스 (이동 +85%, 비행)</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>자동화</t>
+          <t>신규 던전</t>
         </is>
       </c>
       <c r="D67" s="8" t="inlineStr">
         <is>
-          <t>자동 스킬 시전 (인간 플레이어용), 자동 스킬 토글 버튼</t>
+          <t>그림자 미궁 (Lv.38, 8인 파티, 7스테이지, 전설 드롭)</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>미니맵 친구 위치 표시, 보스 표시 강화, DPS 미터 스파크라인</t>
+          <t>던전 시트 신규 추가 (7종 던전 정리)</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t>v1.8</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>시스템</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>혈맹 창고 UI 패널, 보스 신규 디버프 적용</t>
+          <t>공허의 방랑자/불멸자/천공의 군주 3종 추가 (엔드게임)</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.9</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>상태이상</t>
+          <t>기획서</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>신규 디버프 5종 (빙결/감전/출혈/약화/공포)</t>
+          <t>51개 지역, 16종 칭호, 출석/세트/등급 시트 추가</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B71" s="8" t="inlineStr">
@@ -15215,14 +15215,14 @@
       </c>
       <c r="D71" s="8" t="inlineStr">
         <is>
-          <t>포션 단축키 (1/2/3/4), 레벨별 추천 활동 가이드</t>
+          <t>패치 노트 갱신, 낮/밤 시계 + 진행 시간 표시</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -15232,19 +15232,19 @@
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>시스템</t>
+          <t>자동화</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>장비 자동 최적화 (auto_equip_best), 알림 센터</t>
+          <t>자동 스킬 시전 (인간 플레이어용), 자동 스킬 토글 버튼</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B73" s="8" t="inlineStr">
@@ -15254,19 +15254,19 @@
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>컨텐츠</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="D73" s="8" t="inlineStr">
         <is>
-          <t>신규 업적 10종 (30→40), 신규 몬스터 존 3개</t>
+          <t>미니맵 친구 위치 표시, 보스 표시 강화, DPS 미터 스파크라인</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
         <is>
-          <t>v1.7</t>
+          <t>v1.8</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -15276,32 +15276,142 @@
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>시스템</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>인벤토리 검색 + 정렬, PvP 시즌 보드 시각화</t>
+          <t>혈맹 창고 UI 패널, 보스 신규 디버프 적용</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B75" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>상태이상</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>신규 디버프 5종 (빙결/감전/출혈/약화/공포)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="7" t="inlineStr">
+        <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>포션 단축키 (1/2/3/4), 레벨별 추천 활동 가이드</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="8" t="inlineStr">
+        <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B77" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>시스템</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="inlineStr">
+        <is>
+          <t>장비 자동 최적화 (auto_equip_best), 알림 센터</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="7" t="inlineStr">
+        <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>컨텐츠</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>신규 업적 10종 (30→40), 신규 몬스터 존 3개</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="inlineStr">
+        <is>
+          <t>v1.7</t>
+        </is>
+      </c>
+      <c r="B79" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="inlineStr">
+        <is>
+          <t>인벤토리 검색 + 정렬, PvP 시즌 보드 시각화</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="7" t="inlineStr">
+        <is>
           <t>v1.6 이전</t>
         </is>
       </c>
-      <c r="B75" s="8" t="inlineStr">
+      <c r="B80" s="7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C75" s="8" t="inlineStr">
+      <c r="C80" s="7" t="inlineStr">
         <is>
           <t>기반</t>
         </is>
       </c>
-      <c r="D75" s="8" t="inlineStr">
+      <c r="D80" s="7" t="inlineStr">
         <is>
           <t>마을/사냥/PvP/카르마/펫/탈것/제작/교역/길드/공성/투기장 등</t>
         </is>
@@ -15321,7 +15431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E96"/>
+  <dimension ref="A1:E102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -15368,7 +15478,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>v1.30</t>
+          <t>v1.31</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -15378,78 +15488,78 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>boss_rush → server.js</t>
+          <t>auction → server.js</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>5번째 모듈 통합</t>
+          <t>6번째 (마지막) 모듈 통합</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>메모리 세션 기반</t>
+          <t>자동 정산 + 환불 + 양방향 지급</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>v1.30</t>
+          <t>v1.31</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>상태</t>
+          <t>자동화</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>bossRushSessions</t>
+          <t>tickAuctions</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>진행 중 세션 저장</t>
+          <t>10초마다 만료 정산</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>currentWave/시간 추적</t>
+          <t>setInterval 통합</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>v1.30</t>
+          <t>v1.31</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>상태</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>bossRushRanking</t>
+          <t>auction_create</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>글로벌 랭킹 TOP 100</t>
+          <t>경매 등록 (등록 수수료 자동 차감)</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>웨이브 → 시간 정렬</t>
+          <t>3가지 기간</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>v1.30</t>
+          <t>v1.31</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -15459,24 +15569,24 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>boss_rush_enter</t>
+          <t>auction_bid</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>무료/유료/다이아 입장</t>
+          <t>입찰 + 이전 입찰자 자동 환불</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>동시 1개 세션 제한</t>
+          <t>스나이핑 방지 연장</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>v1.30</t>
+          <t>v1.31</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -15486,51 +15596,51 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>boss_rush_advance</t>
+          <t>auction_my</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>웨이브 클리어 보고</t>
+          <t>내 등록/입찰 내역 조회</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>시간 초과 검증</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>v1.30</t>
+          <t>v1.31</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>보상</t>
+          <t>마일스톤</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>풀클리어 보상</t>
+          <t>신규 모듈 6/6</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>20웨이브 누적</t>
+          <t>100% 통합 완료</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>전 서버 알림</t>
+          <t>lottery/fishing/event/season/boss_rush/auction</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>v1.29</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -15540,78 +15650,78 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>season → server.js</t>
+          <t>boss_rush → server.js</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>4번째 모듈 통합</t>
+          <t>5번째 모듈 통합</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>XP 자동 적립 + 보상 수령</t>
+          <t>메모리 세션 기반</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>v1.29</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>자동화</t>
+          <t>상태</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>trackQuest 훅</t>
+          <t>bossRushSessions</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>PvP/보스/월드보스/던전/제작 → 시즌 XP</t>
+          <t>진행 중 세션 저장</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>SEASON_XP_MAP 매핑</t>
+          <t>currentWave/시간 추적</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>v1.29</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>소켓</t>
+          <t>상태</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>season_status</t>
+          <t>bossRushRanking</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>XP/티어/구매여부/수령내역 조회</t>
+          <t>글로벌 랭킹 TOP 100</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>15티어 전체</t>
+          <t>웨이브 → 시간 정렬</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>v1.29</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -15621,24 +15731,24 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>season_buy_pass</t>
+          <t>boss_rush_enter</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>프리미엄 패스 구매 (1500💎)</t>
+          <t>무료/유료/다이아 입장</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>전 서버 알림</t>
+          <t>동시 1개 세션 제한</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>v1.29</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -15648,159 +15758,159 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>season_claim</t>
+          <t>boss_rush_advance</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>티어 보상 수령 (free/premium)</t>
+          <t>웨이브 클리어 보고</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>자동 인벤토리 적용</t>
+          <t>시간 초과 검증</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.30</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>통합</t>
+          <t>보상</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>event → server.js</t>
+          <t>풀클리어 보상</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>3번째 모듈 통합</t>
+          <t>20웨이브 누적</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>축제 시스템 활성화</t>
+          <t>전 서버 알림</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>소켓</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>event_status</t>
+          <t>season → server.js</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>현재 활성 축제 조회</t>
+          <t>4번째 모듈 통합</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>이름/기간/버프/한정 보상</t>
+          <t>XP 자동 적립 + 보상 수령</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>자동화</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>/status JSON</t>
+          <t>trackQuest 훅</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>festival 필드 추가</t>
+          <t>PvP/보스/월드보스/던전/제작 → 시즌 XP</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>대시보드 확인용</t>
+          <t>SEASON_XP_MAP 매핑</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>v1.28</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>NPC</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>축제 인사</t>
+          <t>season_status</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>30% 확률로 NPC가 축제 대사 출력</t>
+          <t>XP/티어/구매여부/수령내역 조회</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>spring_blossom 등 5종</t>
+          <t>15티어 전체</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>통합</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>fishing → server.js</t>
+          <t>season_buy_pass</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>require + 소켓 핸들러 3종</t>
+          <t>프리미엄 패스 구매 (1500💎)</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>두 번째 모듈 통합</t>
+          <t>전 서버 알림</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.29</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -15810,51 +15920,51 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>fishing_status</t>
+          <t>season_claim</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>지역/낚싯대/미끼/시간대 조회</t>
+          <t>티어 보상 수령 (free/premium)</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>클라이언트 표시용</t>
+          <t>자동 인벤토리 적용</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>소켓</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>fishing_cast</t>
+          <t>event → server.js</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>낚시 시도 (지역+낚싯대+미끼 검증)</t>
+          <t>3번째 모듈 통합</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>전설/신화 → 서버 알림</t>
+          <t>축제 시스템 활성화</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>v1.27</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -15864,1880 +15974,1880 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>fishing_buy_rod</t>
+          <t>event_status</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>낚싯대 구매 (골드/다이아)</t>
+          <t>현재 활성 축제 조회</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>5등급 모두</t>
+          <t>이름/기간/버프/한정 보상</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>통합</t>
+          <t>API</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>lottery → server.js</t>
+          <t>/status JSON</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>require + 소켓 핸들러 3종</t>
+          <t>festival 필드 추가</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>첫 모듈 통합 마일스톤</t>
+          <t>대시보드 확인용</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.28</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>소켓 이벤트</t>
+          <t>NPC</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>lottery_status</t>
+          <t>축제 인사</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>상태/가격/상품 풀 조회</t>
+          <t>30% 확률로 NPC가 축제 대사 출력</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>클라이언트 표시용</t>
+          <t>spring_blossom 등 5종</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>소켓 이벤트</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>lottery_free_spin</t>
+          <t>fishing → server.js</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>매일 무료 1회 스핀</t>
+          <t>require + 소켓 핸들러 3종</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>자정 초기화</t>
+          <t>두 번째 모듈 통합</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>v1.26</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>소켓 이벤트</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>lottery_paid_spin</t>
+          <t>fishing_status</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>유료 1회 / 10연속</t>
+          <t>지역/낚싯대/미끼/시간대 조회</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>count: 1 또는 10</t>
+          <t>클라이언트 표시용</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>game/auction.js 신규</t>
+          <t>fishing_cast</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>입찰식 / 3기간 / 5% 인상 / 스나이핑 방지</t>
+          <t>낚시 시도 (지역+낚싯대+미끼 검증)</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>등록 2% + 낙찰 5%</t>
+          <t>전설/신화 → 서버 알림</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>v1.25</t>
+          <t>v1.27</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>경매장</t>
+          <t>소켓</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>활성 한도</t>
+          <t>fishing_buy_rod</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>플레이어당 10개</t>
+          <t>낚싯대 구매 (골드/다이아)</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>자기 입찰 금지</t>
+          <t>5등급 모두</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>game/fishing.js 신규</t>
+          <t>lottery → server.js</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>11종 어종 / 5등급 낚싯대 / 4종 미끼</t>
+          <t>require + 소켓 핸들러 3종</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>신화 크라켄 = 20000G + 칭호</t>
+          <t>첫 모듈 통합 마일스톤</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>v1.24</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>낚시</t>
+          <t>소켓 이벤트</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>전설의 비단잉어</t>
+          <t>lottery_status</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>드래곤 낚싯대 + 가중치 1</t>
+          <t>상태/가격/상품 풀 조회</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>5000G + 평생 행운 +5%</t>
+          <t>클라이언트 표시용</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>소켓 이벤트</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>game/boss_rush.js 신규</t>
+          <t>lottery_free_spin</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>20웨이브 / HP ×1.35 스케일링</t>
+          <t>매일 무료 1회 스핀</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>최종 보상: 200💎 + 용재료 ×5</t>
+          <t>자정 초기화</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.26</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>소켓 이벤트</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>입장</t>
+          <t>lottery_paid_spin</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>매일 무료 3회 / 1000G / 30💎</t>
+          <t>유료 1회 / 10연속</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>랭킹 시스템</t>
+          <t>count: 1 또는 10</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>v1.23</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>보스 러시</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>챔피언 보상</t>
+          <t>game/auction.js 신규</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>1위: 500💎 + 칭호 / 2위: 300💎 / 3위: 200💎</t>
+          <t>입찰식 / 3기간 / 5% 인상 / 스나이핑 방지</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>등록 2% + 낙찰 5%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.25</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>행운의 룰렛</t>
+          <t>경매장</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>game/lottery.js 신규</t>
+          <t>활성 한도</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>10종 보상 / 가중치 1000</t>
+          <t>플레이어당 10개</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>매일 무료 1회 + 유료</t>
+          <t>자기 입찰 금지</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>룰렛 (전설)</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>영웅 장비 상자</t>
+          <t>game/fishing.js 신규</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>확률 0.2% (가장 희귀)</t>
+          <t>11종 어종 / 5등급 낚싯대 / 4종 미끼</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>전설 보상</t>
+          <t>신화 크라켄 = 20000G + 칭호</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>v1.22</t>
+          <t>v1.24</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>룰렛 (전설)</t>
+          <t>낚시</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>200 다이아</t>
+          <t>전설의 비단잉어</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>확률 0.8%</t>
+          <t>드래곤 낚싯대 + 가중치 1</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>잭팟</t>
+          <t>5000G + 평생 행운 +5%</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>신년 축제</t>
+          <t>game/boss_rush.js 신규</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>1/1 ~ 1/7</t>
+          <t>20웨이브 / HP ×1.35 스케일링</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>골드 +50% / EXP +30%</t>
+          <t>최종 보상: 200💎 + 용재료 ×5</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>봄꽃 축제</t>
+          <t>입장</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>4/1 ~ 4/14</t>
+          <t>매일 무료 3회 / 1000G / 30💎</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>HP재생 +30% / 드롭 +20%</t>
+          <t>랭킹 시스템</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.23</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>보스 러시</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>한여름 밤의 축제</t>
+          <t>챔피언 보상</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>7/15 ~ 8/15</t>
+          <t>1위: 500💎 + 칭호 / 2위: 300💎 / 3위: 200💎</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>화염 +30% / PvP 보상 +50%</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>행운의 룰렛</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>할로윈 축제</t>
+          <t>game/lottery.js 신규</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>10/25 ~ 11/1</t>
+          <t>10종 보상 / 가중치 1000</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>크리 +10% / 언데드 +50%</t>
+          <t>매일 무료 1회 + 유료</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>v1.21</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>축제 이벤트</t>
+          <t>룰렛 (전설)</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>겨울 축제</t>
+          <t>영웅 장비 상자</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>12/20 ~ 12/31</t>
+          <t>확률 0.2% (가장 희귀)</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>골드 +30% / EXP +30% / 드롭 +30%</t>
+          <t>전설 보상</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.22</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>룰렛 (전설)</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>game/season.js 신규</t>
+          <t>200 다이아</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>15티어 / 30일 / 무료+프리미엄</t>
+          <t>확률 0.8%</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>만렙 보상: 태초 반지 + 시즌 칭호</t>
+          <t>잭팟</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>XP 획득 7종</t>
+          <t>신년 축제</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>퀘/보스/PvP/월드보스/던전/제작</t>
+          <t>1/1 ~ 1/7</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>일일 +200 ~ 월드보스 +500</t>
+          <t>골드 +50% / EXP +30%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>v1.20</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>시즌 패스</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>프리미엄 가격</t>
+          <t>봄꽃 축제</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>1500 다이아</t>
+          <t>4/1 ~ 4/14</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>시즌 당 1회</t>
+          <t>HP재생 +30% / 드롭 +20%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>Lv.40 달성</t>
+          <t>한여름 밤의 축제</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>각성기 해금 마일스톤</t>
+          <t>7/15 ~ 8/15</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>150💎</t>
+          <t>화염 +30% / PvP 보상 +50%</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Lv.50 달성</t>
+          <t>할로윈 축제</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>환생 가능 마일스톤</t>
+          <t>10/25 ~ 11/1</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>250💎</t>
+          <t>크리 +10% / 언데드 +50%</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.21</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>축제 이벤트</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>첫 환생</t>
+          <t>겨울 축제</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>prestige 1차</t>
+          <t>12/20 ~ 12/31</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>500💎</t>
+          <t>골드 +30% / EXP +30% / 드롭 +30%</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>첫 월드 보스</t>
+          <t>game/season.js 신규</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>월드 보스 처치 보너스</t>
+          <t>15티어 / 30일 / 무료+프리미엄</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>100💎</t>
+          <t>만렙 보상: 태초 반지 + 시즌 칭호</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>v1.19</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>무료 다이아</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>업적 50개</t>
+          <t>XP 획득 7종</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>업적 마일스톤</t>
+          <t>퀘/보스/PvP/월드보스/던전/제작</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>200💎</t>
+          <t>일일 +200 ~ 월드보스 +500</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.20</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>상점 (스킨)</t>
+          <t>시즌 패스</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>불사조 스킨</t>
+          <t>프리미엄 가격</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>1200 다이아</t>
+          <t>1500 다이아</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>불사조 깃털 이펙트 (영구)</t>
+          <t>시즌 당 1회</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>상점 (스킨)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>폭풍 스킨</t>
+          <t>Lv.40 달성</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>1200 다이아</t>
+          <t>각성기 해금 마일스톤</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t>번개 오라 이펙트 (영구)</t>
+          <t>150💎</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>상점 (편의)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>프리미엄 자동물약</t>
+          <t>Lv.50 달성</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>500 다이아</t>
+          <t>환생 가능 마일스톤</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>24시간 자동물약 무한</t>
+          <t>250💎</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>상점 (상자)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>프리미엄 보물 상자</t>
+          <t>첫 환생</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>300 다이아</t>
+          <t>prestige 1차</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
         <is>
-          <t>전설 장비 확정 + 다이아</t>
+          <t>500💎</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>v1.18</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>상점 (재료)</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>전설 재료 패키지</t>
+          <t>첫 월드 보스</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>600 다이아</t>
+          <t>월드 보스 처치 보너스</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>용재료×10 + 영혼석×20 + 마법재료×20</t>
+          <t>100💎</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.19</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>혈맹 Lv.6</t>
+          <t>무료 다이아</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>혈맹의 분노</t>
+          <t>업적 50개</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>크리티컬 +5%</t>
+          <t>업적 마일스톤</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t>60명 정원</t>
+          <t>200💎</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>혈맹 Lv.7</t>
+          <t>상점 (스킨)</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>혈맹의 신속</t>
+          <t>불사조 스킨</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>이동속도 +10%</t>
+          <t>1200 다이아</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>70명 정원</t>
+          <t>불사조 깃털 이펙트 (영구)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>혈맹 Lv.8</t>
+          <t>상점 (스킨)</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>혈맹의 회복</t>
+          <t>폭풍 스킨</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>HP 재생 +50%</t>
+          <t>1200 다이아</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t>80명 정원</t>
+          <t>번개 오라 이펙트 (영구)</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>혈맹 Lv.9</t>
+          <t>상점 (편의)</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>혈맹의 운명</t>
+          <t>프리미엄 자동물약</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>회피 +5%</t>
+          <t>500 다이아</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>90명 정원</t>
+          <t>24시간 자동물약 무한</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>v1.17</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>혈맹 Lv.10</t>
+          <t>상점 (상자)</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>혈맹의 전설</t>
+          <t>프리미엄 보물 상자</t>
         </is>
       </c>
       <c r="D59" s="8" t="inlineStr">
         <is>
-          <t>전 스탯 +5%</t>
+          <t>300 다이아</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t>100명 정원 — 최종</t>
+          <t>전설 장비 확정 + 다이아</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.18</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>상점 (재료)</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>점쟁이</t>
+          <t>전설 재료 패키지</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>운세 / 행운 버프 (밤·카르마 반응)</t>
+          <t>600 다이아</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>상황 대사 4종</t>
+          <t>용재료×10 + 영혼석×20 + 마법재료×20</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>혈맹 Lv.6</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>감정사</t>
+          <t>혈맹의 분노</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>미감정 장비 감정 (Lv.30+ 특수)</t>
+          <t>크리티컬 +5%</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t>상황 대사 4종</t>
+          <t>60명 정원</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>v1.16</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>신규 NPC</t>
+          <t>혈맹 Lv.7</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>수집가</t>
+          <t>혈맹의 신속</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>희귀 아이템 매입 (골드 50000+ 특별)</t>
+          <t>이동속도 +10%</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>상황 대사 4종</t>
+          <t>70명 정원</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>각성기 (어쌔신)</t>
+          <t>혈맹 Lv.8</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>천 개의 칼날</t>
+          <t>혈맹의 회복</t>
         </is>
       </c>
       <c r="D63" s="8" t="inlineStr">
         <is>
-          <t>3.5배 × 7타 / 광역 / 쿨150초</t>
+          <t>HP 재생 +50%</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>80명 정원</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>각성기 (워리어)</t>
+          <t>혈맹 Lv.9</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>대지 가르기</t>
+          <t>혈맹의 운명</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>6.0배 / 광역 5범위 / 스턴 2초</t>
+          <t>회피 +5%</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>90명 정원</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.17</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>각성기 (나이트)</t>
+          <t>혈맹 Lv.10</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>불멸의 수호자</t>
+          <t>혈맹의 전설</t>
         </is>
       </c>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>피해 90% 감소 / 도발 / 10초</t>
+          <t>전 스탯 +5%</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>100명 정원 — 최종</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>각성기 (메이지)</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>시간 정지</t>
+          <t>점쟁이</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>12.0배 / 광역 6범위 / 슬로우 90%</t>
+          <t>운세 / 행운 버프 (밤·카르마 반응)</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>상황 대사 4종</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>v1.15</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>각성기 (클레릭)</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>신의 은총</t>
+          <t>감정사</t>
         </is>
       </c>
       <c r="D67" s="8" t="inlineStr">
         <is>
-          <t>HP 100% 회복 / 전스탯 +50%</t>
+          <t>미감정 장비 감정 (Lv.30+ 특수)</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t>Lv.40</t>
+          <t>상황 대사 4종</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.16</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>신규 NPC</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>폭풍 정복자</t>
+          <t>수집가</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>폭풍의 거인 처치</t>
+          <t>희귀 아이템 매입 (골드 50000+ 특별)</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>10,000G + 150다이아</t>
+          <t>상황 대사 4종</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (어쌔신)</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>연금술사</t>
+          <t>천 개의 칼날</t>
         </is>
       </c>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>엘릭서 10회 제작</t>
+          <t>3.5배 × 7타 / 광역 / 쿨150초</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>5,000G + 80다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (워리어)</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>그림자 정복자</t>
+          <t>대지 가르기</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>그림자 미궁 클리어</t>
+          <t>6.0배 / 광역 5범위 / 스턴 2초</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>8,000G + 120다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (나이트)</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>전설의 동반자</t>
+          <t>불멸의 수호자</t>
         </is>
       </c>
       <c r="D71" s="8" t="inlineStr">
         <is>
-          <t>전설급 펫 진화</t>
+          <t>피해 90% 감소 / 도발 / 10초</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t>6,000G + 100다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
         <is>
-          <t>v1.14</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>업적</t>
+          <t>각성기 (메이지)</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>이국의 상인</t>
+          <t>시간 정지</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>사치품 교역 5회</t>
+          <t>12.0배 / 광역 6범위 / 슬로우 90%</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>4,000G + 60다이아</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.15</t>
         </is>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>월드 보스</t>
+          <t>각성기 (클레릭)</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>폭풍의 거인</t>
+          <t>신의 은총</t>
         </is>
       </c>
       <c r="D73" s="8" t="inlineStr">
         <is>
-          <t>HP 100,000 / ATK 140 / DEF 90</t>
+          <t>HP 100% 회복 / 전스탯 +50%</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t>EXP 10000 + 6000G</t>
+          <t>Lv.40</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>월드 보스</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>시간의 수호자</t>
+          <t>폭풍 정복자</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>HP 70,000 / ATK 170 / DEF 60</t>
+          <t>폭풍의 거인 처치</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>EXP 9000 + 7000G</t>
+          <t>10,000G + 150다이아</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t>v1.13</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>교역품</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t>불사조 깃털 / 공허의 정수 / 천공의 비단</t>
+          <t>연금술사</t>
         </is>
       </c>
       <c r="D75" s="8" t="inlineStr">
         <is>
-          <t>이국의 사치품 3종</t>
+          <t>엘릭서 10회 제작</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
         <is>
-          <t>기본가 600~900G</t>
+          <t>5,000G + 80다이아</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>타이탄의 엘릭서</t>
+          <t>그림자 정복자</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>용재료×3 + 마법재료×10</t>
+          <t>그림자 미궁 클리어</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>ATK ×1.5 / 30분</t>
+          <t>8,000G + 120다이아</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t>강철 엘릭서</t>
+          <t>전설의 동반자</t>
         </is>
       </c>
       <c r="D77" s="8" t="inlineStr">
         <is>
-          <t>철광석×30 + 마법재료×10</t>
+          <t>전설급 펫 진화</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
         <is>
-          <t>DEF ×1.5 / 30분</t>
+          <t>6,000G + 100다이아</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.14</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>업적</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>질풍 엘릭서</t>
+          <t>이국의 상인</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>약초×20 + 마법재료×8</t>
+          <t>사치품 교역 5회</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>SPD ×1.4 / 20분</t>
+          <t>4,000G + 60다이아</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>월드 보스</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>지혜 엘릭서</t>
+          <t>폭풍의 거인</t>
         </is>
       </c>
       <c r="D79" s="8" t="inlineStr">
         <is>
-          <t>마법수정×5 + 영혼재료×5</t>
+          <t>HP 100,000 / ATK 140 / DEF 90</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
         <is>
-          <t>EXP ×2.5 / 15분</t>
+          <t>EXP 10000 + 6000G</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
         <is>
-          <t>v1.12</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>연금술</t>
+          <t>월드 보스</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>행운 엘릭서</t>
+          <t>시간의 수호자</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>보석×10 + 마법재료×5</t>
+          <t>HP 70,000 / ATK 170 / DEF 60</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>GOLD ×2.0 / 15분</t>
+          <t>EXP 9000 + 7000G</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.13</t>
         </is>
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>신규 펫</t>
+          <t>교역품</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t>불사조 (pet_phoenix)</t>
+          <t>불사조 깃털 / 공허의 정수 / 천공의 비단</t>
         </is>
       </c>
       <c r="D81" s="8" t="inlineStr">
         <is>
-          <t>불꽃산 보스 50처치</t>
+          <t>이국의 사치품 3종</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr">
         <is>
-          <t>화염 DMG +20% (진화 +40%)</t>
+          <t>기본가 600~900G</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
-          <t>신규 펫</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>유니콘 (pet_unicorn)</t>
+          <t>타이탄의 엘릭서</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>다이아 800개</t>
+          <t>용재료×3 + 마법재료×10</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>회피 +10% (진화 +20%)</t>
+          <t>ATK ×1.5 / 30분</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t>v1.11</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
-          <t>신규 탈것</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t>페가수스 (mount_pegasus)</t>
+          <t>강철 엘릭서</t>
         </is>
       </c>
       <c r="D83" s="8" t="inlineStr">
         <is>
-          <t>다이아 1200개</t>
+          <t>철광석×30 + 마법재료×10</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
         <is>
-          <t>이동속도 +85% / 비행</t>
+          <t>DEF ×1.5 / 30분</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
         <is>
-          <t>신규 던전</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>그림자 미궁</t>
+          <t>질풍 엘릭서</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>Lv.38 / 8인 파티 / 7스테이지</t>
+          <t>약초×20 + 마법재료×8</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>22000G + 32000EXP</t>
+          <t>SPD ×1.4 / 20분</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t>v1.10</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B85" s="8" t="inlineStr">
         <is>
-          <t>드롭</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t>드래곤 검/망토/투구/장갑</t>
+          <t>지혜 엘릭서</t>
         </is>
       </c>
       <c r="D85" s="8" t="inlineStr">
         <is>
-          <t>그림자 미궁 보스 드롭</t>
+          <t>마법수정×5 + 영혼재료×5</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
         <is>
-          <t>전설급</t>
+          <t>EXP ×2.5 / 15분</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.12</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>연금술</t>
         </is>
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>공허의 방랑자</t>
+          <t>행운 엘릭서</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>몬스터 10,000 처치</t>
+          <t>보석×10 + 마법재료×5</t>
         </is>
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>ATK +7%</t>
+          <t>GOLD ×2.0 / 15분</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B87" s="8" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 펫</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t>불멸자</t>
+          <t>불사조 (pet_phoenix)</t>
         </is>
       </c>
       <c r="D87" s="8" t="inlineStr">
         <is>
-          <t>환생 5회</t>
+          <t>불꽃산 보스 50처치</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr">
         <is>
-          <t>EXP +25%</t>
+          <t>화염 DMG +20% (진화 +40%)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
         <is>
-          <t>전설 칭호</t>
+          <t>신규 펫</t>
         </is>
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>천공의 군주</t>
+          <t>유니콘 (pet_unicorn)</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>월드 보스 10회 처치</t>
+          <t>다이아 800개</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>보스DMG +15%</t>
+          <t>회피 +10% (진화 +20%)</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.11</t>
         </is>
       </c>
       <c r="B89" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>신규 탈것</t>
         </is>
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t>지역 시트 갱신</t>
+          <t>페가수스 (mount_pegasus)</t>
         </is>
       </c>
       <c r="D89" s="8" t="inlineStr">
         <is>
-          <t>25→51개 지역 반영</t>
+          <t>다이아 1200개</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>이동속도 +85% / 비행</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B90" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>신규 던전</t>
         </is>
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>칭호 시트 갱신</t>
+          <t>그림자 미궁</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>7→16종 + 효과/색상 추가</t>
+          <t>Lv.38 / 8인 파티 / 7스테이지</t>
         </is>
       </c>
       <c r="E90" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22000G + 32000EXP</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t>v1.9</t>
+          <t>v1.10</t>
         </is>
       </c>
       <c r="B91" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>드롭</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t>출석 캘린더 시트</t>
+          <t>드래곤 검/망토/투구/장갑</t>
         </is>
       </c>
       <c r="D91" s="8" t="inlineStr">
         <is>
-          <t>신규 추가 (28일 사이클)</t>
+          <t>그림자 미궁 보스 드롭</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>전설급</t>
         </is>
       </c>
     </row>
@@ -17749,22 +17859,22 @@
       </c>
       <c r="B92" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>장비 세트 시트</t>
+          <t>공허의 방랑자</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>신규 추가 (드래곤/영웅/태초)</t>
+          <t>몬스터 10,000 처치</t>
         </is>
       </c>
       <c r="E92" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ATK +7%</t>
         </is>
       </c>
     </row>
@@ -17776,22 +17886,22 @@
       </c>
       <c r="B93" s="8" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t>장비 등급 시트</t>
+          <t>불멸자</t>
         </is>
       </c>
       <c r="D93" s="8" t="inlineStr">
         <is>
-          <t>신규 추가 (5등급 + 랜덤 옵션 7종)</t>
+          <t>환생 5회</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>EXP +25%</t>
         </is>
       </c>
     </row>
@@ -17803,22 +17913,22 @@
       </c>
       <c r="B94" s="7" t="inlineStr">
         <is>
-          <t>기획서</t>
+          <t>전설 칭호</t>
         </is>
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>디버프 시트</t>
+          <t>천공의 군주</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>신규 추가 (10종, v1.7 5종 포함)</t>
+          <t>월드 보스 10회 처치</t>
         </is>
       </c>
       <c r="E94" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>보스DMG +15%</t>
         </is>
       </c>
     </row>
@@ -17835,12 +17945,12 @@
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t>패치 노트 시트</t>
+          <t>지역 시트 갱신</t>
         </is>
       </c>
       <c r="D95" s="8" t="inlineStr">
         <is>
-          <t>신규 추가 (히스토리)</t>
+          <t>25→51개 지역 반영</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
@@ -17852,25 +17962,187 @@
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
         <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B96" s="7" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C96" s="7" t="inlineStr">
+        <is>
+          <t>칭호 시트 갱신</t>
+        </is>
+      </c>
+      <c r="D96" s="7" t="inlineStr">
+        <is>
+          <t>7→16종 + 효과/색상 추가</t>
+        </is>
+      </c>
+      <c r="E96" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="8" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B97" s="8" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>출석 캘린더 시트</t>
+        </is>
+      </c>
+      <c r="D97" s="8" t="inlineStr">
+        <is>
+          <t>신규 추가 (28일 사이클)</t>
+        </is>
+      </c>
+      <c r="E97" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="7" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B98" s="7" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C98" s="7" t="inlineStr">
+        <is>
+          <t>장비 세트 시트</t>
+        </is>
+      </c>
+      <c r="D98" s="7" t="inlineStr">
+        <is>
+          <t>신규 추가 (드래곤/영웅/태초)</t>
+        </is>
+      </c>
+      <c r="E98" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="8" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B99" s="8" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C99" s="8" t="inlineStr">
+        <is>
+          <t>장비 등급 시트</t>
+        </is>
+      </c>
+      <c r="D99" s="8" t="inlineStr">
+        <is>
+          <t>신규 추가 (5등급 + 랜덤 옵션 7종)</t>
+        </is>
+      </c>
+      <c r="E99" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="7" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B100" s="7" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C100" s="7" t="inlineStr">
+        <is>
+          <t>디버프 시트</t>
+        </is>
+      </c>
+      <c r="D100" s="7" t="inlineStr">
+        <is>
+          <t>신규 추가 (10종, v1.7 5종 포함)</t>
+        </is>
+      </c>
+      <c r="E100" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="8" t="inlineStr">
+        <is>
+          <t>v1.9</t>
+        </is>
+      </c>
+      <c r="B101" s="8" t="inlineStr">
+        <is>
+          <t>기획서</t>
+        </is>
+      </c>
+      <c r="C101" s="8" t="inlineStr">
+        <is>
+          <t>패치 노트 시트</t>
+        </is>
+      </c>
+      <c r="D101" s="8" t="inlineStr">
+        <is>
+          <t>신규 추가 (히스토리)</t>
+        </is>
+      </c>
+      <c r="E101" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="7" t="inlineStr">
+        <is>
           <t>v1.10</t>
         </is>
       </c>
-      <c r="B96" s="7" t="inlineStr">
+      <c r="B102" s="7" t="inlineStr">
         <is>
           <t>기획서</t>
         </is>
       </c>
-      <c r="C96" s="7" t="inlineStr">
+      <c r="C102" s="7" t="inlineStr">
         <is>
           <t>던전 시트</t>
         </is>
       </c>
-      <c r="D96" s="7" t="inlineStr">
+      <c r="D102" s="7" t="inlineStr">
         <is>
           <t>신규 추가 (7종 던전)</t>
         </is>
       </c>
-      <c r="E96" s="7" t="inlineStr">
+      <c r="E102" s="7" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
feat: v2.20 — boss summon system (stones → creatures → evolution → boss)
New system: Boss Summon (game/boss_summon.js)
- 8 summon stones (4 elements + dark/light/void/primal)
- 11 summon creatures in 3 tiers
  T1: Fire Imp, Ice Golem, Wind Hawk, Earth Bear
  T2: Storm Drake, Lava Titan, Frost Fairy, Shadow Wolf
  T3: Void Serpent, Holy Angel, Primal Dragon
- Evolution: merge 2 same creatures → 1 evolved (up to 3★)
  Stats ×1.5 per evolution, skill ×1.3
- 4 summonable bosses (Inferno, Leviathan, Tempest, Apocalypse)
  Requires 3 active creatures of matching tier/element
  Apocalypse (80K HP) drops mythic weapon

Server integration:
- Monster kills drop summon stones (15% chance, weighted)
- boss_summon_handlers.js registered in connection.js
- _summons persisted in savePlayer/loadPlayer
- Excel planning doc: sheet 45 (보스 소환 시스템)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutoBattle_io_기획서.xlsx
+++ b/AutoBattle_io_기획서.xlsx
@@ -68,6 +68,7 @@
     <sheet name="혈맹 레이드 상세" sheetId="59" state="visible" r:id="rId59"/>
     <sheet name="무한의 탑 상세" sheetId="60" state="visible" r:id="rId60"/>
     <sheet name="차원 균열 상세" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet name="보스 소환 시스템" sheetId="62" state="visible" r:id="rId62"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -46159,6 +46160,964 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>보스 소환 시스템 (v2.20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>분류</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>이름</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>아이콘</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>재료/요구</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>스탯</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>효과/보상</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>소환석</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>stone_fire</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>화염 소환석</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>몬스터 드롭 15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>소환석</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>stone_water</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>수빙 소환석</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>🔵</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>몬스터 드롭 15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>소환석</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>stone_wind</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>질풍 소환석</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>몬스터 드롭 15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>소환석</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>stone_earth</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>대지 소환석</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>🟤</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>몬스터 드롭 15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>소환석</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>stone_dark</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>암흑 소환석</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>🟣</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>uncommon</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>몬스터 드롭 15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>소환석</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>stone_light</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>성광 소환석</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>uncommon</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>몬스터 드롭 15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>소환석</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>stone_void</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>공허 소환석</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>⚫</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>몬스터 드롭 15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>소환석</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>stone_primal</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>태초 소환석</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>💎</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>epic</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>몬스터 드롭 15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>T1 소환수</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>fire_imp</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>화염 임프</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>🔥</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>화염×3</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>ATK15/DEF5/HP200</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>화염구 (ATK×1.5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>T1 소환수</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>ice_golem</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>빙결 골렘</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>🧊</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>수빙×3</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>ATK8/DEF18/HP400</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>빙결 (3초 둔화)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>T1 소환수</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>wind_hawk</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>질풍 매</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>🦅</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>질풍×3</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>ATK20/DEF3/HP150</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>돌풍 (넉백)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>T1 소환수</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>earth_bear</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>대지 곰</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>🐻</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>대지×3</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>ATK12/DEF15/HP500</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>지진 (범위)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>T2 소환수</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>storm_drake</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>폭풍 드레이크</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>화염+질풍×2</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>ATK25/DEF10/HP350</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>번개 (ATK×2, 마비30%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>T2 소환수</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>lava_titan</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>용암 타이탄</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>🌋</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>화염×2+대지</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>ATK18/DEF22/HP600</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>분화 (범위 ATK×1.5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>T2 소환수</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>frost_fairy</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>서리 요정</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>❄️</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>수빙+성광+질풍</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>ATK12/DEF8/HP250</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>힐 (HP 20% 회복)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>T2 소환수</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>shadow_wolf</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>그림자 늑대</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>🐺</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>암흑×2+대지</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>ATK30/DEF6/HP280</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>기습 (ATK×3, 크리100%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>T3 소환수</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>void_serpent</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>공허의 뱀</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>🐍</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>공허+암흑×2</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>ATK35/DEF12/HP450</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>포식 (50% 흡혈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>T3 소환수</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>holy_angel</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>성스러운 천사</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>👼</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>성광×2+태초</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>ATK22/DEF20/HP500</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>신성 (범위 힐+공격)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>T3 소환수</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>primal_dragon</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>태초의 용</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>🐲</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>태초+공허+화염</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>ATK50/DEF25/HP800</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>브레스 (ATK×2.5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>보스</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>inferno</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>인페르노</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>🔥</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>T1 fire×3</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>HP15K/ATK120/DEF40</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>10K G, 8K EXP, 50D</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>보스</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>leviathan</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>레비아탄</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>🌊</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>T1 water×3</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>HP20K/ATK90/DEF60</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>12K G, 10K EXP, 60D</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>보스</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>tempest</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>템페스트</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>T2 any×3</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>HP30K/ATK150/DEF50</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>20K G, 15K EXP, 100D</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>보스</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>apocalypse</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>아포칼립스</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>💀</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>T3 any×3</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>HP80K/ATK250/DEF80</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>50K G, 40K EXP, 300D + 신화 무기</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>진화</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>동종 2마리 합성</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>1→2→3★</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>ATK/DEF/HP ×1.5</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>스킬 ×1.3</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>최대 3★</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>보관함 20마리</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat: v2.22 — PvP matchmaking system (1v1/3v3, ELO, seasons)
New system: PvP Matchmaking (game/pvp_matchmaking.js)
- Two modes: 1v1 (2 players) and 3v3 (6 players, team balanced)
- ELO rating system (default 1000, K-factor 32/24)
- Dynamic queue range: starts ±100, expands ±50 every 10s (max ±500)
- 7 tier ranks: Bronze → Silver → Gold → Platinum →
  Diamond → Master → Grand Master (ELO 2500+)

Match flow:
  Join queue → Auto-match every 5s → Teams balanced by ELO →
  Fight → Report result → ELO update + rewards + tier check

Rewards: Win 500G/10D (1v1), 800G/15D (3v3) + ELO gain
Season: 7-day cycles, auto-reset, top 100 leaderboard

Server integration:
- Game loop: tryMatch() every 5 seconds, season reset check
- pvp_match_handlers.js with 4 socket events
- ELO/match history persisted in savePlayer
- Excel planning doc: sheet 47

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutoBattle_io_기획서.xlsx
+++ b/AutoBattle_io_기획서.xlsx
@@ -70,6 +70,7 @@
     <sheet name="차원 균열 상세" sheetId="61" state="visible" r:id="rId61"/>
     <sheet name="보스 소환 시스템" sheetId="62" state="visible" r:id="rId62"/>
     <sheet name="날씨 던전 시스템" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet name="PvP 매칭 시스템" sheetId="64" state="visible" r:id="rId64"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47657,6 +47658,480 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>PvP 매칭 시스템 (v2.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>분류</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>인원/값</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>ELO/조건</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>승리 보상</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>패배 보상</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>모드</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>1v1</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>2명</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>ELO K=32</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>승: 500G, 300EXP, 10D</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>패: 150G, 90EXP</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>대기 60초</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>모드</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>3v3</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>6명</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>ELO K=24</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>승: 800G, 500EXP, 15D</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>패: 240G, 150EXP</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>대기 90초</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>ELO</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>기본 레이팅</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>매칭 범위 ±100~500</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>10초마다 ±50 확장</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>티어</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>🥉 브론즈</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>0+</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>시작 티어</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>티어</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>🥈 실버</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>1100+</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr"/>
+      <c r="E8" s="7" t="inlineStr"/>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>티어</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>🥇 골드</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>1300+</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr"/>
+      <c r="E9" s="8" t="inlineStr"/>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>티어</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>💎 플래티넘</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>1500+</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr"/>
+      <c r="E10" s="7" t="inlineStr"/>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>티어</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>💠 다이아몬드</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>1800+</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr"/>
+      <c r="E11" s="8" t="inlineStr"/>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>티어</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>👑 마스터</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>2100+</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr"/>
+      <c r="E12" s="7" t="inlineStr"/>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>티어</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>🌟 그랜드마스터</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>2500+</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>최상위 티어</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>시즌</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>주기</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>7일</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>자동 리셋</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>상위 100명 기록</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>매칭</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>서버 틱</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>5초마다</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>ELO 기반 자동 매칭</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>팀 ELO 균형 배분</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat: v2.23 — bounty hunter system (missions, traps, ranks)
New system: Bounty Hunter (game/bounty_hunter.js)
- 10 daily hunt missions (3 random per day):
  Easy/Normal/Hard/Extreme difficulty
  Zone-specific, tier-specific, weather/night conditions
  Rewards: 2K-15K gold, 1.5K-12K EXP, 10-80 diamonds

- 5 trap items (buy with gold, place in world):
  🪤 Snare (root 3s), ☠️ Poison (DoT 10s),
  💥 Flash (blind 2s), 🕸️ Net (slow 5s), 💣 Bomb (500 dmg)

- 5 hunter ranks (by mission clears):
  🏹 Apprentice → ⚔️ Skilled (+10 track) →
  🗡️ Veteran (+10% reward) → 🎯 Master (-20% trap cost) →
  👑 Legend (15% double reward)

Server integration:
- Monster kills auto-update hunt mission progress
  (zone, tier, weather, night conditions checked)
- Persistent state (_bountyHunter in savePlayer)
- Excel planning doc: sheet 48

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutoBattle_io_기획서.xlsx
+++ b/AutoBattle_io_기획서.xlsx
@@ -71,6 +71,7 @@
     <sheet name="보스 소환 시스템" sheetId="62" state="visible" r:id="rId62"/>
     <sheet name="날씨 던전 시스템" sheetId="63" state="visible" r:id="rId63"/>
     <sheet name="PvP 매칭 시스템" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet name="사냥꾼 시스템" sheetId="65" state="visible" r:id="rId65"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -48132,6 +48133,558 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>사냥꾼 시스템 (v2.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>분류</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>이름/등급</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>조건/효과</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>보상/가격</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>난이도/타입</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>일일 의뢰</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>늑대 떼 소탕</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>숲/normal 10마리</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>2K G, 1.5K EXP, 10D</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>매일 3개 갱신</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>일일 의뢰</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>산적 소굴 정리</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>산악/elite 8마리</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>4K G, 3K EXP, 20D</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>일일 의뢰</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>드래곤 알 수거</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>용둥지/수집 5개</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>8K G, 6K EXP, 40D</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>일일 의뢰</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>유령선 정벌</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>항구/rare 12마리</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>6K G, 5K EXP, 30D</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>일일 의뢰</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>공허 균열 봉인</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>심연/boss 6마리</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>15K G, 12K EXP, 80D</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>extreme</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>일일 의뢰</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>밤의 추적자</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>밤 전용 5마리</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>7K G, 5K EXP, 35D</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>isNight 조건</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>일일 의뢰</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>폭풍 짐승 사냥</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>폭풍 전용 4마리</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>12K G, 10K EXP, 60D</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>extreme</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>storm 조건</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>함정</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>🪤 올가미</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>3초 이동 불가</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>500G</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>root</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>함정</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>☠️ 독 함정</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>10초 독 DPS 5</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>800G</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>dot</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>함정</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>💥 섬광탄</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>2초 실명</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>600G</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>blind</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>함정</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>🕸️ 투망</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>5초 속도 -70%</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>700G</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>slow</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>함정</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>💣 폭탄</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>즉시 500 데미지</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1,200G</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>등급</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>🏹 견습 (0회)</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>기본</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>등급</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>⚔️ 숙련 (10회)</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>추적 범위 +10</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>등급</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>🗡️ 베테랑 (30회)</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>보상 +10%</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>등급</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>🎯 마스터 (60회)</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>함정 비용 -20%</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>등급</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>👑 전설 (100회)</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>15% 확률 보상 2배</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat: v2.24 — race system (4 races with skills & synergy)
New system: Race System (game/race_system.js)
- 4 playable races:
  🧑 Human — balanced, EXP +15%, all equip compatible
  🧝 Elf — agile, Crit +8%, Dodge +5%, MP regen
  ⛏️ Dwarf — tanky, DEF +10, HP +100, craft/enchant bonus
  😈 Demon — offensive, ATK +15, lifesteal 5% (unlock Lv.10)

- Unique active skills per race:
  Human: 💪 Will (all stats +20%, 10s)
  Elf: 🌿 Nature's Blessing (regen + debuff immune, 15s)
  Dwarf: 🛡️ Earth Shield (dmg -50% + knockback immune, 8s)
  Demon: 🔥 Demon Pact (HP -20%, ATK x2 + lifesteal, 12s)

- Per-level growth bonuses differ by race
- Race-specific titles at Lv.30/50
- Party synergy bonuses (2-race combos + 4-race ultimate)
- Race change on prestige only
- Excel planning doc: sheet 49

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutoBattle_io_기획서.xlsx
+++ b/AutoBattle_io_기획서.xlsx
@@ -72,6 +72,7 @@
     <sheet name="날씨 던전 시스템" sheetId="63" state="visible" r:id="rId63"/>
     <sheet name="PvP 매칭 시스템" sheetId="64" state="visible" r:id="rId64"/>
     <sheet name="사냥꾼 시스템" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet name="종족 시스템" sheetId="66" state="visible" r:id="rId66"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -48685,6 +48686,518 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>종족 시스템 (v2.24) — 4종족</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>종족/항목</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>해금/조건</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>패시브</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>성장 보너스</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>액티브 스킬</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>🧑 인간</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Lv.1</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>EXP +15%, 모든 장비 가능</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>HP+2/Lv, ATK+0.5/Lv, DEF+0.5/Lv</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>💪 인간의 의지: 10초 전 스탯 +20% (CD 120초)</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>균형형</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>🧝 엘프</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Lv.1</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Crit +8%, Dodge +5%, MP 리젠 +2%</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>HP+1/Lv, ATK+0.3/Lv, SPD+0.2/Lv</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>🌿 자연의 축복: 15초 HP 리젠 + 독/화상 면역 (CD 90초)</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>민첩/마법형</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>⛏️ 드워프</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Lv.1</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>DEF +10, HP +100, 제작 +15%, 강화 +10%</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>HP+4/Lv, DEF+1.0/Lv</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>🛡️ 대지의 방패: 8초 피해 50% 감소 + 넉백 면역 (CD 100초)</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>탱커/제작형</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>😈 악마</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Lv.10</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>ATK +15, 흡혈 5%, 카르마 감소 50%↓</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>ATK+1.0/Lv, HP+1.5/Lv</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>🔥 악마의 계약: HP 20% 소모 → 12초 ATK 2배 + 흡혈 15% (CD 150초)</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>공격형 (고위험)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>파티 시너지</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>인간+엘프</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>숲과 문명의 조화</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>EXP +10%</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>파티 시너지</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>인간+드워프</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>동맹의 힘</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>DEF +5, ATK +5</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>파티 시너지</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>엘프+드워프</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>고대의 약속</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>제작 +10%, Crit +3%</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>파티 시너지</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>악마+악마</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>어둠의 결속</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>ATK +10, 흡혈 +3%</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>파티 시너지</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>4종족 전부</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>종족 대연합</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>전체 스탯 +8, EXP +15%</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>최고 시너지</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>종족 칭호</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>인간 Lv.30</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>인류의 희망</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>EXP +5%</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>종족 칭호</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>엘프 Lv.30</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>숲의 수호자</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Dodge +3%</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>종족 칭호</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>드워프 Lv.30</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>대장장이의 후예</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>제작 +10%</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>종족 칭호</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>악마 Lv.30</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>심연의 아이</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>흡혈 +3%</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>변경</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>환생 시</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>종족 변경 가능</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>첫 선택 이후 환생으로만 변경</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat: v2.25 — relic fusion system (11 recipes, hidden combos)
New system: Relic Fusion (game/relic_fusion.js)
- 20 relic pool (10 existing + 10 new)
- 11 fusion recipes (3 relics → 1 powerful fused relic):
  Attack: Inferno Blade, Storm Reaver, Void Devourer
  Defense: Eternal Fortress, Holy Guardian
  Utility: Crown of Wisdom, Shadow Dancer
  Elemental: Phoenix Rebirth, Frost Emperor
  Hidden: Primordial God, Abyss Overlord (undisclosed recipes)

- Max 2 fused relics equipped simultaneously
- Recipe book: tracks discovered/crafted combinations
- Hidden combos announced server-wide on first discovery
- Effects include: on-hit procs, on-kill heals, auto-revive,
  freeze chance, chain lightning, party aura

Server integration:
- relic_fusion_handlers.js (fuse/equip/unequip/book)
- Persistent state (_relicFusion in savePlayer)
- Excel planning doc: sheet 50

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutoBattle_io_기획서.xlsx
+++ b/AutoBattle_io_기획서.xlsx
@@ -73,6 +73,7 @@
     <sheet name="PvP 매칭 시스템" sheetId="64" state="visible" r:id="rId64"/>
     <sheet name="사냥꾼 시스템" sheetId="65" state="visible" r:id="rId65"/>
     <sheet name="종족 시스템" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet name="유물 조합 시스템" sheetId="67" state="visible" r:id="rId67"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -49198,6 +49199,518 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>유물 조합 시스템 (v2.25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>계열</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>이름</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>재료 (유물 3개)</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>등급</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>효과</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>공격</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>⚔️🔥 인페르노 블레이드</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>혼돈칼날+화염핵+악마뿔</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>ATK+35, 크리뎀+30%, 10% 화염폭발</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>화염+혼돈 시너지</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>공격</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>⚡⚔️ 폭풍의 파괴자</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>번개송곳니+바람부츠+혼돈칼날</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>ATK+25, SPD+5, Crit+10%, 15% 연쇄번개</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>번개+바람</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>공격</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>🕳️⚔️ 공허의 포식자</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>공허파편+공허수정+악마뿔</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>mythic</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>ATK+50, 흡혈12%, 처치 시 HP 15% 회복</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>최강 공격</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>방어</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>🛡️✨ 영원의 요새</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>영원방패+대지뿌리+서리눈물</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>DEF+40, HP+300, 피감8%, HP30%↓ 무적5초</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>최강 방어</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>방어</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>👼🛡️ 성스러운 수호자</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>성수+천상깃털+영원방패</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>DEF+30, 힐+25%, 파티DEF+10, 사망 시 부활1회</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>서포터</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>유틸</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>👑📖 지혜의 왕관</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>왕관+고대두루마리+진실의눈</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>EXP+30%, 골드+20%, 스킬CD-15%</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>성장 특화</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>유틸</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>🌑💃 그림자 무용수</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>그림자진주+바람부츠+진실의눈</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Dodge+18%, SPD+8, Crit+8%, 회피 시 투명</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>회피 특화</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>원소</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>🔥🐦 불사조의 환생</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>불사조깃털+화염핵+성수</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>mythic</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>FireATK+40, Fire면역50%, 자동부활, 부활 시 폭발</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>불사</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>원소</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>❄️👑 서리 황제</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>서리눈물+왕관+대지뿌리</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>DEF+25, HP+200, 8% 빙결, 주변 속도-20%</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>빙결 컨트롤</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>히든</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>🌟💎 태초신의 유물</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>태초구슬+운명별+천상깃털</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>mythic</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>전체+20, EXP+50%, 골드+50%, 드롭+30%, 황금오라</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>??? 히든</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>히든</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>💀🔮 심연의 지배자</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>공허파편+악마뿔+그림자진주</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>mythic</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>ATK+45, 흡혈15%, Dark+40%, 처치 시 ATK+30%</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>??? 히든</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>설정</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>최대 장착</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>2개</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>동시 장착 가능</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>인벤토리에 보관</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>설정</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>유물 풀</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>20종</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>기존10 + 신규10</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>rare~mythic</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>조합 재료</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>설정</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>레시피</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>11종</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>공개9 + 히든2</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>발견 시 레시피북 등록</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>히든은 직접 실험</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
docs: add 9 missing system sheets to Excel planning doc
Added sheets for v2.27-v2.35 systems:
52. 도전 과제 100개 — 7카테고리, 5티어, 프로필 장식
53. 슈퍼 보스 — 3종 (크로노스/이그니시아/아자토스), 3페이즈
54. 전장 점령 — 8지역, 3진영, 5단계 강화
55. 소원 나무 — 4종 나무, 20종 열매, 계절 보너스
56. 영혼 시스템 — 14영혼 4티어, 합성/각성/공명
57. 시간 여행 던전 — 3시대 + 역설 보스
58. 신화 소환수 — 6신화, 4단계 각성, 2신화 보스
59. 고대 유적 탐험 — 10방 타입, 무한 층, 로그라이크
60. 세계 보스 연대기 — 3시즌, 주간 3단계

Excel total: 77 sheets (was 68)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutoBattle_io_기획서.xlsx
+++ b/AutoBattle_io_기획서.xlsx
@@ -75,6 +75,15 @@
     <sheet name="종족 시스템" sheetId="66" state="visible" r:id="rId66"/>
     <sheet name="유물 조합 시스템" sheetId="67" state="visible" r:id="rId67"/>
     <sheet name="스킬 웨이브 시스템" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet name="도전 과제 100" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet name="슈퍼 보스" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet name="전장 점령" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="소원 나무" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet name="영혼 시스템" sheetId="73" state="visible" r:id="rId73"/>
+    <sheet name="시간 여행 던전" sheetId="74" state="visible" r:id="rId74"/>
+    <sheet name="신화 소환수" sheetId="75" state="visible" r:id="rId75"/>
+    <sheet name="고대 유적 탐험" sheetId="76" state="visible" r:id="rId76"/>
+    <sheet name="세계 보스 연대기" sheetId="77" state="visible" r:id="rId77"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -50224,6 +50233,634 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>도전 과제 100개 (v2.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>카테고리</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>이름</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>목표 (5단계)</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>보상</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>배율</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>전투(20)</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>몬스터 처치</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>1/10/100/500/2000</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>골드+EXP</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>5단계 (브/실/골/플/다)</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>보상 1x~5x 배율</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>전투</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>엘리트 처치</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>1/5/20/50/200</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>골드+다이아</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr"/>
+      <c r="F5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>전투</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>보스 슬레이어</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>1/3/10/25/50</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>골드+다이아</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>전투</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>월드 보스 MVP</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>1/3/5/10/20</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>골드+다이아</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>최고난도</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>전투</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>스킬 웨이브</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>1/10/30/50/100</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>골드+EXP</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr"/>
+      <c r="F8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>성장(20)</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>레벨 달성</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>10/20/30/40/50</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>골드+EXP</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr"/>
+      <c r="F9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>성장</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>환생</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>1/2/3/5/10</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>다이아</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr"/>
+      <c r="F10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>성장</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>유물 조합</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>1/3/5/8/11</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>골드+다이아</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr"/>
+      <c r="F11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>성장</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>별자리 관측</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>1/4/8/12/12</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>골드+다이아</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr"/>
+      <c r="F12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>경제(10)</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>골드 누적</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>10K/100K/500K/1M/5M</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>골드</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr"/>
+      <c r="F13" s="8" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>경제</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>전설 낚시</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>1/2/3/5/10</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>골드+다이아</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>희귀</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>소셜(10)</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>혈맹 활동</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>가입</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>골드</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr"/>
+      <c r="F15" s="8" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>소셜</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>PvP 매칭</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>1/10/30/50/100</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>골드+다이아</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr"/>
+      <c r="F16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>생존(5)</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>화산 생존</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>60/180/300/600/1200초</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>골드+다이아</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr"/>
+      <c r="F17" s="8" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>수집(10)</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>히든 발견</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>1/3/5/8/12</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>골드+다이아</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr"/>
+      <c r="F18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>마스터(10)</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>만렙 달성</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>다이아 200</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr"/>
+      <c r="F19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>마스터</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>그랜드마스터</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>ELO 2500</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>다이아 500</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>최상위</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>특수(15)</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>도박 20연승</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>주사위</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>10K G + 100D</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>특수 조건</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>특수</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>신화 낚시</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>크라켄</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>20K G + 200D</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr"/>
+      <c r="F22" s="7" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>특수</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>#100 완벽한 전설</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>100개 전부 다이아</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>2000D + 무지개 오라</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>최종</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>프로필</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>프레임 5종</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>10/25/50/75/100개</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>브~레인보우</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>장식</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>프로필</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>오라 3종</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>30(전투)/30(수집)/100(전체)</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>화염/빙결/무지개</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>장식</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -50693,6 +51330,2785 @@
       <c r="F16" s="7" t="inlineStr">
         <is>
           <t>90%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>슈퍼 보스 (v2.28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>보스명</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>속성</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>ATK/DEF</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>MVP 보상</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>⏳ 크로노스</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>void</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>500K</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>300/100</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>P1: 시간 둔화 (속도-50%)</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>P2: 시간 역행 (5명 HP 복원)</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>P3: 시간 정지+운석500</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>50K G, 300D, 시간 무기</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>🐉 이그니시아</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>fire</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>600K</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>350/80</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>P1: 불의 비 (5곳 폭격)</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>P2: 용의 포효 (공포+DEF-30%)</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>P3: 불멸 불꽃 (1회 풀힐!)</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>60K G, 400D, 용 검</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>🕳️ 아자토스</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>void</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>800K</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>400/120</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>P1: 공허 침식 (MP 흡수)</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>P2: 차원 붕괴 (맵 축소)</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>P3: 현실 파괴 (HP↔MP!) ATK3배</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>80K G, 500D, 공허 오브</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>설정</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>스폰 시간</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>6/12/18/22시</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>5명+ 접속 시</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>10분 제한</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>기여도 3티어</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>MVP 전설 장비+칭호</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>전장 점령 시스템 (v2.29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>지역/설정</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>골드/비용</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>EXP/효과</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>방어/경비</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>특수</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>🏰 북부 전초</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>100G/주기</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>50 EXP</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>방어 0</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>기본 거점</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>점령 30초</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>🏰 남부 전초</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>100G/주기</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>50 EXP</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>방어 0</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>기본 거점</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>⛏️ 수정 광산</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>200G/주기</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>30 EXP</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>방어 0</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>수정 자원</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>⛏️ 철광석 광산</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>150G/주기</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>40 EXP</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>방어 0</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>철 자원</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>🐉 용의 요새</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>300G/주기</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>100 EXP</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>방어+20</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>핵심 거점</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>최고 수입</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>🕳️ 심연 요새</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>250G/주기</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>80 EXP</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>방어+15</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr"/>
+      <c r="F9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>🗼 마법사 탑</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>180G/주기</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>120 EXP</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>방어+10</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>EXP 특화</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>⛩️ 고대 제단</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>200G/주기</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>200 EXP</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>방어+5</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>축복 특수</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>강화 1단계</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>5,000G</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>DEF+10</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>경비 2명</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr"/>
+      <c r="F12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>강화 5단계</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>100,000G</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>DEF+50</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>경비 8명</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>최대</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>방어측 보너스</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>1.3배</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>전투력</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr"/>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>점령 진행 감소</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>☀️ 태양 기사단</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>공격 특화</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr"/>
+      <c r="D15" s="8" t="inlineStr"/>
+      <c r="E15" s="8" t="inlineStr"/>
+      <c r="F15" s="8" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>🌙 달빛 마법단</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>마법 특화</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr"/>
+      <c r="D16" s="7" t="inlineStr"/>
+      <c r="E16" s="7" t="inlineStr"/>
+      <c r="F16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>⭐ 별의 수호자</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>방어 특화</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr"/>
+      <c r="D17" s="8" t="inlineStr"/>
+      <c r="E17" s="8" t="inlineStr"/>
+      <c r="F17" s="8" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>소원 나무 시스템 (v2.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>나무/항목</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>타입/등급</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>열매/효과</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>계절/시간</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>🌳 세계수</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>균형</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>모든 열매</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>가을 1.5배</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>성장률 1.0</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>범용</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>🔥 화염수</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>공격</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>ATK/크리/화염</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>여름 1.5배</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>성장률 0.9</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>딜러</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>❄️ 서리수</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>방어</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>DEF/HP/빙결</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>겨울 1.5배</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>성장률 0.9</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>탱커</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>✨ 정령수</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>성장</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>EXP/지혜/행운</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>봄 1.5배</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>성장률 1.1</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>성장</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>열매(20종)</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>common 1-2h</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>🍊골드,🍇EXP,🍑회복</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr"/>
+      <c r="E8" s="7" t="inlineStr"/>
+      <c r="F8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr"/>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>uncommon 3-4h</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>🌶️힘,🥝수호,🍒크리,💎다이아</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr"/>
+      <c r="E9" s="8" t="inlineStr"/>
+      <c r="F9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr"/>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>rare 5-6h</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>🔥화염,🧊빙결,📖지혜,🍀행운</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr"/>
+      <c r="E10" s="7" t="inlineStr"/>
+      <c r="F10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr"/>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>legendary 24h</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>🌈무지개,☄️지옥불,💠절대영도,🌟깨달음</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr"/>
+      <c r="E11" s="8" t="inlineStr"/>
+      <c r="F11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>성장</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Lv.0→10</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>물 4시간마다</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>슬롯 3→6</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Lv.8+ 전설 5%</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>소원(500D)</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>💰부의</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>⚔️힘의</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>🛡️수호의</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>📖지혜의</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>🌟기적(전설10%)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>영혼 시스템 (v2.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>티어(드롭률)</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>이름</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>패시브</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>액티브 스킬</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>속성</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>T1(10%)</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>🟢슬라임</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>HP+20</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>earth</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>🐺늑대</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>ATK+3</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>wind</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>💀스켈레톤</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>DEF+3</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>dark</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>👹고블린</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>골드+3%</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>earth</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>T2(5%)</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>🐗오크</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>ATK+8,HP+30</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>전사의 함성 (ATK+20% 5초)</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>fire</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>액티브 보유</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>🦅하피</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>SPD+2,회피+3%</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>질풍 비행 (속도 3배 3초)</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>wind</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>🗿골렘</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>DEF+12,HP+50</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>석화 (4초 무적)</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>earth</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>🧙다크메이지</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>MP+20,EXP+5%</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>마력 폭발 (AoE x2)</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>dark</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>T3(1%)</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>🐲드래곤</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>ATK+20,화염+15%</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>용의 브레스 (AoE x3+화상)</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>fire</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>강력</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>☠️리치</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>흡혈8%,MP+50</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>죽음의 손길 (x5+50%흡수)</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>dark</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>🔥불사조</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>HP+150,자동부활</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>불사의 불꽃 (부활+폭발)</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>fire</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>🐋리바이어던</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>DEF+25,HP+200</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>해일 (범위 넉백+둔화)</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>water</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>T4(0.1%)</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>⏳크로노스</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>전체+8,CD-15%</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>시간 정지 (3초!)</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>void</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>전설</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>🕳️아자토스</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>ATK+30,흡혈10%</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>공허 삼키기 (20% 즉사)</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>void</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>최강</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>합성</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>같은 영혼 3개</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Lv+1 (최대 5)</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>스탯 +30%/레벨</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>2,000G</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>각성</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>T3+ 영혼</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>스탯 2배</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>mat_soul 10개 + 50KG</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr"/>
+      <c r="F19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>공명</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>같은 속성 2+</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>원소 보너스</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>3속성→원소 조화</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>T4×2→전설 공명</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>시간 여행 던전 (v2.32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>던전</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>요구 레벨</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>스테이지 (1→2→3)</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>클리어 보상</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>파편</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>🏛️ 고대</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Lv.25</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>안개+기습 → 석판 퍼즐 → 시간 파수꾼(HP 6K, 10초마다 힐10%)</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>10K G, 50D, 고대 봉인</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>과거 파편</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>1시간 쿨</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>🏙️ 현재</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Lv.35</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>컨베이어 → 원소 변환 → 시간 조율자(HP 10K, 가속 2배)</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>18K G, 80D, 시간 톱니</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>현재 파편</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>1시간 쿨</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>🚀 미래</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Lv.45</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>포탈 순간이동 → 면역 회전 → 오메가(HP 20K, 3시대 동시!)</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>30K G, 150D, 오메가 코어</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>미래 파편</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>1시간 쿨</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>⏳🌀 역설</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Lv.50</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>혼합 8마리 → 시간의 심장(HP 50K!, 즉사 존)</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>80K G, 500D, 시간 군주 세트+칭호</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>3파편 소모</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>3파편 필요</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>신화 소환수 (v2.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>소환수/항목</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>속성/단계</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>출처/요구</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>패시브/스탯</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>스킬 1 / 스킬 2</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>궁극기/보상</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>🐺 펜리르</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>dark</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>북유럽</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>ATK80,크리15%,흡혈8%</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>포식(x4+30%흡수) / 멸망의 울부짖음(AoE+공포)</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>라그나로크 (전체x6+불사+ATK3배)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>🐉 바하무트</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>fire</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>아라비아</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>ATK100,화염30%,화상20%</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>메가 플레어(범위8 x3) / 용신의 포효(버프/디버프)</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>테라 플레어 (전체x8+화면면역)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>🐋 레비아탄 신</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>water</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>히브리</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>DEF70,HP3500,빙결15%</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>심해 감옥(8초 CC) / 쓰나미(범위12 넉백)</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>심해의 심판 (전체 5초 익사!)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>👁️ 오딘</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>light</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>북유럽</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>EXP25%,크리10%,CD-20%</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>군그니르(관통x5 방무) / 지혜의 눈(전장 시야)</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>발할라 (전사5명+파티 불사)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>💀 타나토스</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>dark</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>그리스</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>흡혈12%,즉사&lt;20%</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>죽음의 낫(30%↓ 즉사) / 영혼 수확(ATK+15%)</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>죽음의 문 (HP50%삭감+부활불가)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>🌍 가이아</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>earth</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>그리스</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>HP4000,힐오라3%</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>대지의 축복(40%힐+해제) / 자연의 방벽(15초 방패)</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>생명의 기적 (전원 부활+30초 무적!)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>각성 4단계</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>⭐일반(1x)</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>⭐⭐각성(1.5x)</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐초월(2x)</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>🌟신격화(3x)</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>mat_soul/dragon/primal 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>신화 보스</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>🐍 요르문간드</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>HP 200K</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>펜리르+레비아탄</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>라그나로크 세트+칭호</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>신화 보스</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>🐉 티아마트</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>HP 300K</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>바하무트+타나토스</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>혼돈의 왕관+칭호</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>고대 유적 탐험 (v2.34)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>방 타입</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>확률/위치</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>내용</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>보상/효과</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>스케일</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>⬜ 빈 방</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>안전한 쉼터</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>👹 몬스터</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>전투 (층 스케일)</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>골드+EXP</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>HP=300×1.15^층</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>💰 보물</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>상자 (5등급)</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>1-4층 common ~ 30+층 legendary</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>⚠️ 함정</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>독침/화염/낙석/빙결/차원/저주</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>HP 데미지+디버프</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>6종 랜덤</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>🧩 퍼즐</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>순서/수수께끼/기억/전투</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>uncommon~epic 보상</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>성공률 60%</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>🏪 상인</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>횃불/열쇠/지도/탈출</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>골드 구매</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>5종 상품</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>⛩️ 제단</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>힐/ATK버프/EXP버프/저주/행운/맵공개</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>6종 랜덤</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr"/>
+      <c r="F10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>💀 보스</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>매 층 1개</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>층 수호자 (처치→출구)</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>3000×스케일 HP</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>층당 강해짐</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>🔮 비밀</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>3%</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>고급 보물 (rare~epic)</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>숨겨진 공간</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>열쇠 필요 가능</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>🚪 출구</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>매 층 1개</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>다음 층 (보스 처치 후)</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>무한 깊이</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr"/>
+      <c r="F13" s="8" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>무한 스케일</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>방 수: 8+1.5×층</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>몬스터: HP/ATK/DEF ×1.15^층</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>보물: 층↑ 등급↑</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr"/>
+      <c r="F14" s="7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>세계 보스 연대기 (v2.35)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>시즌</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>장</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>보스</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>기믹</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>보상</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>⚡🔥 라그나로크</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>제1장</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>🧊 흐림투르스</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>HP 150K</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>빙결 파도 (전체 3초 빙결)</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>8K G, 40D</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr"/>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>제2장</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>🔥 수르트</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>HP 250K</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>맵 절반 화염 즉사 존</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>15K G, 80D</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr"/>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>최종장</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>🐍 요르문간드</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>HP 500K</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>해일+독+분노(ATK3배)</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>30K G, 200D, 전설 무기+칭호</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>⚡🏛️ 올림포스</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>제1장</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>🔱 포세이돈</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>HP 180K</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>소용돌이 즉사</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>10K G, 50D</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr"/>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>제2장</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>⚔️ 아레스</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>HP 300K</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>전쟁 광기 (아군 PvP 강제!)</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>18K G, 100D</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr"/>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>최종장</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>⚡ 제우스</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>HP 600K</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>DPS 1위 즉사 번개!</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>40K G, 300D, 아이기스+칭호</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>🐲🌸 동방</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>제1장</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>🦊 구미호</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>HP 120K</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>5명 매혹 (아군 공격!)</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>7K G, 35D</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr"/>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>제2장</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>🐲 용왕</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>HP 280K</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>맵 수중 변환 (속도-50%)</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>16K G, 90D</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr"/>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>최종장</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>☯️ 혼돈</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>HP 700K</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>속성 반전 (잘못 치면 힐!)</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>50K G, 350D, 동방 왕관+칭호</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>설정</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>3시즌 회전</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>주간 리셋</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1→2→3 순차</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>MVP 3배 보상</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>전 서버 협동</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update planning Excel to v2.57 (103 sheets)
Added 7 new sheets:
- 드래곤 라이딩 (8 dragons, stats, breath, passives, rarity)
- 드래곤 성장 & 스킬 (6 stages, 4 foods, 5 flight skills, bond system)
- 드래곤 레이드 (3 bosses: Jormungandr, Bahamut, Nidhogg)
- v2.37~v2.57 패치노트 (features + 15 bug fixes + debug system)
- 시스템 시너지 맵 (12 cross-system interactions documented)
- 기술 아키텍처 (server/client/deploy stack overview)

Updated game version in overview to v2.57.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutoBattle_io_기획서.xlsx
+++ b/AutoBattle_io_기획서.xlsx
@@ -104,6 +104,12 @@
     <sheet name="살아있는 마도서" sheetId="95" state="visible" r:id="rId95"/>
     <sheet name="세계의 씨앗" sheetId="96" state="visible" r:id="rId96"/>
     <sheet name="운명의 직공" sheetId="97" state="visible" r:id="rId97"/>
+    <sheet name="드래곤 라이딩" sheetId="98" state="visible" r:id="rId98"/>
+    <sheet name="드래곤 성장 &amp; 스킬" sheetId="99" state="visible" r:id="rId99"/>
+    <sheet name="드래곤 레이드" sheetId="100" state="visible" r:id="rId100"/>
+    <sheet name="v2.37~v2.57 패치노트" sheetId="101" state="visible" r:id="rId101"/>
+    <sheet name="시스템 시너지" sheetId="102" state="visible" r:id="rId102"/>
+    <sheet name="기술 아키텍처" sheetId="103" state="visible" r:id="rId103"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -704,7 +710,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>v1.9 (전설 칭호 3종 추가)</t>
+          <t>v2.57 (드래곤 라이딩 + 판타지 UI + 디버그 시스템)</t>
         </is>
       </c>
     </row>
@@ -1554,6 +1560,1601 @@
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet100.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>드래곤 레이드 보스</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>보스ID</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>이름</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>아이콘</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>ATK</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>DEF</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>기믹</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>보상</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>필요 드래곤 수</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>특수 드롭</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>드롭 효과</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>ancient_wyrm</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>태고의 대사 요르문간드</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>🐍</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>800</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>독 안개(전체DOT), 꼬리 휩쓸기(넉백), 삼킴(즉사판정)</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>50,000G + 차원석20</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>3마리 이상</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>요르문간드의 비늘 갑옷</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>DEF+80, HP+300, 독저항+50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>sky_titan</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>하늘의 왕 바하무트</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>👑</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>800000</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>메가 플레어(카운트다운 전체), 차원 이동(페이즈), 브레스 반사</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>100,000G + 차원석40</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>5마리 이상</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>바하무트의 날개</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>SPD+10, ATK+50, 전체데미지+15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>void_dragon</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>차원포식자 니드호그</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>🕳️</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>차원 붕괴(맵축소), 존재 삭제(HP비율), 공허 폭발(패턴회피)</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>200,000G + 차원석80</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>7종 전원</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>니드호그의 이빨</t>
+        </is>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>ATK+100, 크리티컬 데미지+30%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet101.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>v2.37 ~ v2.57 패치노트 &amp; 버그 수정</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>버전</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>제목</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>주요 변경사항</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>영향 범위</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>v2.37</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>마법 연구소</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>마법 연구 20종, 스킬 합성 4종, 마법서 시스템</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>game/magic_lab.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>v2.38~v2.56</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>19개 판타지 시스템</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>달빛 성역, 무기 영혼, 부유 요새, 영체 이탈, 저주 던전, 운명의 결투, 영혼 대장간, 환영 투기장, 꿈의 건축가, 별자리 전쟁, 금서의 도서관, 거수 합체, 상인 캐러밴, 기억 궁전, 마왕의 옥좌, 천상 대장간, 살아있는 마도서, 세계의 씨앗, 운명의 직공</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>game/*.js + handlers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>v2.57</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>드래곤 라이딩</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>8종 드래곤 (화/빙/뇌/암/광/지/공/혼), 6단계 성장, 비행 전투, 브레스/스킬, 레이드 보스 3종</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>game/dragon_riding.js + handlers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>v2.57</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>UI 판타지 테마</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Cinzel 판타지 폰트, 마법진 로딩 애니메이션, 아케인 글로우, 파티클 이펙트</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>public/css/style.css + index.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>v2.57</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>보너스 집계 연동</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>드래곤 탑승 패시브 → bonus_aggregator 연동, 성장 단계 비례</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>game/bonus_aggregator.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>v2.57</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>NPC 대화 확장</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>드래곤 탑승 시 NPC 반응 대사, 7종 마스터 특별 대사</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>game/world.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr"/>
+      <c r="B10" s="7" t="inlineStr"/>
+      <c r="C10" s="7" t="inlineStr"/>
+      <c r="D10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8">
+        <f>== 서버 안정화 (버그 수정) ===</f>
+        <v/>
+      </c>
+      <c r="B11" s="8" t="inlineStr"/>
+      <c r="C11" s="8" t="inlineStr"/>
+      <c r="D11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>v2.57-fix</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>playerId 미정의</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>sub-connection 핸들러에 playerId 주입 ($ctx)</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>game/handlers/connection.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>v2.57-fix</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>io 미정의</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>$ctx에 io 주입 (채팅/broadcast 복구)</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>game/handlers/connection.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>v2.57-fix</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>TERRAIN_BARRIERS 미정의</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>core_connection destructure에 추가</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>game/handlers/core_connection.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>v2.57-fix</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>registerLotteryHandlers 크래시</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>inventory_connection.js 중복 핸들러 207줄 제거</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>game/handlers/inventory_connection.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>v2.57-fix</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>giveExp(owner) 버그</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>봇 킬 시 경험치가 봇에게 → realOwner로 수정</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>game/loops.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>v2.57-fix</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>entityIdCounter undefined</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>$.nextEntityId() 함수 사용으로 교체 (6곳)</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>game/loops.js + handlers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>v2.57-fix</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>worldBoss const 재할당</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>$.setWorldBoss(null)로 변경</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>game/loops.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>v2.57-fix</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>투사체 이동 누락</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>handleCollisions에 서버 측 투사체 위치 업데이트 추가</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>game/loops.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>v2.57-fix</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>monsterDelta null → Unity 크래시</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>삭제 몬스터를 removedMonsters[] 배열로 분리</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>game/loops.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>v2.57-fix</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>minimap null 에러</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>null 몬스터 건너뛰기 + delta merge 방식 변경</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>public/js/minimap.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>v2.57-fix</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>서브메뉴 JS 코드 노출</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>innerHTML+onclick → createElement+addEventListener</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>public/js/effects.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>v2.57-fix</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>한글 폰트 깨짐</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Cinzel 한글 fallback Noto Sans KR 추가</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>public/css/style.css + index.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>v2.57-fix</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>savePlayer/getExpRequired 미정의</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>handleCollisions에 $.savePlayer, $.getExpRequired 추가</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>game/loops.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr"/>
+      <c r="B25" s="8" t="inlineStr"/>
+      <c r="C25" s="8" t="inlineStr"/>
+      <c r="D25" s="8" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7">
+        <f>== 디버그 시스템 ===</f>
+        <v/>
+      </c>
+      <c r="B26" s="7" t="inlineStr"/>
+      <c r="C26" s="7" t="inlineStr"/>
+      <c r="D26" s="7" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>v2.57</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>서버 로그 링 버퍼</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>console.log/error/warn 200줄 캡처, GET /debug/logs</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>server.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>v2.57</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>클라이언트 에러 수집</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>window.onerror → POST /debug/client-error → 오버레이</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>public/index.html + server.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>v2.57</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>크래시 핸들러</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>unhandledRejection + uncaughtException 로깅</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>server.js</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet102.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>시스템 간 시너지 맵</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>시스템 A</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>시스템 B</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>시너지 내용</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>효과</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>구현 파일</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>드래곤 라이딩</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>보너스 집계</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>드래곤 탑승 시 패시브 → 보너스 집계에 표시</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>속성 데미지, 회피, 흡혈 등</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>bonus_aggregator.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>드래곤 라이딩</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>NPC 대화</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>드래곤 탑승 시 NPC 특수 대사</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>대장장이/힐러/상점 반응</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>world.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>혈통</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>PvP</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>혈통 상성: 용&gt;정령&gt;천사&gt;악마&gt;용</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>상성 유리 시 데미지 +20%</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>bloodline.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>별자리</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>계절</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>현재 계절 별자리 = 전투력 1.5배</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>봄(양/처녀), 여름(사자/전갈) 등</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>constellation.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>무기 영혼</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>몬스터 처치</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>영혼 각인 시 해당 몬스터 스킬 획득</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>키메라 무기(2영혼 합성)</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>weapon_soul.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>저주 던전</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>저주 장비</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>던전 저주+장비 저주 시너지</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>예: 유리몸+피의저주 = 광전사</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>cursed_dungeon.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>살아있는 마도서</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>금서 도서관</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>마도서 숙련도 → 금서 시전 대가 감소</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>최대 30% 대가 감소</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>living_grimoire.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>꿈의 건축가</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>기억 궁전</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>자신의 기억을 던전으로 재현</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>악몽 난이도 보상 2.5배</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>dream_architect.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>영혼 계약</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>보스 소환</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>보스 영혼 파편 → 계약 → 소환수</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>소환수 레벨업 가능</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>soul_contract.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>고대 언어</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>마법 연구소</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>6문자 조합 커스텀 마법</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>4문자 궁극 주문 "창세의 빛"</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>ancient_language.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>운명의 직공</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>PvP</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>저주 실 사용 시 카르마 감소</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>반작용: 시전자에게도 디버프</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>fate_weaver.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>환생</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>기억 궁전</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>전생 기억 → 던전화</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>같은 클래스 환생 시 기억 중첩 (최대 x2.5)</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>past_life.js</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet103.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>기술 아키텍처</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>설명</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>파일 경로</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>서버</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Node.js + Express</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>게임 서버 + 정적 파일 서빙</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>server.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>서버</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Socket.IO</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>실시간 양방향 통신</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>server.js + handlers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>서버</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>MySQL (Railway)</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>플레이어 저장, 우편함</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>server/db.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>서버</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>게임 루프</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>33ms 틱 (30fps): 이동/충돌/AI/스킬</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>game/loops.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>서버</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>핸들러 구조</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>connection.js → 6개 sub-connection + 100+ 모듈 핸들러</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>game/handlers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>서버</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>디버그</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>GET /debug/logs, /debug/client-errors, /status</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>server.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr"/>
+      <c r="B10" s="7" t="inlineStr"/>
+      <c r="C10" s="7" t="inlineStr"/>
+      <c r="D10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>클라이언트</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Unity WebGL</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>3D 렌더링, 캐릭터/몬스터 표시</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Assets/Script/GameManager.cs</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>클라이언트</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>HTML UI</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>메뉴, 인벤토리, 상점, 채팅, 미니맵</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>public/index.html + js/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>클라이언트</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>CSS</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>다크 판타지 테마 (Cinzel + Noto Sans KR)</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>public/css/style.css</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr"/>
+      <c r="B14" s="7" t="inlineStr"/>
+      <c r="C14" s="7" t="inlineStr"/>
+      <c r="D14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>배포</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Railway</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>자동 배포 (git push → build → deploy)</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>package.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>배포</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>MySQL</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Railway MySQL 플러그인 (${{MySQL.MYSQL_URL}})</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>환경변수</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>배포</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>도메인</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>baduk-marble-production.up.railway.app</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Railway 설정</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr"/>
+      <c r="B18" s="7" t="inlineStr"/>
+      <c r="C18" s="7" t="inlineStr"/>
+      <c r="D18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>모듈 수</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>게임 모듈</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>140+ .js 파일</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>game/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>모듈 수</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>소켓 핸들러</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>118+ handler 파일</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>game/handlers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>모듈 수</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>데이터 모듈</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>6개 (zones, equipment, quests, economy, world_data, server_data)</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>game/data/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -72130,4 +73731,1215 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet98.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>드래곤 라이딩 시스템 (v2.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>드래곤ID</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>이름</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>아이콘</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>속성</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>ATK</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>DEF</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>SPD</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>브레스</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>패시브</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>레어도</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>알 획득 방법</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>드롭률</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>fire</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>화염룡 이그니스</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>🔥</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>화(火)</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>800</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>화염 브레스 (ATK×3 화염)</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>화 속성 데미지 +30%</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>용의 둥지 (화산 지역) 보스</t>
+        </is>
+      </c>
+      <c r="M4" s="7" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>ice</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>빙결룡 프로스트</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>❄️</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>빙(氷)</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>900</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>냉기 브레스 (동결3초+ATK×2)</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>빙 저항+50%, 적 이속-20%</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
+        <is>
+          <t>빙하 동굴 보스</t>
+        </is>
+      </c>
+      <c r="M5" s="8" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>thunder</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>뇌전룡 볼텍스</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>뇌(雷)</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>700</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>140</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>뇌전 브레스 (랜덤3체 ATK×2.5)</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>공속+40%, 크리+15%</t>
+        </is>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>뇌운 봉우리 보스</t>
+        </is>
+      </c>
+      <c r="M6" s="7" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>shadow</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>암흑룡 네크로스</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>🌑</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>암(暗)</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>850</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>110</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>암흑 브레스 (HP흡수 ATK×2+공포2초)</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>암 속성+25%, 흡혈+10%</t>
+        </is>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="L7" s="8" t="inlineStr">
+        <is>
+          <t>암흑 심연 보스</t>
+        </is>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>holy</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>성룡 아우렐리우스</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>✨</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>광(光)</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>성광 브레스 (ATK×2 광역+아군HP15%회복)</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>광 속성+20%, 자동회복3%/초</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>천상 신전 보스</t>
+        </is>
+      </c>
+      <c r="M8" s="7" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>earth</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>대지룡 테라</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>🌍</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>지(地)</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>지진 브레스 (주변 ATK×2+스턴2초)</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>DEF+40%, 넉백 면역</t>
+        </is>
+      </c>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="L9" s="8" t="inlineStr">
+        <is>
+          <t>대지의 심장 보스</t>
+        </is>
+      </c>
+      <c r="M9" s="8" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>void</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>공허룡 아비스</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>🕳️</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>공허</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>750</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>160</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>공허 브레스 (현재HP 20% 삭제)</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>전속성 저항+15%, 회피+10%</t>
+        </is>
+      </c>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>Legendary</t>
+        </is>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>차원의 틈 보스 (Lv.40+)</t>
+        </is>
+      </c>
+      <c r="M10" s="7" t="inlineStr">
+        <is>
+          <t>3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>chaos</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>혼돈룡 카오스</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>🌀</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>혼돈</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>혼돈 브레스 (랜덤속성 ATK×4+랜덤 버프/디버프)</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>전체 스탯+15%, 매10초 랜덤 강력 버프</t>
+        </is>
+      </c>
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>Mythic</t>
+        </is>
+      </c>
+      <c r="L11" s="8" t="inlineStr">
+        <is>
+          <t>7종 드래곤 만렙 달성 보상</t>
+        </is>
+      </c>
+      <c r="M11" s="8" t="inlineStr">
+        <is>
+          <t>자동 해금</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet99.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>드래곤 성장 &amp; 비행 스킬 상세</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>단계명</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>아이콘</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>필요 레벨</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>필요 먹이 횟수</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>스탯 배율</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>설명</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7">
+        <f>== 성장 단계 (6단계) ===</f>
+        <v/>
+      </c>
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>알</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>🥚</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>0x</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>부화를 기다리는 알</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>해츨링</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>🐣</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>0.3x</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>갓 태어난 아기 용</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>유룡</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>🐉</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>0.5x</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>날개가 자라기 시작 — 탑승 가능!</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>성룡</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>🐲</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>0.8x</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>하늘을 나는 성체 용</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>고대룡</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>👑</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>1.0x</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>수천 년을 살아온 고대의 존재</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>신룡</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>⭐</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>1.5x</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>신의 영역에 도달한 전설의 용</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr"/>
+      <c r="B11" s="8" t="inlineStr"/>
+      <c r="C11" s="8" t="inlineStr"/>
+      <c r="D11" s="8" t="inlineStr"/>
+      <c r="E11" s="8" t="inlineStr"/>
+      <c r="F11" s="8" t="inlineStr"/>
+      <c r="G11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7">
+        <f>== 먹이 아이템 ===</f>
+        <v/>
+      </c>
+      <c r="B12" s="7" t="inlineStr"/>
+      <c r="C12" s="7" t="inlineStr"/>
+      <c r="D12" s="7" t="inlineStr"/>
+      <c r="E12" s="7" t="inlineStr"/>
+      <c r="F12" s="7" t="inlineStr"/>
+      <c r="G12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>dragon_meat</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>용의 고기</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr"/>
+      <c r="D13" s="8" t="inlineStr"/>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>EXP 50</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>500G</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>기본 먹이</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>dragon_crystal</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>마력 결정</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr"/>
+      <c r="D14" s="7" t="inlineStr"/>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>EXP 150</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>2,000G</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>마력이 응축된 결정</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>dragon_heart</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>드래곤 하트</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr"/>
+      <c r="D15" s="8" t="inlineStr"/>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>EXP 500</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>10,000G</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>보스 드래곤의 심장</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>dragon_stardust</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>별의 먹지</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr"/>
+      <c r="D16" s="7" t="inlineStr"/>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>EXP 1,000</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>이벤트/레이드</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>최상급 먹이</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr"/>
+      <c r="B17" s="8" t="inlineStr"/>
+      <c r="C17" s="8" t="inlineStr"/>
+      <c r="D17" s="8" t="inlineStr"/>
+      <c r="E17" s="8" t="inlineStr"/>
+      <c r="F17" s="8" t="inlineStr"/>
+      <c r="G17" s="8" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7">
+        <f>== 비행 스킬 (탑승 시 사용) ===</f>
+        <v/>
+      </c>
+      <c r="B18" s="7" t="inlineStr"/>
+      <c r="C18" s="7" t="inlineStr"/>
+      <c r="D18" s="7" t="inlineStr"/>
+      <c r="E18" s="7" t="inlineStr"/>
+      <c r="F18" s="7" t="inlineStr"/>
+      <c r="G18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>divebomb</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>급강하 폭격</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr"/>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>유룡(2단계)</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>쿨 15초</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>ATK×5 단일+스턴2초</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>wingblade</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>날개 칼바람</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr"/>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>해츨링(1단계)</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>쿨 10초</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>주변 ATK×2 광역</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>skydance</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>하늘춤</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr"/>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>성룡(3단계)</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>쿨 20초</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>5초 무적+회피100%</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>dragonroar</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>용의 포효</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr"/>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>고대룡(4단계)</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>쿨 30초</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>적 전원 공포3초+DEF-30%</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>dracosurge</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>드래곤 서지</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr"/>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>신룡(5단계)</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>쿨 60초</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>30초간 스탯2배+브레스 강화</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr"/>
+      <c r="B24" s="7" t="inlineStr"/>
+      <c r="C24" s="7" t="inlineStr"/>
+      <c r="D24" s="7" t="inlineStr"/>
+      <c r="E24" s="7" t="inlineStr"/>
+      <c r="F24" s="7" t="inlineStr"/>
+      <c r="G24" s="7" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8">
+        <f>== 친밀도 ===</f>
+        <v/>
+      </c>
+      <c r="B25" s="8" t="inlineStr"/>
+      <c r="C25" s="8" t="inlineStr"/>
+      <c r="D25" s="8" t="inlineStr"/>
+      <c r="E25" s="8" t="inlineStr"/>
+      <c r="F25" s="8" t="inlineStr"/>
+      <c r="G25" s="8" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>시스템</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>먹이 1회당 +1 (최대 100)</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr"/>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>친밀도 50+시 allStats 보너스</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr"/>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>보너스 = (친밀도-50) × 0.001</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>레벨업 시 스탯 × (1 + 레벨×0.03) × (1 + 친밀도×0.002)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs+ui: 기획서 135시트 최종 + SLG UI 폴리싱
## 기획서 135시트 (최종)
- 전체 용병 목록 42종 (16종 추가 반영)
- 공성전 맵 v3.0 (25×20, 5레인, 특수지형)
- 전체 이벤트 11종 시트
- 전체 무역 루트 10개 시트

## SLG UI 폴리싱
- 용병 카드 디자인 (등급 테두리+글로우)
- 파티 편성 시각화 (아이콘+별+레벨)
- 등급별 필터 탭 (전체/신화/전설/...)
- 전투력 강조 표시
- 무역 루트 카드 (이윤율/위험도 컬러)
- merc-card, trade-route CSS 컴포넌트

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AutoBattle_io_기획서.xlsx
+++ b/AutoBattle_io_기획서.xlsx
@@ -138,8 +138,10 @@
     <sheet name="SLG 뷰 진급 진화" sheetId="129" state="visible" r:id="rId129"/>
     <sheet name="공성전 배치 상세" sheetId="130" state="visible" r:id="rId130"/>
     <sheet name="공성전 IO 전투" sheetId="131" state="visible" r:id="rId131"/>
-    <sheet name="무역 시스템 구현" sheetId="132" state="visible" r:id="rId132"/>
-    <sheet name="전체 용병 목록 v3" sheetId="133" state="visible" r:id="rId133"/>
+    <sheet name="전체 이벤트 목록" sheetId="132" state="visible" r:id="rId132"/>
+    <sheet name="전체 무역 루트" sheetId="133" state="visible" r:id="rId133"/>
+    <sheet name="무역 시스템 구현" sheetId="134" state="visible" r:id="rId134"/>
+    <sheet name="전체 용병 목록 v3" sheetId="135" state="visible" r:id="rId135"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -12962,7 +12964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13230,6 +13232,147 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr"/>
+      <c r="B20" s="8" t="inlineStr"/>
+      <c r="C20" s="8" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>v3.0 맵</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>크기</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>25×20 그리드, 5레인</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>v3.0 맵</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>벽 5개</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>우회 필요한 장애물</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>v3.0 맵</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>회복 지대</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>HP 자동 회복 구역</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>v3.0 맵</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>감속 지대</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>이동속도 감소 구역</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>v3.0 맵</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>시야 차단</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>어둠 속 이동</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>v3.0 함정</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>감속 덫 🕸️</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>이동 -50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>v3.0 함정</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>텔레포트 🌀</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>시작점 강제 이동</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>v3.0 함정</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>소환 👹</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>해골 3체 소환</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
@@ -13239,6 +13382,852 @@
 </file>
 
 <file path=xl/worksheets/sheet132.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>전체 이벤트 목록 (11종)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>이벤트</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>아이콘</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>주기</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>효과</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>용병 대회</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>🏟️</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>1시간</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>용병 토너먼트, 1위 20000G+100💎</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>무역 축제</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>💰</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>2시간</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>교역 이윤 2배</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>공성 시즌</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>🏰</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>4시간</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>공성 보상 3배</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>용병 모집</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>🎴</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>3시간</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>소환 등급 +1 보장</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>보스 침공</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>👹</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>1.5시간</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>월드 보스 모든 성 공격</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>보물 사냥</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>🗺️</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>1시간</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>맵에 보물, 희귀 용병</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>용병 대전쟁</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>⚔️</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>2시간</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>서버 전체 용병 전쟁</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>드래곤 침공</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>🐲</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>3시간</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>드래곤 군단 협동 방어</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>암시장</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>🌑</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>1.5시간</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>희귀품 할인 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>경험치 폭풍</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>📈</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>1시간</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>용병 EXP 2배</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>혈맹 집결</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>🏴</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>4시간</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>혈맹 공성 보상 5배</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet133.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>전체 무역 루트 (10개)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>출발</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>도착</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>물품</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>매입</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>매도</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>위험</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>시간</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>이윤</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>바람개비</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>별빛 항구</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>곡물</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>30초</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>80%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>별빛 항구</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>달빛 오아시스</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>해산물</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>280</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>45초</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>87%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>달빛 오아시스</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>구름마루</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>향신료</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>60초</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>구름마루</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>신전 마을</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>광석</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>550</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>90초</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>신전 마을</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>사막 시장</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>마법 결정</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>120초</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>사막 시장</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>바람개비</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>보석</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>800</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>1500</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>150초</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>88%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>동쪽 항구</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>신전 마을</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>성수</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>750</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>35%</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>80초</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>88%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>구름마루</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>사막 시장</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>용린</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>70%</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>180초</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>120%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>바람개비</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>구름마루</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>목재</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>40초</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>별빛 항구</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>동쪽 항구</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>비단</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>480</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>60초</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>92%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet134.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13680,13 +14669,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet133.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet135.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -13701,7 +14690,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>전체 용병 목록 v3.0</t>
+          <t>전체 용병 목록 v3.0 (42종)</t>
         </is>
       </c>
     </row>
@@ -14664,6 +15653,598 @@
       <c r="G28" s="8" t="inlineStr">
         <is>
           <t>전체 8배+스턴</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>창병 🔱</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>전사</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>130</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>찌르기 1.8배</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>수도승 🙏</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>전사</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>연타 ×4</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>도둑 💰</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>암살</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>골드 50 훔침</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>고급</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>기마병 🐴</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>전사</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>돌격 2.5배</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>고급</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>석궁병 🏹</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>사수</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t>관통 3배</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>고급</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>주술사 🪬</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>마법</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>적 DEF-30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>고급</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>무희 💃</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>치유</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="G35" s="9" t="inlineStr">
+        <is>
+          <t>아군 SPD+20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>희귀</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>사무라이 ⚔️</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>전사</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>확정크리 4.5배</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>희귀</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>저격수 🎯</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>사수</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="G37" s="9" t="inlineStr">
+        <is>
+          <t>헤드샷 6배!</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>희귀</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>드루이드 🌿</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>치유</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>전체 50+재생</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>희귀</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>화염술사 🔥</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>마법</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>광역 3.5배+화상</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>영웅</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>마왕 👿</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>마법</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>280</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>광역 6배 암흑</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>영웅</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>수호천사 😇</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>치유</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+      <c r="G41" s="9" t="inlineStr">
+        <is>
+          <t>전체 80힐+보호막</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>영웅</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>검성 🗡️</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>전사</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>260</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>5연참 3배</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>전설</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>세계수 정령 🌳</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>치유</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>전체 150힐+부활</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>전설</t>
+        </is>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>공허의 왕 🌀</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>마법</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>전체 8배 공허</t>
         </is>
       </c>
     </row>

</xml_diff>